<commit_message>
Mise à jour DPS — 21/04/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1163">
   <si>
     <t>Début</t>
   </si>
@@ -3320,6 +3320,12 @@
   </si>
   <si>
     <t>Renfort DPS-Me - Concert Naza</t>
+  </si>
+  <si>
+    <t>21-04-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Concert Louis Tomlinson</t>
   </si>
   <si>
     <t>22-04-2026</t>
@@ -3856,7 +3862,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P632"/>
+  <dimension ref="A1:P633"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -26857,11 +26863,21 @@
       <c r="E596" t="s">
         <v>19</v>
       </c>
-      <c r="F596"/>
-      <c r="G596"/>
-      <c r="H596"/>
-      <c r="I596"/>
-      <c r="J596"/>
+      <c r="F596">
+        <v>0</v>
+      </c>
+      <c r="G596">
+        <v>0</v>
+      </c>
+      <c r="H596">
+        <v>0</v>
+      </c>
+      <c r="I596">
+        <v>0</v>
+      </c>
+      <c r="J596">
+        <v>0</v>
+      </c>
       <c r="K596" t="s">
         <v>20</v>
       </c>
@@ -27098,7 +27114,7 @@
       </c>
       <c r="C602"/>
       <c r="D602" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="E602" t="s">
         <v>19</v>
@@ -27112,16 +27128,16 @@
         <v>20</v>
       </c>
       <c r="L602" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M602">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N602">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O602">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="P602"/>
     </row>
@@ -27134,10 +27150,10 @@
       </c>
       <c r="C603"/>
       <c r="D603" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="E603" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F603"/>
       <c r="G603"/>
@@ -27151,13 +27167,13 @@
         <v>21</v>
       </c>
       <c r="M603">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="N603">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O603">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P603"/>
     </row>
@@ -27170,7 +27186,7 @@
       </c>
       <c r="C604"/>
       <c r="D604" t="s">
-        <v>539</v>
+        <v>34</v>
       </c>
       <c r="E604" t="s">
         <v>187</v>
@@ -27187,29 +27203,29 @@
         <v>21</v>
       </c>
       <c r="M604">
-        <v>10.5</v>
+        <v>6.5</v>
       </c>
       <c r="N604">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="O604">
-        <v>112</v>
+        <v>12</v>
       </c>
       <c r="P604"/>
     </row>
     <row r="605" spans="1:16">
       <c r="A605" t="s">
-        <v>1105</v>
+        <v>1107</v>
       </c>
       <c r="B605" t="s">
-        <v>827</v>
+        <v>1108</v>
       </c>
       <c r="C605"/>
       <c r="D605" t="s">
-        <v>55</v>
+        <v>539</v>
       </c>
       <c r="E605" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F605"/>
       <c r="G605"/>
@@ -27223,13 +27239,13 @@
         <v>21</v>
       </c>
       <c r="M605">
-        <v>5</v>
+        <v>10.5</v>
       </c>
       <c r="N605">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="O605">
-        <v>15</v>
+        <v>112</v>
       </c>
       <c r="P605"/>
     </row>
@@ -27238,11 +27254,11 @@
         <v>1107</v>
       </c>
       <c r="B606" t="s">
-        <v>1108</v>
+        <v>827</v>
       </c>
       <c r="C606"/>
       <c r="D606" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="E606" t="s">
         <v>19</v>
@@ -27256,16 +27272,16 @@
         <v>20</v>
       </c>
       <c r="L606" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M606">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="N606">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O606">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="P606"/>
     </row>
@@ -27292,16 +27308,16 @@
         <v>20</v>
       </c>
       <c r="L607" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M607">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="N607">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O607">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="P607"/>
     </row>
@@ -27314,10 +27330,10 @@
       </c>
       <c r="C608"/>
       <c r="D608" t="s">
-        <v>641</v>
+        <v>34</v>
       </c>
       <c r="E608" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F608"/>
       <c r="G608"/>
@@ -27331,13 +27347,13 @@
         <v>21</v>
       </c>
       <c r="M608">
-        <v>12.5</v>
+        <v>6</v>
       </c>
       <c r="N608">
         <v>4</v>
       </c>
       <c r="O608">
-        <v>42.5</v>
+        <v>24</v>
       </c>
       <c r="P608"/>
     </row>
@@ -27350,7 +27366,7 @@
       </c>
       <c r="C609"/>
       <c r="D609" t="s">
-        <v>686</v>
+        <v>641</v>
       </c>
       <c r="E609" t="s">
         <v>187</v>
@@ -27367,13 +27383,13 @@
         <v>21</v>
       </c>
       <c r="M609">
-        <v>6.5</v>
+        <v>12.5</v>
       </c>
       <c r="N609">
         <v>4</v>
       </c>
       <c r="O609">
-        <v>26</v>
+        <v>42.5</v>
       </c>
       <c r="P609"/>
     </row>
@@ -27386,7 +27402,7 @@
       </c>
       <c r="C610"/>
       <c r="D610" t="s">
-        <v>1117</v>
+        <v>686</v>
       </c>
       <c r="E610" t="s">
         <v>187</v>
@@ -27400,32 +27416,32 @@
         <v>20</v>
       </c>
       <c r="L610" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M610">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="N610">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O610">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="P610"/>
     </row>
     <row r="611" spans="1:16">
       <c r="A611" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B611" t="s">
         <v>1118</v>
-      </c>
-      <c r="B611" t="s">
-        <v>1119</v>
       </c>
       <c r="C611"/>
       <c r="D611" t="s">
-        <v>34</v>
+        <v>1119</v>
       </c>
       <c r="E611" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F611"/>
       <c r="G611"/>
@@ -27436,16 +27452,16 @@
         <v>20</v>
       </c>
       <c r="L611" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M611">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N611">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O611">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="P611"/>
     </row>
@@ -27461,7 +27477,7 @@
         <v>34</v>
       </c>
       <c r="E612" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F612"/>
       <c r="G612"/>
@@ -27472,16 +27488,16 @@
         <v>20</v>
       </c>
       <c r="L612" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M612">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N612">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O612">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="P612"/>
     </row>
@@ -27490,11 +27506,11 @@
         <v>1122</v>
       </c>
       <c r="B613" t="s">
-        <v>237</v>
+        <v>1123</v>
       </c>
       <c r="C613"/>
       <c r="D613" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E613" t="s">
         <v>187</v>
@@ -27508,29 +27524,29 @@
         <v>20</v>
       </c>
       <c r="L613" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M613">
-        <v>9.02</v>
+        <v>6</v>
       </c>
       <c r="N613">
         <v>3</v>
       </c>
       <c r="O613">
-        <v>27.060001373291</v>
+        <v>18</v>
       </c>
       <c r="P613"/>
     </row>
     <row r="614" spans="1:16">
       <c r="A614" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="B614" t="s">
-        <v>1124</v>
+        <v>237</v>
       </c>
       <c r="C614"/>
       <c r="D614" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="E614" t="s">
         <v>187</v>
@@ -27544,16 +27560,16 @@
         <v>20</v>
       </c>
       <c r="L614" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M614">
-        <v>6</v>
+        <v>9.02</v>
       </c>
       <c r="N614">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O614">
-        <v>12</v>
+        <v>27.060001373291</v>
       </c>
       <c r="P614"/>
     </row>
@@ -27586,9 +27602,11 @@
         <v>6</v>
       </c>
       <c r="N615">
-        <v>0</v>
-      </c>
-      <c r="O615"/>
+        <v>2</v>
+      </c>
+      <c r="O615">
+        <v>12</v>
+      </c>
       <c r="P615"/>
     </row>
     <row r="616" spans="1:16">
@@ -27596,7 +27614,7 @@
         <v>1127</v>
       </c>
       <c r="B616" t="s">
-        <v>192</v>
+        <v>1128</v>
       </c>
       <c r="C616"/>
       <c r="D616" t="s">
@@ -27614,29 +27632,27 @@
         <v>20</v>
       </c>
       <c r="L616" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M616">
         <v>6</v>
       </c>
       <c r="N616">
-        <v>2</v>
-      </c>
-      <c r="O616">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O616"/>
       <c r="P616"/>
     </row>
     <row r="617" spans="1:16">
       <c r="A617" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="B617" t="s">
-        <v>1129</v>
+        <v>192</v>
       </c>
       <c r="C617"/>
       <c r="D617" t="s">
-        <v>259</v>
+        <v>34</v>
       </c>
       <c r="E617" t="s">
         <v>187</v>
@@ -27653,13 +27669,13 @@
         <v>21</v>
       </c>
       <c r="M617">
-        <v>5.98</v>
+        <v>6</v>
       </c>
       <c r="N617">
         <v>2</v>
       </c>
       <c r="O617">
-        <v>11.960000038147</v>
+        <v>12</v>
       </c>
       <c r="P617"/>
     </row>
@@ -27689,13 +27705,13 @@
         <v>21</v>
       </c>
       <c r="M618">
-        <v>12</v>
+        <v>5.98</v>
       </c>
       <c r="N618">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O618">
-        <v>12</v>
+        <v>11.960000038147</v>
       </c>
       <c r="P618"/>
     </row>
@@ -27737,14 +27753,14 @@
     </row>
     <row r="620" spans="1:16">
       <c r="A620" t="s">
-        <v>1132</v>
+        <v>1134</v>
       </c>
       <c r="B620" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="C620"/>
       <c r="D620" t="s">
-        <v>476</v>
+        <v>259</v>
       </c>
       <c r="E620" t="s">
         <v>187</v>
@@ -27761,26 +27777,26 @@
         <v>21</v>
       </c>
       <c r="M620">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="N620">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O620">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="P620"/>
     </row>
     <row r="621" spans="1:16">
       <c r="A621" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="B621" t="s">
         <v>1136</v>
       </c>
       <c r="C621"/>
       <c r="D621" t="s">
-        <v>34</v>
+        <v>476</v>
       </c>
       <c r="E621" t="s">
         <v>187</v>
@@ -27797,13 +27813,13 @@
         <v>21</v>
       </c>
       <c r="M621">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N621">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O621">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P621"/>
     </row>
@@ -27816,7 +27832,7 @@
       </c>
       <c r="C622"/>
       <c r="D622" t="s">
-        <v>1139</v>
+        <v>34</v>
       </c>
       <c r="E622" t="s">
         <v>187</v>
@@ -27830,27 +27846,29 @@
         <v>20</v>
       </c>
       <c r="L622" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M622">
+        <v>6</v>
+      </c>
+      <c r="N622">
         <v>2</v>
       </c>
-      <c r="N622">
-        <v>0</v>
-      </c>
-      <c r="O622"/>
+      <c r="O622">
+        <v>12</v>
+      </c>
       <c r="P622"/>
     </row>
     <row r="623" spans="1:16">
       <c r="A623" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B623" t="s">
         <v>1140</v>
-      </c>
-      <c r="B623" t="s">
-        <v>1141</v>
       </c>
       <c r="C623"/>
       <c r="D623" t="s">
-        <v>123</v>
+        <v>1141</v>
       </c>
       <c r="E623" t="s">
         <v>187</v>
@@ -27864,10 +27882,10 @@
         <v>20</v>
       </c>
       <c r="L623" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M623">
-        <v>9.5</v>
+        <v>2</v>
       </c>
       <c r="N623">
         <v>0</v>
@@ -27880,11 +27898,11 @@
         <v>1142</v>
       </c>
       <c r="B624" t="s">
-        <v>778</v>
+        <v>1143</v>
       </c>
       <c r="C624"/>
       <c r="D624" t="s">
-        <v>1143</v>
+        <v>123</v>
       </c>
       <c r="E624" t="s">
         <v>187</v>
@@ -27898,17 +27916,15 @@
         <v>20</v>
       </c>
       <c r="L624" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M624">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="N624">
-        <v>9</v>
-      </c>
-      <c r="O624">
-        <v>90</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O624"/>
       <c r="P624"/>
     </row>
     <row r="625" spans="1:16">
@@ -27916,11 +27932,11 @@
         <v>1144</v>
       </c>
       <c r="B625" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="C625"/>
       <c r="D625" t="s">
-        <v>1143</v>
+        <v>1145</v>
       </c>
       <c r="E625" t="s">
         <v>187</v>
@@ -27937,26 +27953,26 @@
         <v>50</v>
       </c>
       <c r="M625">
+        <v>10</v>
+      </c>
+      <c r="N625">
         <v>9</v>
       </c>
-      <c r="N625">
-        <v>4</v>
-      </c>
       <c r="O625">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="P625"/>
     </row>
     <row r="626" spans="1:16">
       <c r="A626" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="B626" t="s">
-        <v>1146</v>
+        <v>780</v>
       </c>
       <c r="C626"/>
       <c r="D626" t="s">
-        <v>205</v>
+        <v>1145</v>
       </c>
       <c r="E626" t="s">
         <v>187</v>
@@ -27970,16 +27986,16 @@
         <v>20</v>
       </c>
       <c r="L626" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M626">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N626">
         <v>4</v>
       </c>
       <c r="O626">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="P626"/>
     </row>
@@ -27992,7 +28008,7 @@
       </c>
       <c r="C627"/>
       <c r="D627" t="s">
-        <v>1149</v>
+        <v>205</v>
       </c>
       <c r="E627" t="s">
         <v>187</v>
@@ -28006,29 +28022,29 @@
         <v>20</v>
       </c>
       <c r="L627" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M627">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N627">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O627">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="P627"/>
     </row>
     <row r="628" spans="1:16">
       <c r="A628" t="s">
-        <v>1147</v>
+        <v>1149</v>
       </c>
       <c r="B628" t="s">
         <v>1150</v>
       </c>
       <c r="C628"/>
       <c r="D628" t="s">
-        <v>1149</v>
+        <v>1151</v>
       </c>
       <c r="E628" t="s">
         <v>187</v>
@@ -28045,26 +28061,26 @@
         <v>50</v>
       </c>
       <c r="M628">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N628">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O628">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="P628"/>
     </row>
     <row r="629" spans="1:16">
       <c r="A629" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="B629" t="s">
         <v>1152</v>
       </c>
       <c r="C629"/>
       <c r="D629" t="s">
-        <v>1149</v>
+        <v>1151</v>
       </c>
       <c r="E629" t="s">
         <v>187</v>
@@ -28081,13 +28097,13 @@
         <v>50</v>
       </c>
       <c r="M629">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N629">
         <v>5</v>
       </c>
       <c r="O629">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="P629"/>
     </row>
@@ -28100,7 +28116,7 @@
       </c>
       <c r="C630"/>
       <c r="D630" t="s">
-        <v>1149</v>
+        <v>1151</v>
       </c>
       <c r="E630" t="s">
         <v>187</v>
@@ -28120,10 +28136,10 @@
         <v>11</v>
       </c>
       <c r="N630">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="O630">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="P630"/>
     </row>
@@ -28136,7 +28152,7 @@
       </c>
       <c r="C631"/>
       <c r="D631" t="s">
-        <v>1157</v>
+        <v>1151</v>
       </c>
       <c r="E631" t="s">
         <v>187</v>
@@ -28150,29 +28166,29 @@
         <v>20</v>
       </c>
       <c r="L631" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M631">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N631">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O631">
-        <v>63</v>
+        <v>121</v>
       </c>
       <c r="P631"/>
     </row>
     <row r="632" spans="1:16">
       <c r="A632" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B632" t="s">
         <v>1158</v>
-      </c>
-      <c r="B632" t="s">
-        <v>1159</v>
       </c>
       <c r="C632"/>
       <c r="D632" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="E632" t="s">
         <v>187</v>
@@ -28186,18 +28202,54 @@
         <v>20</v>
       </c>
       <c r="L632" t="s">
+        <v>21</v>
+      </c>
+      <c r="M632">
+        <v>9</v>
+      </c>
+      <c r="N632">
+        <v>7</v>
+      </c>
+      <c r="O632">
+        <v>63</v>
+      </c>
+      <c r="P632"/>
+    </row>
+    <row r="633" spans="1:16">
+      <c r="A633" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B633" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C633"/>
+      <c r="D633" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E633" t="s">
+        <v>187</v>
+      </c>
+      <c r="F633"/>
+      <c r="G633"/>
+      <c r="H633"/>
+      <c r="I633"/>
+      <c r="J633"/>
+      <c r="K633" t="s">
+        <v>20</v>
+      </c>
+      <c r="L633" t="s">
         <v>75</v>
       </c>
-      <c r="M632">
+      <c r="M633">
         <v>120</v>
       </c>
-      <c r="N632">
+      <c r="N633">
         <v>2</v>
       </c>
-      <c r="O632">
+      <c r="O633">
         <v>240</v>
       </c>
-      <c r="P632"/>
+      <c r="P633"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour DPS — 23/04/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1174">
   <si>
     <t>Début</t>
   </si>
@@ -3409,6 +3409,12 @@
     <t>20-05-2026</t>
   </si>
   <si>
+    <t>21-05-2026</t>
+  </si>
+  <si>
+    <t>[PROV] Fête de la musique</t>
+  </si>
+  <si>
     <t>22-05-2026</t>
   </si>
   <si>
@@ -3436,6 +3442,12 @@
     <t>Renfort DPS-ME - Concert Wizkid</t>
   </si>
   <si>
+    <t>30-05-2026</t>
+  </si>
+  <si>
+    <t>Course Amnestienne</t>
+  </si>
+  <si>
     <t>02-06-2026</t>
   </si>
   <si>
@@ -3451,6 +3463,15 @@
     <t>Forum des Transitions énergétiques et écologiques</t>
   </si>
   <si>
+    <t>07-06-2026</t>
+  </si>
+  <si>
+    <t>[Prov] La ruée des fadas</t>
+  </si>
+  <si>
+    <t>IdF</t>
+  </si>
+  <si>
     <t>13-06-2026</t>
   </si>
   <si>
@@ -3484,6 +3505,9 @@
     <t>[PROV] Solidays J2</t>
   </si>
   <si>
+    <t>[PROV] La marche des fiertés</t>
+  </si>
+  <si>
     <t>28-06-2026</t>
   </si>
   <si>
@@ -3497,6 +3521,15 @@
   </si>
   <si>
     <t>Annecy</t>
+  </si>
+  <si>
+    <t>13-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feu d'arifice </t>
+  </si>
+  <si>
+    <t>Choisy</t>
   </si>
   <si>
     <t>15-07-2026</t>
@@ -3862,7 +3895,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P633"/>
+  <dimension ref="A1:P638"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -27117,7 +27150,7 @@
         <v>34</v>
       </c>
       <c r="E602" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F602"/>
       <c r="G602"/>
@@ -27170,10 +27203,10 @@
         <v>5</v>
       </c>
       <c r="N603">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O603">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="P603"/>
     </row>
@@ -27189,7 +27222,7 @@
         <v>34</v>
       </c>
       <c r="E604" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F604"/>
       <c r="G604"/>
@@ -27206,10 +27239,10 @@
         <v>6.5</v>
       </c>
       <c r="N604">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O604">
-        <v>12</v>
+        <v>18.5</v>
       </c>
       <c r="P604"/>
     </row>
@@ -27566,10 +27599,10 @@
         <v>9.02</v>
       </c>
       <c r="N614">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O614">
-        <v>27.060001373291</v>
+        <v>36.080001831055</v>
       </c>
       <c r="P614"/>
     </row>
@@ -27655,7 +27688,7 @@
         <v>34</v>
       </c>
       <c r="E617" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F617"/>
       <c r="G617"/>
@@ -27672,10 +27705,10 @@
         <v>6</v>
       </c>
       <c r="N617">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O617">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="P617"/>
     </row>
@@ -27688,7 +27721,7 @@
       </c>
       <c r="C618"/>
       <c r="D618" t="s">
-        <v>259</v>
+        <v>18</v>
       </c>
       <c r="E618" t="s">
         <v>187</v>
@@ -27705,14 +27738,12 @@
         <v>21</v>
       </c>
       <c r="M618">
-        <v>5.98</v>
+        <v>8</v>
       </c>
       <c r="N618">
-        <v>2</v>
-      </c>
-      <c r="O618">
-        <v>11.960000038147</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O618"/>
       <c r="P618"/>
     </row>
     <row r="619" spans="1:16">
@@ -27741,13 +27772,13 @@
         <v>21</v>
       </c>
       <c r="M619">
-        <v>12</v>
+        <v>5.98</v>
       </c>
       <c r="N619">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O619">
-        <v>12</v>
+        <v>11.960000038147</v>
       </c>
       <c r="P619"/>
     </row>
@@ -27789,14 +27820,14 @@
     </row>
     <row r="621" spans="1:16">
       <c r="A621" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="B621" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="C621"/>
       <c r="D621" t="s">
-        <v>476</v>
+        <v>259</v>
       </c>
       <c r="E621" t="s">
         <v>187</v>
@@ -27813,26 +27844,26 @@
         <v>21</v>
       </c>
       <c r="M621">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="N621">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O621">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="P621"/>
     </row>
     <row r="622" spans="1:16">
       <c r="A622" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="B622" t="s">
         <v>1138</v>
       </c>
       <c r="C622"/>
       <c r="D622" t="s">
-        <v>34</v>
+        <v>476</v>
       </c>
       <c r="E622" t="s">
         <v>187</v>
@@ -27849,13 +27880,13 @@
         <v>21</v>
       </c>
       <c r="M622">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N622">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O622">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="P622"/>
     </row>
@@ -27868,7 +27899,7 @@
       </c>
       <c r="C623"/>
       <c r="D623" t="s">
-        <v>1141</v>
+        <v>34</v>
       </c>
       <c r="E623" t="s">
         <v>187</v>
@@ -27882,27 +27913,29 @@
         <v>20</v>
       </c>
       <c r="L623" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M623">
+        <v>6</v>
+      </c>
+      <c r="N623">
         <v>2</v>
       </c>
-      <c r="N623">
-        <v>0</v>
-      </c>
-      <c r="O623"/>
+      <c r="O623">
+        <v>12</v>
+      </c>
       <c r="P623"/>
     </row>
     <row r="624" spans="1:16">
       <c r="A624" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B624" t="s">
         <v>1142</v>
-      </c>
-      <c r="B624" t="s">
-        <v>1143</v>
       </c>
       <c r="C624"/>
       <c r="D624" t="s">
-        <v>123</v>
+        <v>589</v>
       </c>
       <c r="E624" t="s">
         <v>187</v>
@@ -27919,20 +27952,22 @@
         <v>21</v>
       </c>
       <c r="M624">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="N624">
-        <v>0</v>
-      </c>
-      <c r="O624"/>
+        <v>1</v>
+      </c>
+      <c r="O624">
+        <v>7</v>
+      </c>
       <c r="P624"/>
     </row>
     <row r="625" spans="1:16">
       <c r="A625" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B625" t="s">
         <v>1144</v>
-      </c>
-      <c r="B625" t="s">
-        <v>778</v>
       </c>
       <c r="C625"/>
       <c r="D625" t="s">
@@ -27950,17 +27985,15 @@
         <v>20</v>
       </c>
       <c r="L625" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="M625">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="N625">
-        <v>9</v>
-      </c>
-      <c r="O625">
-        <v>90</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O625"/>
       <c r="P625"/>
     </row>
     <row r="626" spans="1:16">
@@ -27968,11 +28001,11 @@
         <v>1146</v>
       </c>
       <c r="B626" t="s">
-        <v>780</v>
+        <v>1147</v>
       </c>
       <c r="C626"/>
       <c r="D626" t="s">
-        <v>1145</v>
+        <v>123</v>
       </c>
       <c r="E626" t="s">
         <v>187</v>
@@ -27986,29 +28019,29 @@
         <v>20</v>
       </c>
       <c r="L626" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M626">
-        <v>9</v>
+        <v>9.5</v>
       </c>
       <c r="N626">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O626">
-        <v>36</v>
+        <v>9.5</v>
       </c>
       <c r="P626"/>
     </row>
     <row r="627" spans="1:16">
       <c r="A627" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="B627" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="C627"/>
       <c r="D627" t="s">
-        <v>205</v>
+        <v>1150</v>
       </c>
       <c r="E627" t="s">
         <v>187</v>
@@ -28025,26 +28058,24 @@
         <v>21</v>
       </c>
       <c r="M627">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N627">
-        <v>4</v>
-      </c>
-      <c r="O627">
-        <v>28</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O627"/>
       <c r="P627"/>
     </row>
     <row r="628" spans="1:16">
       <c r="A628" t="s">
-        <v>1149</v>
+        <v>1151</v>
       </c>
       <c r="B628" t="s">
-        <v>1150</v>
+        <v>778</v>
       </c>
       <c r="C628"/>
       <c r="D628" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="E628" t="s">
         <v>187</v>
@@ -28061,26 +28092,26 @@
         <v>50</v>
       </c>
       <c r="M628">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N628">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O628">
-        <v>15</v>
+        <v>90</v>
       </c>
       <c r="P628"/>
     </row>
     <row r="629" spans="1:16">
       <c r="A629" t="s">
-        <v>1149</v>
+        <v>1153</v>
       </c>
       <c r="B629" t="s">
-        <v>1152</v>
+        <v>780</v>
       </c>
       <c r="C629"/>
       <c r="D629" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="E629" t="s">
         <v>187</v>
@@ -28097,26 +28128,26 @@
         <v>50</v>
       </c>
       <c r="M629">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N629">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O629">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P629"/>
     </row>
     <row r="630" spans="1:16">
       <c r="A630" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="B630" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="C630"/>
       <c r="D630" t="s">
-        <v>1151</v>
+        <v>205</v>
       </c>
       <c r="E630" t="s">
         <v>187</v>
@@ -28130,29 +28161,29 @@
         <v>20</v>
       </c>
       <c r="L630" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M630">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N630">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O630">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="P630"/>
     </row>
     <row r="631" spans="1:16">
       <c r="A631" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="B631" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="C631"/>
       <c r="D631" t="s">
-        <v>1151</v>
+        <v>1158</v>
       </c>
       <c r="E631" t="s">
         <v>187</v>
@@ -28169,26 +28200,26 @@
         <v>50</v>
       </c>
       <c r="M631">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N631">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="O631">
-        <v>121</v>
+        <v>15</v>
       </c>
       <c r="P631"/>
     </row>
     <row r="632" spans="1:16">
       <c r="A632" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="B632" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="C632"/>
       <c r="D632" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="E632" t="s">
         <v>187</v>
@@ -28202,16 +28233,16 @@
         <v>20</v>
       </c>
       <c r="L632" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M632">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N632">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O632">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="P632"/>
     </row>
@@ -28224,7 +28255,7 @@
       </c>
       <c r="C633"/>
       <c r="D633" t="s">
-        <v>1162</v>
+        <v>1158</v>
       </c>
       <c r="E633" t="s">
         <v>187</v>
@@ -28238,18 +28269,194 @@
         <v>20</v>
       </c>
       <c r="L633" t="s">
+        <v>50</v>
+      </c>
+      <c r="M633">
+        <v>11</v>
+      </c>
+      <c r="N633">
+        <v>5</v>
+      </c>
+      <c r="O633">
+        <v>55</v>
+      </c>
+      <c r="P633"/>
+    </row>
+    <row r="634" spans="1:16">
+      <c r="A634" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B634" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C634"/>
+      <c r="D634" t="s">
+        <v>18</v>
+      </c>
+      <c r="E634" t="s">
+        <v>187</v>
+      </c>
+      <c r="F634"/>
+      <c r="G634"/>
+      <c r="H634"/>
+      <c r="I634"/>
+      <c r="J634"/>
+      <c r="K634" t="s">
+        <v>20</v>
+      </c>
+      <c r="L634" t="s">
+        <v>21</v>
+      </c>
+      <c r="M634">
+        <v>8</v>
+      </c>
+      <c r="N634">
+        <v>0</v>
+      </c>
+      <c r="O634"/>
+      <c r="P634"/>
+    </row>
+    <row r="635" spans="1:16">
+      <c r="A635" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B635" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C635"/>
+      <c r="D635" t="s">
+        <v>1158</v>
+      </c>
+      <c r="E635" t="s">
+        <v>187</v>
+      </c>
+      <c r="F635"/>
+      <c r="G635"/>
+      <c r="H635"/>
+      <c r="I635"/>
+      <c r="J635"/>
+      <c r="K635" t="s">
+        <v>20</v>
+      </c>
+      <c r="L635" t="s">
+        <v>50</v>
+      </c>
+      <c r="M635">
+        <v>11</v>
+      </c>
+      <c r="N635">
+        <v>11</v>
+      </c>
+      <c r="O635">
+        <v>121</v>
+      </c>
+      <c r="P635"/>
+    </row>
+    <row r="636" spans="1:16">
+      <c r="A636" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B636" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C636"/>
+      <c r="D636" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E636" t="s">
+        <v>187</v>
+      </c>
+      <c r="F636"/>
+      <c r="G636"/>
+      <c r="H636"/>
+      <c r="I636"/>
+      <c r="J636"/>
+      <c r="K636" t="s">
+        <v>20</v>
+      </c>
+      <c r="L636" t="s">
+        <v>21</v>
+      </c>
+      <c r="M636">
+        <v>9</v>
+      </c>
+      <c r="N636">
+        <v>7</v>
+      </c>
+      <c r="O636">
+        <v>63</v>
+      </c>
+      <c r="P636"/>
+    </row>
+    <row r="637" spans="1:16">
+      <c r="A637" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B637" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C637"/>
+      <c r="D637" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E637" t="s">
+        <v>19</v>
+      </c>
+      <c r="F637"/>
+      <c r="G637"/>
+      <c r="H637"/>
+      <c r="I637"/>
+      <c r="J637"/>
+      <c r="K637" t="s">
+        <v>20</v>
+      </c>
+      <c r="L637" t="s">
+        <v>21</v>
+      </c>
+      <c r="M637">
+        <v>3</v>
+      </c>
+      <c r="N637">
+        <v>0</v>
+      </c>
+      <c r="O637"/>
+      <c r="P637"/>
+    </row>
+    <row r="638" spans="1:16">
+      <c r="A638" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B638" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C638"/>
+      <c r="D638" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E638" t="s">
+        <v>187</v>
+      </c>
+      <c r="F638"/>
+      <c r="G638"/>
+      <c r="H638"/>
+      <c r="I638"/>
+      <c r="J638"/>
+      <c r="K638" t="s">
+        <v>20</v>
+      </c>
+      <c r="L638" t="s">
         <v>75</v>
       </c>
-      <c r="M633">
+      <c r="M638">
         <v>120</v>
       </c>
-      <c r="N633">
+      <c r="N638">
         <v>2</v>
       </c>
-      <c r="O633">
+      <c r="O638">
         <v>240</v>
       </c>
-      <c r="P633"/>
+      <c r="P638"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour DPS — 04/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1207">
   <si>
     <t>Début</t>
   </si>
@@ -3340,24 +3340,48 @@
     <t>Renfort DPS-ME - Finales CDF de Basket</t>
   </si>
   <si>
+    <t>25-04-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Finale CDF Basket</t>
+  </si>
+  <si>
     <t>28-04-2026</t>
   </si>
   <si>
     <t>Foire du Trone 2026</t>
   </si>
   <si>
+    <t>Course d'entreprise</t>
+  </si>
+  <si>
+    <t>Villeneuve-la-Garenne</t>
+  </si>
+  <si>
     <t>29-04-2026</t>
   </si>
   <si>
     <t>Renfort DPS-ME - Concert Amel Bent</t>
   </si>
   <si>
+    <t>02-05-2026</t>
+  </si>
+  <si>
+    <t>Renfort PSG  Lorient Ligue 1</t>
+  </si>
+  <si>
     <t>03-05-2026</t>
   </si>
   <si>
     <t>Renfort DPS-ME - Concert Tame Impala</t>
   </si>
   <si>
+    <t>Interclub Athlétisme</t>
+  </si>
+  <si>
+    <t>Noisy-le-Grand</t>
+  </si>
+  <si>
     <t>04-05-2026</t>
   </si>
   <si>
@@ -3370,6 +3394,24 @@
     <t>Printemps des Associations</t>
   </si>
   <si>
+    <t>07-05-2026</t>
+  </si>
+  <si>
+    <t>Soirée Électronique - Boiler Room J1</t>
+  </si>
+  <si>
+    <t>Parc floral, Hall de la p</t>
+  </si>
+  <si>
+    <t>08-05-2026</t>
+  </si>
+  <si>
+    <t>Soirée électronique - Boiler Room Paris J2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paris 12 </t>
+  </si>
+  <si>
     <t>09-05-2026</t>
   </si>
   <si>
@@ -3412,81 +3454,99 @@
     <t>21-05-2026</t>
   </si>
   <si>
+    <t>Exercice SOGEPP TRAPIL/TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gennevilliers </t>
+  </si>
+  <si>
+    <t>Festival Educ'Sport</t>
+  </si>
+  <si>
+    <t>Paris - UFR Cité Paris</t>
+  </si>
+  <si>
+    <t>22-05-2026</t>
+  </si>
+  <si>
+    <t>[Prov] Le Cercle Festival J1</t>
+  </si>
+  <si>
+    <t>23-05-2026</t>
+  </si>
+  <si>
+    <t>[Prov] Le Cercle Festival J2</t>
+  </si>
+  <si>
+    <t>24-05-2026</t>
+  </si>
+  <si>
+    <t>[Prov] Le Cercle Festival J3</t>
+  </si>
+  <si>
+    <t>[Prov]course du Château de Vincennes</t>
+  </si>
+  <si>
+    <t>27-05-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Handball PSG vs Nantes</t>
+  </si>
+  <si>
+    <t>30-05-2026</t>
+  </si>
+  <si>
+    <t>Course Amnestienne</t>
+  </si>
+  <si>
+    <t>02-06-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rugby à 5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stade Charlety </t>
+  </si>
+  <si>
+    <t>04-06-2026</t>
+  </si>
+  <si>
+    <t>Forum des Transitions énergétiques et écologiques</t>
+  </si>
+  <si>
+    <t>07-06-2026</t>
+  </si>
+  <si>
+    <t>[Prov] La ruée des fadas</t>
+  </si>
+  <si>
+    <t>IdF</t>
+  </si>
+  <si>
+    <t>13-06-2026</t>
+  </si>
+  <si>
+    <t>Hippodrome Paris-Vincenne</t>
+  </si>
+  <si>
+    <t>14-06-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maison des arts Martiaux </t>
+  </si>
+  <si>
+    <t>17-06-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeux des collèges </t>
+  </si>
+  <si>
+    <t>21-06-2026</t>
+  </si>
+  <si>
     <t>[PROV] Fête de la musique</t>
   </si>
   <si>
-    <t>22-05-2026</t>
-  </si>
-  <si>
-    <t>[Prov] Le Cercle Festival J1</t>
-  </si>
-  <si>
-    <t>23-05-2026</t>
-  </si>
-  <si>
-    <t>[Prov] Le Cercle Festival J2</t>
-  </si>
-  <si>
-    <t>24-05-2026</t>
-  </si>
-  <si>
-    <t>[Prov] Le Cercle Festival J3</t>
-  </si>
-  <si>
-    <t>[Prov]course du Château de Vincennes</t>
-  </si>
-  <si>
-    <t>25-05-2026</t>
-  </si>
-  <si>
-    <t>Renfort DPS-ME - Concert Wizkid</t>
-  </si>
-  <si>
-    <t>30-05-2026</t>
-  </si>
-  <si>
-    <t>Course Amnestienne</t>
-  </si>
-  <si>
-    <t>02-06-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rugby à 5 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stade Charlety </t>
-  </si>
-  <si>
-    <t>04-06-2026</t>
-  </si>
-  <si>
-    <t>Forum des Transitions énergétiques et écologiques</t>
-  </si>
-  <si>
-    <t>07-06-2026</t>
-  </si>
-  <si>
-    <t>[Prov] La ruée des fadas</t>
-  </si>
-  <si>
-    <t>IdF</t>
-  </si>
-  <si>
-    <t>13-06-2026</t>
-  </si>
-  <si>
-    <t>Hippodrome Paris-Vincenne</t>
-  </si>
-  <si>
-    <t>14-06-2026</t>
-  </si>
-  <si>
-    <t>17-06-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jeux des collèges </t>
-  </si>
-  <si>
     <t>26-06-2026</t>
   </si>
   <si>
@@ -3508,12 +3568,39 @@
     <t>[PROV] La marche des fiertés</t>
   </si>
   <si>
+    <t>FestiMarne 2026 - J1</t>
+  </si>
+  <si>
+    <t>Marne</t>
+  </si>
+  <si>
     <t>28-06-2026</t>
   </si>
   <si>
     <t>[PROV] Solidays J3</t>
   </si>
   <si>
+    <t>FestiMarne 2026 - J2</t>
+  </si>
+  <si>
+    <t>29-06-2026</t>
+  </si>
+  <si>
+    <t>Tournage Le réseau Corneille</t>
+  </si>
+  <si>
+    <t>Tunnel Canal Saint martin</t>
+  </si>
+  <si>
+    <t>01-07-2026</t>
+  </si>
+  <si>
+    <t>Spectacle sur l'eau</t>
+  </si>
+  <si>
+    <t>Canal de l'ourcq</t>
+  </si>
+  <si>
     <t>04-07-2026</t>
   </si>
   <si>
@@ -3523,6 +3610,9 @@
     <t>Annecy</t>
   </si>
   <si>
+    <t xml:space="preserve">Renfort Compagny Cup </t>
+  </si>
+  <si>
     <t>13-07-2026</t>
   </si>
   <si>
@@ -3530,6 +3620,15 @@
   </si>
   <si>
     <t>Choisy</t>
+  </si>
+  <si>
+    <t>Poissy</t>
+  </si>
+  <si>
+    <t>Triel Sur Seine</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Bonneuil-sur-Marne</t>
   </si>
   <si>
     <t>15-07-2026</t>
@@ -3895,7 +3994,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P638"/>
+  <dimension ref="A1:P657"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -27255,10 +27354,10 @@
       </c>
       <c r="C605"/>
       <c r="D605" t="s">
-        <v>539</v>
+        <v>34</v>
       </c>
       <c r="E605" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F605"/>
       <c r="G605"/>
@@ -27269,38 +27368,48 @@
         <v>20</v>
       </c>
       <c r="L605" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M605">
-        <v>10.5</v>
+        <v>13</v>
       </c>
       <c r="N605">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="O605">
-        <v>112</v>
+        <v>13</v>
       </c>
       <c r="P605"/>
     </row>
     <row r="606" spans="1:16">
       <c r="A606" t="s">
-        <v>1107</v>
+        <v>1109</v>
       </c>
       <c r="B606" t="s">
-        <v>827</v>
+        <v>1110</v>
       </c>
       <c r="C606"/>
       <c r="D606" t="s">
-        <v>55</v>
+        <v>539</v>
       </c>
       <c r="E606" t="s">
         <v>19</v>
       </c>
-      <c r="F606"/>
-      <c r="G606"/>
-      <c r="H606"/>
-      <c r="I606"/>
-      <c r="J606"/>
+      <c r="F606">
+        <v>5</v>
+      </c>
+      <c r="G606">
+        <v>0</v>
+      </c>
+      <c r="H606">
+        <v>0</v>
+      </c>
+      <c r="I606">
+        <v>0</v>
+      </c>
+      <c r="J606">
+        <v>3</v>
+      </c>
       <c r="K606" t="s">
         <v>20</v>
       </c>
@@ -27308,13 +27417,13 @@
         <v>21</v>
       </c>
       <c r="M606">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N606">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="O606">
-        <v>15</v>
+        <v>112.5</v>
       </c>
       <c r="P606"/>
     </row>
@@ -27323,11 +27432,11 @@
         <v>1109</v>
       </c>
       <c r="B607" t="s">
-        <v>1110</v>
+        <v>827</v>
       </c>
       <c r="C607"/>
       <c r="D607" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="E607" t="s">
         <v>19</v>
@@ -27341,38 +27450,48 @@
         <v>20</v>
       </c>
       <c r="L607" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M607">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="N607">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O607">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="P607"/>
     </row>
     <row r="608" spans="1:16">
       <c r="A608" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B608" t="s">
         <v>1111</v>
-      </c>
-      <c r="B608" t="s">
-        <v>1112</v>
       </c>
       <c r="C608"/>
       <c r="D608" t="s">
-        <v>34</v>
+        <v>1112</v>
       </c>
       <c r="E608" t="s">
         <v>19</v>
       </c>
-      <c r="F608"/>
-      <c r="G608"/>
-      <c r="H608"/>
-      <c r="I608"/>
-      <c r="J608"/>
+      <c r="F608">
+        <v>0</v>
+      </c>
+      <c r="G608">
+        <v>0</v>
+      </c>
+      <c r="H608">
+        <v>0</v>
+      </c>
+      <c r="I608">
+        <v>0</v>
+      </c>
+      <c r="J608">
+        <v>0</v>
+      </c>
       <c r="K608" t="s">
         <v>20</v>
       </c>
@@ -27380,13 +27499,13 @@
         <v>21</v>
       </c>
       <c r="M608">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N608">
         <v>4</v>
       </c>
       <c r="O608">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="P608"/>
     </row>
@@ -27399,10 +27518,10 @@
       </c>
       <c r="C609"/>
       <c r="D609" t="s">
-        <v>641</v>
+        <v>34</v>
       </c>
       <c r="E609" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F609"/>
       <c r="G609"/>
@@ -27413,16 +27532,16 @@
         <v>20</v>
       </c>
       <c r="L609" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M609">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="N609">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O609">
-        <v>42.5</v>
+        <v>10</v>
       </c>
       <c r="P609"/>
     </row>
@@ -27435,10 +27554,10 @@
       </c>
       <c r="C610"/>
       <c r="D610" t="s">
-        <v>686</v>
+        <v>55</v>
       </c>
       <c r="E610" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F610"/>
       <c r="G610"/>
@@ -27449,16 +27568,16 @@
         <v>20</v>
       </c>
       <c r="L610" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M610">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="N610">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O610">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="P610"/>
     </row>
@@ -27471,10 +27590,10 @@
       </c>
       <c r="C611"/>
       <c r="D611" t="s">
-        <v>1119</v>
+        <v>34</v>
       </c>
       <c r="E611" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F611"/>
       <c r="G611"/>
@@ -27485,68 +27604,78 @@
         <v>20</v>
       </c>
       <c r="L611" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M611">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N611">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O611">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="P611"/>
     </row>
     <row r="612" spans="1:16">
       <c r="A612" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
       <c r="B612" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="C612"/>
       <c r="D612" t="s">
-        <v>34</v>
+        <v>1120</v>
       </c>
       <c r="E612" t="s">
         <v>19</v>
       </c>
-      <c r="F612"/>
-      <c r="G612"/>
-      <c r="H612"/>
-      <c r="I612"/>
-      <c r="J612"/>
+      <c r="F612">
+        <v>4</v>
+      </c>
+      <c r="G612">
+        <v>0</v>
+      </c>
+      <c r="H612">
+        <v>0</v>
+      </c>
+      <c r="I612">
+        <v>0</v>
+      </c>
+      <c r="J612">
+        <v>0</v>
+      </c>
       <c r="K612" t="s">
         <v>20</v>
       </c>
       <c r="L612" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M612">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="N612">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O612">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="P612"/>
     </row>
     <row r="613" spans="1:16">
       <c r="A613" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B613" t="s">
         <v>1122</v>
-      </c>
-      <c r="B613" t="s">
-        <v>1123</v>
       </c>
       <c r="C613"/>
       <c r="D613" t="s">
-        <v>34</v>
+        <v>641</v>
       </c>
       <c r="E613" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F613"/>
       <c r="G613"/>
@@ -27557,32 +27686,32 @@
         <v>20</v>
       </c>
       <c r="L613" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M613">
+        <v>12.5</v>
+      </c>
+      <c r="N613">
         <v>6</v>
       </c>
-      <c r="N613">
-        <v>3</v>
-      </c>
       <c r="O613">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="P613"/>
     </row>
     <row r="614" spans="1:16">
       <c r="A614" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B614" t="s">
         <v>1124</v>
-      </c>
-      <c r="B614" t="s">
-        <v>237</v>
       </c>
       <c r="C614"/>
       <c r="D614" t="s">
-        <v>18</v>
+        <v>686</v>
       </c>
       <c r="E614" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F614"/>
       <c r="G614"/>
@@ -27596,13 +27725,13 @@
         <v>21</v>
       </c>
       <c r="M614">
-        <v>9.02</v>
+        <v>6.5</v>
       </c>
       <c r="N614">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O614">
-        <v>36.080001831055</v>
+        <v>32.5</v>
       </c>
       <c r="P614"/>
     </row>
@@ -27615,10 +27744,10 @@
       </c>
       <c r="C615"/>
       <c r="D615" t="s">
-        <v>34</v>
+        <v>1127</v>
       </c>
       <c r="E615" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F615"/>
       <c r="G615"/>
@@ -27629,29 +27758,29 @@
         <v>20</v>
       </c>
       <c r="L615" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M615">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="N615">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="O615">
-        <v>12</v>
+        <v>144</v>
       </c>
       <c r="P615"/>
     </row>
     <row r="616" spans="1:16">
       <c r="A616" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B616" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="C616"/>
       <c r="D616" t="s">
-        <v>34</v>
+        <v>1130</v>
       </c>
       <c r="E616" t="s">
         <v>187</v>
@@ -27665,30 +27794,32 @@
         <v>20</v>
       </c>
       <c r="L616" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M616">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="N616">
-        <v>0</v>
-      </c>
-      <c r="O616"/>
+        <v>10</v>
+      </c>
+      <c r="O616">
+        <v>120</v>
+      </c>
       <c r="P616"/>
     </row>
     <row r="617" spans="1:16">
       <c r="A617" t="s">
-        <v>1129</v>
+        <v>1131</v>
       </c>
       <c r="B617" t="s">
-        <v>192</v>
+        <v>1132</v>
       </c>
       <c r="C617"/>
       <c r="D617" t="s">
-        <v>34</v>
+        <v>1133</v>
       </c>
       <c r="E617" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F617"/>
       <c r="G617"/>
@@ -27699,32 +27830,32 @@
         <v>20</v>
       </c>
       <c r="L617" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M617">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N617">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O617">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="P617"/>
     </row>
     <row r="618" spans="1:16">
       <c r="A618" t="s">
-        <v>1130</v>
+        <v>1134</v>
       </c>
       <c r="B618" t="s">
-        <v>1131</v>
+        <v>1135</v>
       </c>
       <c r="C618"/>
       <c r="D618" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E618" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F618"/>
       <c r="G618"/>
@@ -27741,24 +27872,26 @@
         <v>8</v>
       </c>
       <c r="N618">
-        <v>0</v>
-      </c>
-      <c r="O618"/>
+        <v>5</v>
+      </c>
+      <c r="O618">
+        <v>40</v>
+      </c>
       <c r="P618"/>
     </row>
     <row r="619" spans="1:16">
       <c r="A619" t="s">
-        <v>1132</v>
+        <v>1136</v>
       </c>
       <c r="B619" t="s">
-        <v>1133</v>
+        <v>1137</v>
       </c>
       <c r="C619"/>
       <c r="D619" t="s">
-        <v>259</v>
+        <v>34</v>
       </c>
       <c r="E619" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F619"/>
       <c r="G619"/>
@@ -27772,26 +27905,26 @@
         <v>21</v>
       </c>
       <c r="M619">
-        <v>5.98</v>
+        <v>6</v>
       </c>
       <c r="N619">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O619">
-        <v>11.960000038147</v>
+        <v>30</v>
       </c>
       <c r="P619"/>
     </row>
     <row r="620" spans="1:16">
       <c r="A620" t="s">
-        <v>1134</v>
+        <v>1138</v>
       </c>
       <c r="B620" t="s">
-        <v>1135</v>
+        <v>237</v>
       </c>
       <c r="C620"/>
       <c r="D620" t="s">
-        <v>259</v>
+        <v>18</v>
       </c>
       <c r="E620" t="s">
         <v>187</v>
@@ -27808,26 +27941,26 @@
         <v>21</v>
       </c>
       <c r="M620">
-        <v>12</v>
+        <v>9.02</v>
       </c>
       <c r="N620">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O620">
-        <v>12</v>
+        <v>63.140003204346</v>
       </c>
       <c r="P620"/>
     </row>
     <row r="621" spans="1:16">
       <c r="A621" t="s">
-        <v>1136</v>
+        <v>1139</v>
       </c>
       <c r="B621" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="C621"/>
       <c r="D621" t="s">
-        <v>259</v>
+        <v>34</v>
       </c>
       <c r="E621" t="s">
         <v>187</v>
@@ -27841,29 +27974,29 @@
         <v>20</v>
       </c>
       <c r="L621" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M621">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="N621">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O621">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="P621"/>
     </row>
     <row r="622" spans="1:16">
       <c r="A622" t="s">
-        <v>1136</v>
+        <v>1141</v>
       </c>
       <c r="B622" t="s">
-        <v>1138</v>
+        <v>1142</v>
       </c>
       <c r="C622"/>
       <c r="D622" t="s">
-        <v>476</v>
+        <v>34</v>
       </c>
       <c r="E622" t="s">
         <v>187</v>
@@ -27880,29 +28013,29 @@
         <v>21</v>
       </c>
       <c r="M622">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N622">
         <v>3</v>
       </c>
       <c r="O622">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P622"/>
     </row>
     <row r="623" spans="1:16">
       <c r="A623" t="s">
-        <v>1139</v>
+        <v>1143</v>
       </c>
       <c r="B623" t="s">
-        <v>1140</v>
+        <v>192</v>
       </c>
       <c r="C623"/>
       <c r="D623" t="s">
         <v>34</v>
       </c>
       <c r="E623" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F623"/>
       <c r="G623"/>
@@ -27919,23 +28052,23 @@
         <v>6</v>
       </c>
       <c r="N623">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O623">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="P623"/>
     </row>
     <row r="624" spans="1:16">
       <c r="A624" t="s">
-        <v>1141</v>
+        <v>1143</v>
       </c>
       <c r="B624" t="s">
-        <v>1142</v>
+        <v>1110</v>
       </c>
       <c r="C624"/>
       <c r="D624" t="s">
-        <v>589</v>
+        <v>539</v>
       </c>
       <c r="E624" t="s">
         <v>187</v>
@@ -27952,29 +28085,29 @@
         <v>21</v>
       </c>
       <c r="M624">
-        <v>7</v>
+        <v>9.5</v>
       </c>
       <c r="N624">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O624">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="P624"/>
     </row>
     <row r="625" spans="1:16">
       <c r="A625" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="B625" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="C625"/>
       <c r="D625" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="E625" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F625"/>
       <c r="G625"/>
@@ -27985,10 +28118,10 @@
         <v>20</v>
       </c>
       <c r="L625" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M625">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="N625">
         <v>0</v>
@@ -27998,14 +28131,14 @@
     </row>
     <row r="626" spans="1:16">
       <c r="A626" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="B626" t="s">
         <v>1147</v>
       </c>
       <c r="C626"/>
       <c r="D626" t="s">
-        <v>123</v>
+        <v>1148</v>
       </c>
       <c r="E626" t="s">
         <v>187</v>
@@ -28022,26 +28155,26 @@
         <v>21</v>
       </c>
       <c r="M626">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="N626">
         <v>1</v>
       </c>
       <c r="O626">
-        <v>9.5</v>
+        <v>3</v>
       </c>
       <c r="P626"/>
     </row>
     <row r="627" spans="1:16">
       <c r="A627" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="B627" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="C627"/>
       <c r="D627" t="s">
-        <v>1150</v>
+        <v>259</v>
       </c>
       <c r="E627" t="s">
         <v>187</v>
@@ -28058,12 +28191,14 @@
         <v>21</v>
       </c>
       <c r="M627">
-        <v>6</v>
+        <v>5.98</v>
       </c>
       <c r="N627">
-        <v>0</v>
-      </c>
-      <c r="O627"/>
+        <v>2</v>
+      </c>
+      <c r="O627">
+        <v>11.960000038147</v>
+      </c>
       <c r="P627"/>
     </row>
     <row r="628" spans="1:16">
@@ -28071,11 +28206,11 @@
         <v>1151</v>
       </c>
       <c r="B628" t="s">
-        <v>778</v>
+        <v>1152</v>
       </c>
       <c r="C628"/>
       <c r="D628" t="s">
-        <v>1152</v>
+        <v>259</v>
       </c>
       <c r="E628" t="s">
         <v>187</v>
@@ -28089,16 +28224,16 @@
         <v>20</v>
       </c>
       <c r="L628" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M628">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N628">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="O628">
-        <v>90</v>
+        <v>24</v>
       </c>
       <c r="P628"/>
     </row>
@@ -28107,11 +28242,11 @@
         <v>1153</v>
       </c>
       <c r="B629" t="s">
-        <v>780</v>
+        <v>1154</v>
       </c>
       <c r="C629"/>
       <c r="D629" t="s">
-        <v>1152</v>
+        <v>259</v>
       </c>
       <c r="E629" t="s">
         <v>187</v>
@@ -28125,29 +28260,29 @@
         <v>20</v>
       </c>
       <c r="L629" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M629">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N629">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O629">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="P629"/>
     </row>
     <row r="630" spans="1:16">
       <c r="A630" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B630" t="s">
         <v>1155</v>
       </c>
       <c r="C630"/>
       <c r="D630" t="s">
-        <v>205</v>
+        <v>476</v>
       </c>
       <c r="E630" t="s">
         <v>187</v>
@@ -28164,26 +28299,26 @@
         <v>21</v>
       </c>
       <c r="M630">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N630">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O630">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="P630"/>
     </row>
     <row r="631" spans="1:16">
       <c r="A631" t="s">
-        <v>1156</v>
+        <v>1153</v>
       </c>
       <c r="B631" t="s">
-        <v>1157</v>
+        <v>1110</v>
       </c>
       <c r="C631"/>
       <c r="D631" t="s">
-        <v>1158</v>
+        <v>539</v>
       </c>
       <c r="E631" t="s">
         <v>187</v>
@@ -28197,16 +28332,16 @@
         <v>20</v>
       </c>
       <c r="L631" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M631">
-        <v>5</v>
+        <v>11.5</v>
       </c>
       <c r="N631">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O631">
-        <v>15</v>
+        <v>11.5</v>
       </c>
       <c r="P631"/>
     </row>
@@ -28215,11 +28350,11 @@
         <v>1156</v>
       </c>
       <c r="B632" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="C632"/>
       <c r="D632" t="s">
-        <v>1158</v>
+        <v>34</v>
       </c>
       <c r="E632" t="s">
         <v>187</v>
@@ -28233,29 +28368,29 @@
         <v>20</v>
       </c>
       <c r="L632" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M632">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N632">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O632">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="P632"/>
     </row>
     <row r="633" spans="1:16">
       <c r="A633" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="B633" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="C633"/>
       <c r="D633" t="s">
-        <v>1158</v>
+        <v>589</v>
       </c>
       <c r="E633" t="s">
         <v>187</v>
@@ -28269,16 +28404,16 @@
         <v>20</v>
       </c>
       <c r="L633" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M633">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N633">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O633">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="P633"/>
     </row>
@@ -28287,11 +28422,11 @@
         <v>1160</v>
       </c>
       <c r="B634" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="C634"/>
       <c r="D634" t="s">
-        <v>18</v>
+        <v>1162</v>
       </c>
       <c r="E634" t="s">
         <v>187</v>
@@ -28305,10 +28440,10 @@
         <v>20</v>
       </c>
       <c r="L634" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M634">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="N634">
         <v>0</v>
@@ -28325,7 +28460,7 @@
       </c>
       <c r="C635"/>
       <c r="D635" t="s">
-        <v>1158</v>
+        <v>123</v>
       </c>
       <c r="E635" t="s">
         <v>187</v>
@@ -28339,16 +28474,16 @@
         <v>20</v>
       </c>
       <c r="L635" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M635">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="N635">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="O635">
-        <v>121</v>
+        <v>9.5</v>
       </c>
       <c r="P635"/>
     </row>
@@ -28378,14 +28513,12 @@
         <v>21</v>
       </c>
       <c r="M636">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N636">
-        <v>7</v>
-      </c>
-      <c r="O636">
-        <v>63</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O636"/>
       <c r="P636"/>
     </row>
     <row r="637" spans="1:16">
@@ -28393,14 +28526,14 @@
         <v>1168</v>
       </c>
       <c r="B637" t="s">
-        <v>1169</v>
+        <v>778</v>
       </c>
       <c r="C637"/>
       <c r="D637" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="E637" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F637"/>
       <c r="G637"/>
@@ -28411,27 +28544,29 @@
         <v>20</v>
       </c>
       <c r="L637" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M637">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="N637">
-        <v>0</v>
-      </c>
-      <c r="O637"/>
+        <v>8</v>
+      </c>
+      <c r="O637">
+        <v>80</v>
+      </c>
       <c r="P637"/>
     </row>
     <row r="638" spans="1:16">
       <c r="A638" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="B638" t="s">
-        <v>1172</v>
+        <v>780</v>
       </c>
       <c r="C638"/>
       <c r="D638" t="s">
-        <v>1173</v>
+        <v>1169</v>
       </c>
       <c r="E638" t="s">
         <v>187</v>
@@ -28445,18 +28580,678 @@
         <v>20</v>
       </c>
       <c r="L638" t="s">
+        <v>50</v>
+      </c>
+      <c r="M638">
+        <v>9</v>
+      </c>
+      <c r="N638">
+        <v>3</v>
+      </c>
+      <c r="O638">
+        <v>27</v>
+      </c>
+      <c r="P638"/>
+    </row>
+    <row r="639" spans="1:16">
+      <c r="A639" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B639" t="s">
+        <v>643</v>
+      </c>
+      <c r="C639"/>
+      <c r="D639" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E639" t="s">
+        <v>187</v>
+      </c>
+      <c r="F639"/>
+      <c r="G639"/>
+      <c r="H639"/>
+      <c r="I639"/>
+      <c r="J639"/>
+      <c r="K639" t="s">
+        <v>20</v>
+      </c>
+      <c r="L639" t="s">
+        <v>25</v>
+      </c>
+      <c r="M639">
+        <v>8.25</v>
+      </c>
+      <c r="N639">
+        <v>0</v>
+      </c>
+      <c r="O639"/>
+      <c r="P639"/>
+    </row>
+    <row r="640" spans="1:16">
+      <c r="A640" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B640" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C640"/>
+      <c r="D640" t="s">
+        <v>205</v>
+      </c>
+      <c r="E640" t="s">
+        <v>187</v>
+      </c>
+      <c r="F640"/>
+      <c r="G640"/>
+      <c r="H640"/>
+      <c r="I640"/>
+      <c r="J640"/>
+      <c r="K640" t="s">
+        <v>20</v>
+      </c>
+      <c r="L640" t="s">
+        <v>21</v>
+      </c>
+      <c r="M640">
+        <v>7</v>
+      </c>
+      <c r="N640">
+        <v>4</v>
+      </c>
+      <c r="O640">
+        <v>28</v>
+      </c>
+      <c r="P640"/>
+    </row>
+    <row r="641" spans="1:16">
+      <c r="A641" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B641" t="s">
+        <v>1175</v>
+      </c>
+      <c r="C641"/>
+      <c r="D641" t="s">
+        <v>18</v>
+      </c>
+      <c r="E641" t="s">
+        <v>187</v>
+      </c>
+      <c r="F641"/>
+      <c r="G641"/>
+      <c r="H641"/>
+      <c r="I641"/>
+      <c r="J641"/>
+      <c r="K641" t="s">
+        <v>20</v>
+      </c>
+      <c r="L641" t="s">
+        <v>21</v>
+      </c>
+      <c r="M641">
+        <v>0</v>
+      </c>
+      <c r="N641">
+        <v>0</v>
+      </c>
+      <c r="O641"/>
+      <c r="P641"/>
+    </row>
+    <row r="642" spans="1:16">
+      <c r="A642" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B642" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C642"/>
+      <c r="D642" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E642" t="s">
+        <v>187</v>
+      </c>
+      <c r="F642"/>
+      <c r="G642"/>
+      <c r="H642"/>
+      <c r="I642"/>
+      <c r="J642"/>
+      <c r="K642" t="s">
+        <v>20</v>
+      </c>
+      <c r="L642" t="s">
+        <v>50</v>
+      </c>
+      <c r="M642">
+        <v>5</v>
+      </c>
+      <c r="N642">
+        <v>4</v>
+      </c>
+      <c r="O642">
+        <v>20</v>
+      </c>
+      <c r="P642"/>
+    </row>
+    <row r="643" spans="1:16">
+      <c r="A643" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B643" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C643"/>
+      <c r="D643" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E643" t="s">
+        <v>187</v>
+      </c>
+      <c r="F643"/>
+      <c r="G643"/>
+      <c r="H643"/>
+      <c r="I643"/>
+      <c r="J643"/>
+      <c r="K643" t="s">
+        <v>20</v>
+      </c>
+      <c r="L643" t="s">
+        <v>50</v>
+      </c>
+      <c r="M643">
+        <v>7</v>
+      </c>
+      <c r="N643">
+        <v>10</v>
+      </c>
+      <c r="O643">
+        <v>70</v>
+      </c>
+      <c r="P643"/>
+    </row>
+    <row r="644" spans="1:16">
+      <c r="A644" t="s">
+        <v>1180</v>
+      </c>
+      <c r="B644" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C644"/>
+      <c r="D644" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E644" t="s">
+        <v>187</v>
+      </c>
+      <c r="F644"/>
+      <c r="G644"/>
+      <c r="H644"/>
+      <c r="I644"/>
+      <c r="J644"/>
+      <c r="K644" t="s">
+        <v>20</v>
+      </c>
+      <c r="L644" t="s">
+        <v>50</v>
+      </c>
+      <c r="M644">
+        <v>11</v>
+      </c>
+      <c r="N644">
+        <v>6</v>
+      </c>
+      <c r="O644">
+        <v>66</v>
+      </c>
+      <c r="P644"/>
+    </row>
+    <row r="645" spans="1:16">
+      <c r="A645" t="s">
+        <v>1180</v>
+      </c>
+      <c r="B645" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C645"/>
+      <c r="D645" t="s">
+        <v>18</v>
+      </c>
+      <c r="E645" t="s">
+        <v>187</v>
+      </c>
+      <c r="F645"/>
+      <c r="G645"/>
+      <c r="H645"/>
+      <c r="I645"/>
+      <c r="J645"/>
+      <c r="K645" t="s">
+        <v>20</v>
+      </c>
+      <c r="L645" t="s">
+        <v>21</v>
+      </c>
+      <c r="M645">
+        <v>8</v>
+      </c>
+      <c r="N645">
+        <v>0</v>
+      </c>
+      <c r="O645"/>
+      <c r="P645"/>
+    </row>
+    <row r="646" spans="1:16">
+      <c r="A646" t="s">
+        <v>1180</v>
+      </c>
+      <c r="B646" t="s">
+        <v>1183</v>
+      </c>
+      <c r="C646"/>
+      <c r="D646" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E646" t="s">
+        <v>19</v>
+      </c>
+      <c r="F646"/>
+      <c r="G646"/>
+      <c r="H646"/>
+      <c r="I646"/>
+      <c r="J646"/>
+      <c r="K646" t="s">
+        <v>20</v>
+      </c>
+      <c r="L646" t="s">
         <v>75</v>
       </c>
-      <c r="M638">
+      <c r="M646">
+        <v>5</v>
+      </c>
+      <c r="N646">
+        <v>0</v>
+      </c>
+      <c r="O646"/>
+      <c r="P646"/>
+    </row>
+    <row r="647" spans="1:16">
+      <c r="A647" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B647" t="s">
+        <v>1186</v>
+      </c>
+      <c r="C647"/>
+      <c r="D647" t="s">
+        <v>1178</v>
+      </c>
+      <c r="E647" t="s">
+        <v>187</v>
+      </c>
+      <c r="F647"/>
+      <c r="G647"/>
+      <c r="H647"/>
+      <c r="I647"/>
+      <c r="J647"/>
+      <c r="K647" t="s">
+        <v>20</v>
+      </c>
+      <c r="L647" t="s">
+        <v>50</v>
+      </c>
+      <c r="M647">
+        <v>11</v>
+      </c>
+      <c r="N647">
+        <v>11</v>
+      </c>
+      <c r="O647">
+        <v>121</v>
+      </c>
+      <c r="P647"/>
+    </row>
+    <row r="648" spans="1:16">
+      <c r="A648" t="s">
+        <v>1185</v>
+      </c>
+      <c r="B648" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C648"/>
+      <c r="D648" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E648" t="s">
+        <v>19</v>
+      </c>
+      <c r="F648"/>
+      <c r="G648"/>
+      <c r="H648"/>
+      <c r="I648"/>
+      <c r="J648"/>
+      <c r="K648" t="s">
+        <v>20</v>
+      </c>
+      <c r="L648" t="s">
+        <v>21</v>
+      </c>
+      <c r="M648">
+        <v>5</v>
+      </c>
+      <c r="N648">
+        <v>0</v>
+      </c>
+      <c r="O648"/>
+      <c r="P648"/>
+    </row>
+    <row r="649" spans="1:16">
+      <c r="A649" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B649" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C649"/>
+      <c r="D649" t="s">
+        <v>1190</v>
+      </c>
+      <c r="E649" t="s">
+        <v>19</v>
+      </c>
+      <c r="F649"/>
+      <c r="G649"/>
+      <c r="H649"/>
+      <c r="I649"/>
+      <c r="J649"/>
+      <c r="K649" t="s">
+        <v>20</v>
+      </c>
+      <c r="L649" t="s">
+        <v>21</v>
+      </c>
+      <c r="M649">
+        <v>4</v>
+      </c>
+      <c r="N649">
+        <v>0</v>
+      </c>
+      <c r="O649"/>
+      <c r="P649"/>
+    </row>
+    <row r="650" spans="1:16">
+      <c r="A650" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B650" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C650"/>
+      <c r="D650" t="s">
+        <v>1193</v>
+      </c>
+      <c r="E650" t="s">
+        <v>19</v>
+      </c>
+      <c r="F650"/>
+      <c r="G650"/>
+      <c r="H650"/>
+      <c r="I650"/>
+      <c r="J650"/>
+      <c r="K650" t="s">
+        <v>20</v>
+      </c>
+      <c r="L650" t="s">
+        <v>21</v>
+      </c>
+      <c r="M650">
+        <v>3</v>
+      </c>
+      <c r="N650">
+        <v>0</v>
+      </c>
+      <c r="O650"/>
+      <c r="P650"/>
+    </row>
+    <row r="651" spans="1:16">
+      <c r="A651" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B651" t="s">
+        <v>1195</v>
+      </c>
+      <c r="C651"/>
+      <c r="D651" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E651" t="s">
+        <v>187</v>
+      </c>
+      <c r="F651"/>
+      <c r="G651"/>
+      <c r="H651"/>
+      <c r="I651"/>
+      <c r="J651"/>
+      <c r="K651" t="s">
+        <v>20</v>
+      </c>
+      <c r="L651" t="s">
+        <v>21</v>
+      </c>
+      <c r="M651">
+        <v>9</v>
+      </c>
+      <c r="N651">
+        <v>8</v>
+      </c>
+      <c r="O651">
+        <v>72</v>
+      </c>
+      <c r="P651"/>
+    </row>
+    <row r="652" spans="1:16">
+      <c r="A652" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B652" t="s">
+        <v>1197</v>
+      </c>
+      <c r="C652"/>
+      <c r="D652" t="s">
+        <v>228</v>
+      </c>
+      <c r="E652" t="s">
+        <v>19</v>
+      </c>
+      <c r="F652"/>
+      <c r="G652"/>
+      <c r="H652"/>
+      <c r="I652"/>
+      <c r="J652"/>
+      <c r="K652" t="s">
+        <v>20</v>
+      </c>
+      <c r="L652" t="s">
+        <v>21</v>
+      </c>
+      <c r="M652">
+        <v>11</v>
+      </c>
+      <c r="N652">
+        <v>0</v>
+      </c>
+      <c r="O652"/>
+      <c r="P652"/>
+    </row>
+    <row r="653" spans="1:16">
+      <c r="A653" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B653" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C653"/>
+      <c r="D653" t="s">
+        <v>1200</v>
+      </c>
+      <c r="E653" t="s">
+        <v>19</v>
+      </c>
+      <c r="F653"/>
+      <c r="G653"/>
+      <c r="H653"/>
+      <c r="I653"/>
+      <c r="J653"/>
+      <c r="K653" t="s">
+        <v>20</v>
+      </c>
+      <c r="L653" t="s">
+        <v>21</v>
+      </c>
+      <c r="M653">
+        <v>3</v>
+      </c>
+      <c r="N653">
+        <v>0</v>
+      </c>
+      <c r="O653"/>
+      <c r="P653"/>
+    </row>
+    <row r="654" spans="1:16">
+      <c r="A654" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B654" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C654"/>
+      <c r="D654" t="s">
+        <v>1201</v>
+      </c>
+      <c r="E654" t="s">
+        <v>19</v>
+      </c>
+      <c r="F654"/>
+      <c r="G654"/>
+      <c r="H654"/>
+      <c r="I654"/>
+      <c r="J654"/>
+      <c r="K654" t="s">
+        <v>20</v>
+      </c>
+      <c r="L654" t="s">
+        <v>21</v>
+      </c>
+      <c r="M654">
+        <v>3</v>
+      </c>
+      <c r="N654">
+        <v>0</v>
+      </c>
+      <c r="O654"/>
+      <c r="P654"/>
+    </row>
+    <row r="655" spans="1:16">
+      <c r="A655" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B655" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C655"/>
+      <c r="D655" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E655" t="s">
+        <v>19</v>
+      </c>
+      <c r="F655"/>
+      <c r="G655"/>
+      <c r="H655"/>
+      <c r="I655"/>
+      <c r="J655"/>
+      <c r="K655" t="s">
+        <v>20</v>
+      </c>
+      <c r="L655" t="s">
+        <v>21</v>
+      </c>
+      <c r="M655">
+        <v>1.5</v>
+      </c>
+      <c r="N655">
+        <v>0</v>
+      </c>
+      <c r="O655"/>
+      <c r="P655"/>
+    </row>
+    <row r="656" spans="1:16">
+      <c r="A656" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B656" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C656"/>
+      <c r="D656" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E656" t="s">
+        <v>19</v>
+      </c>
+      <c r="F656"/>
+      <c r="G656"/>
+      <c r="H656"/>
+      <c r="I656"/>
+      <c r="J656"/>
+      <c r="K656" t="s">
+        <v>20</v>
+      </c>
+      <c r="L656" t="s">
+        <v>21</v>
+      </c>
+      <c r="M656">
+        <v>4</v>
+      </c>
+      <c r="N656">
+        <v>0</v>
+      </c>
+      <c r="O656"/>
+      <c r="P656"/>
+    </row>
+    <row r="657" spans="1:16">
+      <c r="A657" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B657" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C657"/>
+      <c r="D657" t="s">
+        <v>1206</v>
+      </c>
+      <c r="E657" t="s">
+        <v>187</v>
+      </c>
+      <c r="F657"/>
+      <c r="G657"/>
+      <c r="H657"/>
+      <c r="I657"/>
+      <c r="J657"/>
+      <c r="K657" t="s">
+        <v>20</v>
+      </c>
+      <c r="L657" t="s">
+        <v>75</v>
+      </c>
+      <c r="M657">
         <v>120</v>
       </c>
-      <c r="N638">
-        <v>2</v>
-      </c>
-      <c r="O638">
-        <v>240</v>
-      </c>
-      <c r="P638"/>
+      <c r="N657">
+        <v>4</v>
+      </c>
+      <c r="O657">
+        <v>480</v>
+      </c>
+      <c r="P657"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour DPS — 06/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1208">
   <si>
     <t>Début</t>
   </si>
@@ -3397,7 +3397,7 @@
     <t>07-05-2026</t>
   </si>
   <si>
-    <t>Soirée Électronique - Boiler Room J1</t>
+    <t>Soirée Électronique - Boiler Room Paris J1</t>
   </si>
   <si>
     <t>Parc floral, Hall de la p</t>
@@ -3448,6 +3448,18 @@
     <t>Renfort DPS-ME - Concert Twice J2</t>
   </si>
   <si>
+    <t>18-05-2026</t>
+  </si>
+  <si>
+    <t>Renfort Concert Conan Gray - J1</t>
+  </si>
+  <si>
+    <t>19-05-2026</t>
+  </si>
+  <si>
+    <t>Renfort Concert Conan Gray - J2</t>
+  </si>
+  <si>
     <t>20-05-2026</t>
   </si>
   <si>
@@ -3460,33 +3472,15 @@
     <t xml:space="preserve">Gennevilliers </t>
   </si>
   <si>
-    <t>Festival Educ'Sport</t>
-  </si>
-  <si>
-    <t>Paris - UFR Cité Paris</t>
-  </si>
-  <si>
-    <t>22-05-2026</t>
-  </si>
-  <si>
-    <t>[Prov] Le Cercle Festival J1</t>
+    <t>Salon SantExpo</t>
   </si>
   <si>
     <t>23-05-2026</t>
   </si>
   <si>
-    <t>[Prov] Le Cercle Festival J2</t>
-  </si>
-  <si>
     <t>24-05-2026</t>
   </si>
   <si>
-    <t>[Prov] Le Cercle Festival J3</t>
-  </si>
-  <si>
-    <t>[Prov]course du Château de Vincennes</t>
-  </si>
-  <si>
     <t>27-05-2026</t>
   </si>
   <si>
@@ -3497,6 +3491,15 @@
   </si>
   <si>
     <t>Course Amnestienne</t>
+  </si>
+  <si>
+    <t>31-05-2026</t>
+  </si>
+  <si>
+    <t>Relais de la SPA</t>
+  </si>
+  <si>
+    <t>Domaine National de Saint</t>
   </si>
   <si>
     <t>02-06-2026</t>
@@ -27644,7 +27647,7 @@
         <v>0</v>
       </c>
       <c r="J612">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K612" t="s">
         <v>20</v>
@@ -27677,11 +27680,21 @@
       <c r="E613" t="s">
         <v>19</v>
       </c>
-      <c r="F613"/>
-      <c r="G613"/>
-      <c r="H613"/>
-      <c r="I613"/>
-      <c r="J613"/>
+      <c r="F613">
+        <v>4</v>
+      </c>
+      <c r="G613">
+        <v>0</v>
+      </c>
+      <c r="H613">
+        <v>0</v>
+      </c>
+      <c r="I613">
+        <v>0</v>
+      </c>
+      <c r="J613">
+        <v>0</v>
+      </c>
       <c r="K613" t="s">
         <v>20</v>
       </c>
@@ -27713,11 +27726,21 @@
       <c r="E614" t="s">
         <v>19</v>
       </c>
-      <c r="F614"/>
-      <c r="G614"/>
-      <c r="H614"/>
-      <c r="I614"/>
-      <c r="J614"/>
+      <c r="F614">
+        <v>1</v>
+      </c>
+      <c r="G614">
+        <v>0</v>
+      </c>
+      <c r="H614">
+        <v>0</v>
+      </c>
+      <c r="I614">
+        <v>0</v>
+      </c>
+      <c r="J614">
+        <v>0</v>
+      </c>
       <c r="K614" t="s">
         <v>20</v>
       </c>
@@ -27764,10 +27787,10 @@
         <v>12</v>
       </c>
       <c r="N615">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O615">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="P615"/>
     </row>
@@ -27783,7 +27806,7 @@
         <v>1130</v>
       </c>
       <c r="E616" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F616"/>
       <c r="G616"/>
@@ -27800,10 +27823,10 @@
         <v>12</v>
       </c>
       <c r="N616">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="O616">
-        <v>120</v>
+        <v>156</v>
       </c>
       <c r="P616"/>
     </row>
@@ -27819,7 +27842,7 @@
         <v>1133</v>
       </c>
       <c r="E617" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F617"/>
       <c r="G617"/>
@@ -27836,10 +27859,10 @@
         <v>7</v>
       </c>
       <c r="N617">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O617">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P617"/>
     </row>
@@ -28016,10 +28039,10 @@
         <v>6</v>
       </c>
       <c r="N622">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O622">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="P622"/>
     </row>
@@ -28028,14 +28051,14 @@
         <v>1143</v>
       </c>
       <c r="B623" t="s">
-        <v>192</v>
+        <v>1144</v>
       </c>
       <c r="C623"/>
       <c r="D623" t="s">
-        <v>34</v>
+        <v>362</v>
       </c>
       <c r="E623" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F623"/>
       <c r="G623"/>
@@ -28046,29 +28069,27 @@
         <v>20</v>
       </c>
       <c r="L623" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M623">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="N623">
-        <v>4</v>
-      </c>
-      <c r="O623">
-        <v>24</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O623"/>
       <c r="P623"/>
     </row>
     <row r="624" spans="1:16">
       <c r="A624" t="s">
-        <v>1143</v>
+        <v>1145</v>
       </c>
       <c r="B624" t="s">
-        <v>1110</v>
+        <v>1146</v>
       </c>
       <c r="C624"/>
       <c r="D624" t="s">
-        <v>539</v>
+        <v>362</v>
       </c>
       <c r="E624" t="s">
         <v>187</v>
@@ -28082,29 +28103,29 @@
         <v>20</v>
       </c>
       <c r="L624" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M624">
-        <v>9.5</v>
+        <v>5.5</v>
       </c>
       <c r="N624">
         <v>2</v>
       </c>
       <c r="O624">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="P624"/>
     </row>
     <row r="625" spans="1:16">
       <c r="A625" t="s">
-        <v>1144</v>
+        <v>1147</v>
       </c>
       <c r="B625" t="s">
-        <v>1145</v>
+        <v>192</v>
       </c>
       <c r="C625"/>
       <c r="D625" t="s">
-        <v>1146</v>
+        <v>34</v>
       </c>
       <c r="E625" t="s">
         <v>19</v>
@@ -28121,24 +28142,26 @@
         <v>21</v>
       </c>
       <c r="M625">
-        <v>4.5</v>
+        <v>6</v>
       </c>
       <c r="N625">
-        <v>0</v>
-      </c>
-      <c r="O625"/>
+        <v>4</v>
+      </c>
+      <c r="O625">
+        <v>24</v>
+      </c>
       <c r="P625"/>
     </row>
     <row r="626" spans="1:16">
       <c r="A626" t="s">
-        <v>1144</v>
+        <v>1147</v>
       </c>
       <c r="B626" t="s">
-        <v>1147</v>
+        <v>1110</v>
       </c>
       <c r="C626"/>
       <c r="D626" t="s">
-        <v>1148</v>
+        <v>539</v>
       </c>
       <c r="E626" t="s">
         <v>187</v>
@@ -28155,29 +28178,29 @@
         <v>21</v>
       </c>
       <c r="M626">
-        <v>12</v>
+        <v>9.5</v>
       </c>
       <c r="N626">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O626">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="P626"/>
     </row>
     <row r="627" spans="1:16">
       <c r="A627" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B627" t="s">
         <v>1149</v>
-      </c>
-      <c r="B627" t="s">
-        <v>1150</v>
       </c>
       <c r="C627"/>
       <c r="D627" t="s">
-        <v>259</v>
+        <v>1150</v>
       </c>
       <c r="E627" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F627"/>
       <c r="G627"/>
@@ -28191,26 +28214,24 @@
         <v>21</v>
       </c>
       <c r="M627">
-        <v>5.98</v>
+        <v>4.5</v>
       </c>
       <c r="N627">
-        <v>2</v>
-      </c>
-      <c r="O627">
-        <v>11.960000038147</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O627"/>
       <c r="P627"/>
     </row>
     <row r="628" spans="1:16">
       <c r="A628" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B628" t="s">
         <v>1151</v>
-      </c>
-      <c r="B628" t="s">
-        <v>1152</v>
       </c>
       <c r="C628"/>
       <c r="D628" t="s">
-        <v>259</v>
+        <v>610</v>
       </c>
       <c r="E628" t="s">
         <v>187</v>
@@ -28227,26 +28248,26 @@
         <v>21</v>
       </c>
       <c r="M628">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N628">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O628">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="P628"/>
     </row>
     <row r="629" spans="1:16">
       <c r="A629" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B629" t="s">
-        <v>1154</v>
+        <v>421</v>
       </c>
       <c r="C629"/>
       <c r="D629" t="s">
-        <v>259</v>
+        <v>18</v>
       </c>
       <c r="E629" t="s">
         <v>187</v>
@@ -28263,14 +28284,12 @@
         <v>21</v>
       </c>
       <c r="M629">
-        <v>12</v>
+        <v>6.02</v>
       </c>
       <c r="N629">
-        <v>2</v>
-      </c>
-      <c r="O629">
-        <v>24</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O629"/>
       <c r="P629"/>
     </row>
     <row r="630" spans="1:16">
@@ -28278,11 +28297,11 @@
         <v>1153</v>
       </c>
       <c r="B630" t="s">
-        <v>1155</v>
+        <v>1110</v>
       </c>
       <c r="C630"/>
       <c r="D630" t="s">
-        <v>476</v>
+        <v>539</v>
       </c>
       <c r="E630" t="s">
         <v>187</v>
@@ -28299,26 +28318,26 @@
         <v>21</v>
       </c>
       <c r="M630">
-        <v>5</v>
+        <v>11.5</v>
       </c>
       <c r="N630">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O630">
-        <v>15</v>
+        <v>69</v>
       </c>
       <c r="P630"/>
     </row>
     <row r="631" spans="1:16">
       <c r="A631" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="B631" t="s">
-        <v>1110</v>
+        <v>1155</v>
       </c>
       <c r="C631"/>
       <c r="D631" t="s">
-        <v>539</v>
+        <v>34</v>
       </c>
       <c r="E631" t="s">
         <v>187</v>
@@ -28335,13 +28354,13 @@
         <v>21</v>
       </c>
       <c r="M631">
-        <v>11.5</v>
+        <v>5.5</v>
       </c>
       <c r="N631">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O631">
-        <v>11.5</v>
+        <v>16.5</v>
       </c>
       <c r="P631"/>
     </row>
@@ -28354,7 +28373,7 @@
       </c>
       <c r="C632"/>
       <c r="D632" t="s">
-        <v>34</v>
+        <v>589</v>
       </c>
       <c r="E632" t="s">
         <v>187</v>
@@ -28371,13 +28390,13 @@
         <v>21</v>
       </c>
       <c r="M632">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="N632">
         <v>2</v>
       </c>
       <c r="O632">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P632"/>
     </row>
@@ -28390,7 +28409,7 @@
       </c>
       <c r="C633"/>
       <c r="D633" t="s">
-        <v>589</v>
+        <v>1160</v>
       </c>
       <c r="E633" t="s">
         <v>187</v>
@@ -28407,26 +28426,26 @@
         <v>21</v>
       </c>
       <c r="M633">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N633">
         <v>2</v>
       </c>
       <c r="O633">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P633"/>
     </row>
     <row r="634" spans="1:16">
       <c r="A634" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="B634" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="C634"/>
       <c r="D634" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="E634" t="s">
         <v>187</v>
@@ -28453,10 +28472,10 @@
     </row>
     <row r="635" spans="1:16">
       <c r="A635" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="B635" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="C635"/>
       <c r="D635" t="s">
@@ -28489,14 +28508,14 @@
     </row>
     <row r="636" spans="1:16">
       <c r="A636" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="B636" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="C636"/>
       <c r="D636" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="E636" t="s">
         <v>187</v>
@@ -28523,14 +28542,14 @@
     </row>
     <row r="637" spans="1:16">
       <c r="A637" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="B637" t="s">
         <v>778</v>
       </c>
       <c r="C637"/>
       <c r="D637" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="E637" t="s">
         <v>187</v>
@@ -28550,23 +28569,23 @@
         <v>10</v>
       </c>
       <c r="N637">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O637">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="P637"/>
     </row>
     <row r="638" spans="1:16">
       <c r="A638" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="B638" t="s">
         <v>780</v>
       </c>
       <c r="C638"/>
       <c r="D638" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="E638" t="s">
         <v>187</v>
@@ -28595,14 +28614,14 @@
     </row>
     <row r="639" spans="1:16">
       <c r="A639" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="B639" t="s">
         <v>643</v>
       </c>
       <c r="C639"/>
       <c r="D639" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="E639" t="s">
         <v>187</v>
@@ -28629,10 +28648,10 @@
     </row>
     <row r="640" spans="1:16">
       <c r="A640" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="B640" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="C640"/>
       <c r="D640" t="s">
@@ -28665,10 +28684,10 @@
     </row>
     <row r="641" spans="1:16">
       <c r="A641" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="B641" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="C641"/>
       <c r="D641" t="s">
@@ -28699,14 +28718,14 @@
     </row>
     <row r="642" spans="1:16">
       <c r="A642" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="B642" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="C642"/>
       <c r="D642" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="E642" t="s">
         <v>187</v>
@@ -28735,14 +28754,14 @@
     </row>
     <row r="643" spans="1:16">
       <c r="A643" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="B643" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="C643"/>
       <c r="D643" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="E643" t="s">
         <v>187</v>
@@ -28762,23 +28781,23 @@
         <v>7</v>
       </c>
       <c r="N643">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O643">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P643"/>
     </row>
     <row r="644" spans="1:16">
       <c r="A644" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="B644" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="C644"/>
       <c r="D644" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="E644" t="s">
         <v>187</v>
@@ -28807,10 +28826,10 @@
     </row>
     <row r="645" spans="1:16">
       <c r="A645" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="B645" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="C645"/>
       <c r="D645" t="s">
@@ -28841,14 +28860,14 @@
     </row>
     <row r="646" spans="1:16">
       <c r="A646" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="B646" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="C646"/>
       <c r="D646" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="E646" t="s">
         <v>19</v>
@@ -28875,14 +28894,14 @@
     </row>
     <row r="647" spans="1:16">
       <c r="A647" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="B647" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="C647"/>
       <c r="D647" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="E647" t="s">
         <v>187</v>
@@ -28902,23 +28921,23 @@
         <v>11</v>
       </c>
       <c r="N647">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O647">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="P647"/>
     </row>
     <row r="648" spans="1:16">
       <c r="A648" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="B648" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="C648"/>
       <c r="D648" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="E648" t="s">
         <v>19</v>
@@ -28945,14 +28964,14 @@
     </row>
     <row r="649" spans="1:16">
       <c r="A649" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="B649" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="C649"/>
       <c r="D649" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="E649" t="s">
         <v>19</v>
@@ -28979,14 +28998,14 @@
     </row>
     <row r="650" spans="1:16">
       <c r="A650" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="B650" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="C650"/>
       <c r="D650" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="E650" t="s">
         <v>19</v>
@@ -29013,14 +29032,14 @@
     </row>
     <row r="651" spans="1:16">
       <c r="A651" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="B651" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="C651"/>
       <c r="D651" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="E651" t="s">
         <v>187</v>
@@ -29049,10 +29068,10 @@
     </row>
     <row r="652" spans="1:16">
       <c r="A652" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="B652" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="C652"/>
       <c r="D652" t="s">
@@ -29083,14 +29102,14 @@
     </row>
     <row r="653" spans="1:16">
       <c r="A653" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="B653" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C653"/>
       <c r="D653" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="E653" t="s">
         <v>19</v>
@@ -29117,14 +29136,14 @@
     </row>
     <row r="654" spans="1:16">
       <c r="A654" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="B654" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C654"/>
       <c r="D654" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="E654" t="s">
         <v>19</v>
@@ -29151,14 +29170,14 @@
     </row>
     <row r="655" spans="1:16">
       <c r="A655" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="B655" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C655"/>
       <c r="D655" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="E655" t="s">
         <v>19</v>
@@ -29185,14 +29204,14 @@
     </row>
     <row r="656" spans="1:16">
       <c r="A656" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="B656" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C656"/>
       <c r="D656" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="E656" t="s">
         <v>19</v>
@@ -29219,14 +29238,14 @@
     </row>
     <row r="657" spans="1:16">
       <c r="A657" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="B657" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="C657"/>
       <c r="D657" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="E657" t="s">
         <v>187</v>

</xml_diff>

<commit_message>
Mise à jour DPS — 13/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -28093,10 +28093,10 @@
         <v>9.02</v>
       </c>
       <c r="N622">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O622">
-        <v>45.100002288818</v>
+        <v>27.060001373291</v>
       </c>
       <c r="P622"/>
     </row>
@@ -28112,7 +28112,7 @@
         <v>34</v>
       </c>
       <c r="E623" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F623"/>
       <c r="G623"/>
@@ -28129,10 +28129,10 @@
         <v>6</v>
       </c>
       <c r="N623">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O623">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="P623"/>
     </row>
@@ -28201,9 +28201,11 @@
         <v>5.5</v>
       </c>
       <c r="N625">
-        <v>0</v>
-      </c>
-      <c r="O625"/>
+        <v>1</v>
+      </c>
+      <c r="O625">
+        <v>5.5</v>
+      </c>
       <c r="P625"/>
     </row>
     <row r="626" spans="1:16">
@@ -28271,10 +28273,10 @@
         <v>1.5</v>
       </c>
       <c r="N627">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O627">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="P627"/>
     </row>
@@ -28343,10 +28345,10 @@
         <v>9.5</v>
       </c>
       <c r="N629">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O629">
-        <v>25</v>
+        <v>47.5</v>
       </c>
       <c r="P629"/>
     </row>
@@ -28413,10 +28415,10 @@
         <v>10</v>
       </c>
       <c r="N631">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O631">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="P631"/>
     </row>
@@ -28449,10 +28451,10 @@
         <v>6.02</v>
       </c>
       <c r="N632">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O632">
-        <v>6.0199999809265</v>
+        <v>24.079999923706</v>
       </c>
       <c r="P632"/>
     </row>
@@ -28557,10 +28559,10 @@
         <v>8</v>
       </c>
       <c r="N635">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O635">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="P635"/>
     </row>
@@ -28576,7 +28578,7 @@
         <v>34</v>
       </c>
       <c r="E636" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F636"/>
       <c r="G636"/>
@@ -28665,10 +28667,10 @@
         <v>7</v>
       </c>
       <c r="N638">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O638">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="P638"/>
     </row>
@@ -28701,10 +28703,10 @@
         <v>6</v>
       </c>
       <c r="N639">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O639">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="P639"/>
     </row>
@@ -28983,9 +28985,11 @@
         <v>6</v>
       </c>
       <c r="N647">
-        <v>0</v>
-      </c>
-      <c r="O647"/>
+        <v>2</v>
+      </c>
+      <c r="O647">
+        <v>12</v>
+      </c>
       <c r="P647"/>
     </row>
     <row r="648" spans="1:16">
@@ -29087,10 +29091,10 @@
         <v>7</v>
       </c>
       <c r="N650">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O650">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="P650"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour DPS — 18/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1220">
   <si>
     <t>Début</t>
   </si>
@@ -3487,7 +3487,7 @@
     <t>24-05-2026</t>
   </si>
   <si>
-    <t>[PROV] PdP France Angleterre</t>
+    <t>Renfort France-Angleterre</t>
   </si>
   <si>
     <t>26-05-2026</t>
@@ -3508,6 +3508,12 @@
     <t>PLDA</t>
   </si>
   <si>
+    <t>29-05-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Concert Bouss</t>
+  </si>
+  <si>
     <t>30-05-2026</t>
   </si>
   <si>
@@ -3530,6 +3536,12 @@
   </si>
   <si>
     <t xml:space="preserve">Stade Charlety </t>
+  </si>
+  <si>
+    <t>06-06-2026</t>
+  </si>
+  <si>
+    <t>On sla coule 12</t>
   </si>
   <si>
     <t>07-06-2026</t>
@@ -4021,7 +4033,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P664"/>
+  <dimension ref="A1:P666"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854004" bestFit="true" customWidth="true" style="0"/>
@@ -28078,11 +28090,21 @@
       <c r="E622" t="s">
         <v>19</v>
       </c>
-      <c r="F622"/>
-      <c r="G622"/>
-      <c r="H622"/>
-      <c r="I622"/>
-      <c r="J622"/>
+      <c r="F622">
+        <v>4</v>
+      </c>
+      <c r="G622">
+        <v>0</v>
+      </c>
+      <c r="H622">
+        <v>0</v>
+      </c>
+      <c r="I622">
+        <v>0</v>
+      </c>
+      <c r="J622">
+        <v>0</v>
+      </c>
       <c r="K622" t="s">
         <v>20</v>
       </c>
@@ -28148,7 +28170,7 @@
         <v>34</v>
       </c>
       <c r="E624" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F624"/>
       <c r="G624"/>
@@ -28165,10 +28187,10 @@
         <v>6</v>
       </c>
       <c r="N624">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O624">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="P624"/>
     </row>
@@ -28184,7 +28206,7 @@
         <v>362</v>
       </c>
       <c r="E625" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F625"/>
       <c r="G625"/>
@@ -28220,7 +28242,7 @@
         <v>362</v>
       </c>
       <c r="E626" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F626"/>
       <c r="G626"/>
@@ -28256,7 +28278,7 @@
         <v>589</v>
       </c>
       <c r="E627" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F627"/>
       <c r="G627"/>
@@ -28328,7 +28350,7 @@
         <v>539</v>
       </c>
       <c r="E629" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F629"/>
       <c r="G629"/>
@@ -28398,7 +28420,7 @@
         <v>610</v>
       </c>
       <c r="E631" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F631"/>
       <c r="G631"/>
@@ -28487,10 +28509,10 @@
         <v>11.5</v>
       </c>
       <c r="N633">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O633">
-        <v>103.5</v>
+        <v>126.5</v>
       </c>
       <c r="P633"/>
     </row>
@@ -28506,7 +28528,7 @@
         <v>55</v>
       </c>
       <c r="E634" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F634"/>
       <c r="G634"/>
@@ -28517,7 +28539,7 @@
         <v>20</v>
       </c>
       <c r="L634" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M634">
         <v>5</v>
@@ -28559,10 +28581,10 @@
         <v>8</v>
       </c>
       <c r="N635">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O635">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="P635"/>
     </row>
@@ -28631,10 +28653,10 @@
         <v>7.25</v>
       </c>
       <c r="N637">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O637">
-        <v>43.5</v>
+        <v>65.25</v>
       </c>
       <c r="P637"/>
     </row>
@@ -28647,7 +28669,7 @@
       </c>
       <c r="C638"/>
       <c r="D638" t="s">
-        <v>589</v>
+        <v>34</v>
       </c>
       <c r="E638" t="s">
         <v>187</v>
@@ -28664,13 +28686,13 @@
         <v>21</v>
       </c>
       <c r="M638">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N638">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O638">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="P638"/>
     </row>
@@ -28683,7 +28705,7 @@
       </c>
       <c r="C639"/>
       <c r="D639" t="s">
-        <v>1167</v>
+        <v>589</v>
       </c>
       <c r="E639" t="s">
         <v>187</v>
@@ -28700,26 +28722,26 @@
         <v>21</v>
       </c>
       <c r="M639">
+        <v>7</v>
+      </c>
+      <c r="N639">
         <v>6</v>
       </c>
-      <c r="N639">
-        <v>5</v>
-      </c>
       <c r="O639">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="P639"/>
     </row>
     <row r="640" spans="1:16">
       <c r="A640" t="s">
+        <v>1167</v>
+      </c>
+      <c r="B640" t="s">
         <v>1168</v>
-      </c>
-      <c r="B640" t="s">
-        <v>1169</v>
       </c>
       <c r="C640"/>
       <c r="D640" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="E640" t="s">
         <v>187</v>
@@ -28733,29 +28755,29 @@
         <v>20</v>
       </c>
       <c r="L640" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M640">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N640">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O640">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="P640"/>
     </row>
     <row r="641" spans="1:16">
       <c r="A641" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B641" t="s">
         <v>1171</v>
-      </c>
-      <c r="B641" t="s">
-        <v>1172</v>
       </c>
       <c r="C641"/>
       <c r="D641" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="E641" t="s">
         <v>187</v>
@@ -28769,27 +28791,29 @@
         <v>20</v>
       </c>
       <c r="L641" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M641">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N641">
-        <v>0</v>
-      </c>
-      <c r="O641"/>
+        <v>1</v>
+      </c>
+      <c r="O641">
+        <v>2</v>
+      </c>
       <c r="P641"/>
     </row>
     <row r="642" spans="1:16">
       <c r="A642" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B642" t="s">
         <v>1174</v>
-      </c>
-      <c r="B642" t="s">
-        <v>778</v>
       </c>
       <c r="C642"/>
       <c r="D642" t="s">
-        <v>1175</v>
+        <v>179</v>
       </c>
       <c r="E642" t="s">
         <v>187</v>
@@ -28803,29 +28827,27 @@
         <v>20</v>
       </c>
       <c r="L642" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="M642">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N642">
-        <v>11</v>
-      </c>
-      <c r="O642">
-        <v>110</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O642"/>
       <c r="P642"/>
     </row>
     <row r="643" spans="1:16">
       <c r="A643" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B643" t="s">
         <v>1176</v>
-      </c>
-      <c r="B643" t="s">
-        <v>780</v>
       </c>
       <c r="C643"/>
       <c r="D643" t="s">
-        <v>1175</v>
+        <v>1177</v>
       </c>
       <c r="E643" t="s">
         <v>187</v>
@@ -28839,29 +28861,29 @@
         <v>20</v>
       </c>
       <c r="L643" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M643">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N643">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O643">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="P643"/>
     </row>
     <row r="644" spans="1:16">
       <c r="A644" t="s">
-        <v>1176</v>
+        <v>1178</v>
       </c>
       <c r="B644" t="s">
-        <v>643</v>
+        <v>778</v>
       </c>
       <c r="C644"/>
       <c r="D644" t="s">
-        <v>1177</v>
+        <v>1179</v>
       </c>
       <c r="E644" t="s">
         <v>187</v>
@@ -28875,27 +28897,29 @@
         <v>20</v>
       </c>
       <c r="L644" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M644">
-        <v>8.25</v>
+        <v>10</v>
       </c>
       <c r="N644">
-        <v>0</v>
-      </c>
-      <c r="O644"/>
+        <v>12</v>
+      </c>
+      <c r="O644">
+        <v>120</v>
+      </c>
       <c r="P644"/>
     </row>
     <row r="645" spans="1:16">
       <c r="A645" t="s">
-        <v>1178</v>
+        <v>1180</v>
       </c>
       <c r="B645" t="s">
-        <v>546</v>
+        <v>780</v>
       </c>
       <c r="C645"/>
       <c r="D645" t="s">
-        <v>34</v>
+        <v>1179</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -28909,27 +28933,29 @@
         <v>20</v>
       </c>
       <c r="L645" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M645">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N645">
-        <v>0</v>
-      </c>
-      <c r="O645"/>
+        <v>4</v>
+      </c>
+      <c r="O645">
+        <v>36</v>
+      </c>
       <c r="P645"/>
     </row>
     <row r="646" spans="1:16">
       <c r="A646" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="B646" t="s">
-        <v>1180</v>
+        <v>643</v>
       </c>
       <c r="C646"/>
       <c r="D646" t="s">
-        <v>205</v>
+        <v>1181</v>
       </c>
       <c r="E646" t="s">
         <v>187</v>
@@ -28943,25 +28969,23 @@
         <v>20</v>
       </c>
       <c r="L646" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M646">
-        <v>7</v>
+        <v>8.25</v>
       </c>
       <c r="N646">
-        <v>4</v>
-      </c>
-      <c r="O646">
-        <v>28</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O646"/>
       <c r="P646"/>
     </row>
     <row r="647" spans="1:16">
       <c r="A647" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="B647" t="s">
-        <v>1182</v>
+        <v>546</v>
       </c>
       <c r="C647"/>
       <c r="D647" t="s">
@@ -28985,11 +29009,9 @@
         <v>6</v>
       </c>
       <c r="N647">
-        <v>2</v>
-      </c>
-      <c r="O647">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O647"/>
       <c r="P647"/>
     </row>
     <row r="648" spans="1:16">
@@ -29001,7 +29023,7 @@
       </c>
       <c r="C648"/>
       <c r="D648" t="s">
-        <v>18</v>
+        <v>205</v>
       </c>
       <c r="E648" t="s">
         <v>187</v>
@@ -29018,12 +29040,14 @@
         <v>21</v>
       </c>
       <c r="M648">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N648">
-        <v>0</v>
-      </c>
-      <c r="O648"/>
+        <v>4</v>
+      </c>
+      <c r="O648">
+        <v>28</v>
+      </c>
       <c r="P648"/>
     </row>
     <row r="649" spans="1:16">
@@ -29035,7 +29059,7 @@
       </c>
       <c r="C649"/>
       <c r="D649" t="s">
-        <v>1187</v>
+        <v>34</v>
       </c>
       <c r="E649" t="s">
         <v>187</v>
@@ -29049,29 +29073,29 @@
         <v>20</v>
       </c>
       <c r="L649" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M649">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N649">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O649">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P649"/>
     </row>
     <row r="650" spans="1:16">
       <c r="A650" t="s">
-        <v>1185</v>
+        <v>1187</v>
       </c>
       <c r="B650" t="s">
         <v>1188</v>
       </c>
       <c r="C650"/>
       <c r="D650" t="s">
-        <v>1187</v>
+        <v>18</v>
       </c>
       <c r="E650" t="s">
         <v>187</v>
@@ -29085,17 +29109,15 @@
         <v>20</v>
       </c>
       <c r="L650" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M650">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N650">
-        <v>12</v>
-      </c>
-      <c r="O650">
-        <v>84</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O650"/>
       <c r="P650"/>
     </row>
     <row r="651" spans="1:16">
@@ -29107,7 +29129,7 @@
       </c>
       <c r="C651"/>
       <c r="D651" t="s">
-        <v>1187</v>
+        <v>1191</v>
       </c>
       <c r="E651" t="s">
         <v>187</v>
@@ -29124,13 +29146,13 @@
         <v>50</v>
       </c>
       <c r="M651">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N651">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O651">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="P651"/>
     </row>
@@ -29139,11 +29161,11 @@
         <v>1189</v>
       </c>
       <c r="B652" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="C652"/>
       <c r="D652" t="s">
-        <v>18</v>
+        <v>1191</v>
       </c>
       <c r="E652" t="s">
         <v>187</v>
@@ -29157,30 +29179,32 @@
         <v>20</v>
       </c>
       <c r="L652" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M652">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N652">
-        <v>0</v>
-      </c>
-      <c r="O652"/>
+        <v>12</v>
+      </c>
+      <c r="O652">
+        <v>84</v>
+      </c>
       <c r="P652"/>
     </row>
     <row r="653" spans="1:16">
       <c r="A653" t="s">
-        <v>1189</v>
+        <v>1193</v>
       </c>
       <c r="B653" t="s">
-        <v>1192</v>
+        <v>1194</v>
       </c>
       <c r="C653"/>
       <c r="D653" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="E653" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F653"/>
       <c r="G653"/>
@@ -29191,27 +29215,29 @@
         <v>20</v>
       </c>
       <c r="L653" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="M653">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N653">
-        <v>0</v>
-      </c>
-      <c r="O653"/>
+        <v>6</v>
+      </c>
+      <c r="O653">
+        <v>66</v>
+      </c>
       <c r="P653"/>
     </row>
     <row r="654" spans="1:16">
       <c r="A654" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="B654" t="s">
         <v>1195</v>
       </c>
       <c r="C654"/>
       <c r="D654" t="s">
-        <v>1187</v>
+        <v>18</v>
       </c>
       <c r="E654" t="s">
         <v>187</v>
@@ -29225,29 +29251,27 @@
         <v>20</v>
       </c>
       <c r="L654" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M654">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N654">
-        <v>10</v>
-      </c>
-      <c r="O654">
-        <v>110</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O654"/>
       <c r="P654"/>
     </row>
     <row r="655" spans="1:16">
       <c r="A655" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="B655" t="s">
         <v>1196</v>
       </c>
       <c r="C655"/>
       <c r="D655" t="s">
-        <v>1193</v>
+        <v>1197</v>
       </c>
       <c r="E655" t="s">
         <v>19</v>
@@ -29261,7 +29285,7 @@
         <v>20</v>
       </c>
       <c r="L655" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M655">
         <v>5</v>
@@ -29274,17 +29298,17 @@
     </row>
     <row r="656" spans="1:16">
       <c r="A656" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="B656" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="C656"/>
       <c r="D656" t="s">
-        <v>1199</v>
+        <v>1191</v>
       </c>
       <c r="E656" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F656"/>
       <c r="G656"/>
@@ -29295,27 +29319,29 @@
         <v>20</v>
       </c>
       <c r="L656" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M656">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N656">
-        <v>0</v>
-      </c>
-      <c r="O656"/>
+        <v>11</v>
+      </c>
+      <c r="O656">
+        <v>121</v>
+      </c>
       <c r="P656"/>
     </row>
     <row r="657" spans="1:16">
       <c r="A657" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B657" t="s">
         <v>1200</v>
-      </c>
-      <c r="B657" t="s">
-        <v>1201</v>
       </c>
       <c r="C657"/>
       <c r="D657" t="s">
-        <v>1202</v>
+        <v>1197</v>
       </c>
       <c r="E657" t="s">
         <v>19</v>
@@ -29332,7 +29358,7 @@
         <v>21</v>
       </c>
       <c r="M657">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N657">
         <v>0</v>
@@ -29342,17 +29368,17 @@
     </row>
     <row r="658" spans="1:16">
       <c r="A658" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="B658" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="C658"/>
       <c r="D658" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="E658" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F658"/>
       <c r="G658"/>
@@ -29366,26 +29392,24 @@
         <v>21</v>
       </c>
       <c r="M658">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="N658">
-        <v>8</v>
-      </c>
-      <c r="O658">
-        <v>72</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O658"/>
       <c r="P658"/>
     </row>
     <row r="659" spans="1:16">
       <c r="A659" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="B659" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C659"/>
       <c r="D659" t="s">
-        <v>228</v>
+        <v>1206</v>
       </c>
       <c r="E659" t="s">
         <v>19</v>
@@ -29402,7 +29426,7 @@
         <v>21</v>
       </c>
       <c r="M659">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="N659">
         <v>0</v>
@@ -29422,7 +29446,7 @@
         <v>1209</v>
       </c>
       <c r="E660" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="F660"/>
       <c r="G660"/>
@@ -29436,12 +29460,14 @@
         <v>21</v>
       </c>
       <c r="M660">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N660">
-        <v>0</v>
-      </c>
-      <c r="O660"/>
+        <v>8</v>
+      </c>
+      <c r="O660">
+        <v>72</v>
+      </c>
       <c r="P660"/>
     </row>
     <row r="661" spans="1:16">
@@ -29449,11 +29475,11 @@
         <v>1207</v>
       </c>
       <c r="B661" t="s">
-        <v>1208</v>
+        <v>1210</v>
       </c>
       <c r="C661"/>
       <c r="D661" t="s">
-        <v>1210</v>
+        <v>228</v>
       </c>
       <c r="E661" t="s">
         <v>19</v>
@@ -29470,7 +29496,7 @@
         <v>21</v>
       </c>
       <c r="M661">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N661">
         <v>0</v>
@@ -29480,14 +29506,14 @@
     </row>
     <row r="662" spans="1:16">
       <c r="A662" t="s">
-        <v>1207</v>
+        <v>1211</v>
       </c>
       <c r="B662" t="s">
-        <v>1208</v>
+        <v>1212</v>
       </c>
       <c r="C662"/>
       <c r="D662" t="s">
-        <v>1211</v>
+        <v>1213</v>
       </c>
       <c r="E662" t="s">
         <v>19</v>
@@ -29504,7 +29530,7 @@
         <v>21</v>
       </c>
       <c r="M662">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="N662">
         <v>0</v>
@@ -29514,14 +29540,14 @@
     </row>
     <row r="663" spans="1:16">
       <c r="A663" t="s">
-        <v>1207</v>
+        <v>1211</v>
       </c>
       <c r="B663" t="s">
-        <v>1208</v>
+        <v>1212</v>
       </c>
       <c r="C663"/>
       <c r="D663" t="s">
-        <v>1212</v>
+        <v>1214</v>
       </c>
       <c r="E663" t="s">
         <v>19</v>
@@ -29538,7 +29564,7 @@
         <v>21</v>
       </c>
       <c r="M663">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N663">
         <v>0</v>
@@ -29548,17 +29574,17 @@
     </row>
     <row r="664" spans="1:16">
       <c r="A664" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
       <c r="B664" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
       <c r="C664"/>
       <c r="D664" t="s">
         <v>1215</v>
       </c>
       <c r="E664" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="F664"/>
       <c r="G664"/>
@@ -29569,18 +29595,86 @@
         <v>20</v>
       </c>
       <c r="L664" t="s">
+        <v>21</v>
+      </c>
+      <c r="M664">
+        <v>1.5</v>
+      </c>
+      <c r="N664">
+        <v>0</v>
+      </c>
+      <c r="O664"/>
+      <c r="P664"/>
+    </row>
+    <row r="665" spans="1:16">
+      <c r="A665" t="s">
+        <v>1211</v>
+      </c>
+      <c r="B665" t="s">
+        <v>1212</v>
+      </c>
+      <c r="C665"/>
+      <c r="D665" t="s">
+        <v>1216</v>
+      </c>
+      <c r="E665" t="s">
+        <v>19</v>
+      </c>
+      <c r="F665"/>
+      <c r="G665"/>
+      <c r="H665"/>
+      <c r="I665"/>
+      <c r="J665"/>
+      <c r="K665" t="s">
+        <v>20</v>
+      </c>
+      <c r="L665" t="s">
+        <v>21</v>
+      </c>
+      <c r="M665">
+        <v>4</v>
+      </c>
+      <c r="N665">
+        <v>0</v>
+      </c>
+      <c r="O665"/>
+      <c r="P665"/>
+    </row>
+    <row r="666" spans="1:16">
+      <c r="A666" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B666" t="s">
+        <v>1218</v>
+      </c>
+      <c r="C666"/>
+      <c r="D666" t="s">
+        <v>1219</v>
+      </c>
+      <c r="E666" t="s">
+        <v>187</v>
+      </c>
+      <c r="F666"/>
+      <c r="G666"/>
+      <c r="H666"/>
+      <c r="I666"/>
+      <c r="J666"/>
+      <c r="K666" t="s">
+        <v>20</v>
+      </c>
+      <c r="L666" t="s">
         <v>75</v>
       </c>
-      <c r="M664">
+      <c r="M666">
         <v>120</v>
       </c>
-      <c r="N664">
+      <c r="N666">
         <v>4</v>
       </c>
-      <c r="O664">
+      <c r="O666">
         <v>480</v>
       </c>
-      <c r="P664"/>
+      <c r="P666"/>
     </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>

</xml_diff>

<commit_message>
Mise à jour DPS — 19/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569F98DC-06A1-4A23-9D6D-BDBE3FE9C140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B37DDB-D671-4327-A780-117EAAFE16E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3990" uniqueCount="1217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3996" uniqueCount="1217">
   <si>
     <t>Début</t>
   </si>
@@ -3499,12 +3499,6 @@
     <t>28-05-2026</t>
   </si>
   <si>
-    <t>[PROV] Concert Damso</t>
-  </si>
-  <si>
-    <t>PLDA</t>
-  </si>
-  <si>
     <t>29-05-2026</t>
   </si>
   <si>
@@ -3674,6 +3668,12 @@
   </si>
   <si>
     <t>Carhaix (29)</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Rocket League Paris Major 2 (J3)</t>
+  </si>
+  <si>
+    <t>Renfort DPS-GE  - Concert DAMSO (J1)</t>
   </si>
 </sst>
 </file>
@@ -4028,7 +4028,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P663"/>
+  <dimension ref="A1:P664"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -24783,7 +24783,7 @@
         <v>18</v>
       </c>
       <c r="E629" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K629" t="s">
         <v>20</v>
@@ -24795,10 +24795,10 @@
         <v>6.02</v>
       </c>
       <c r="N629">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O629">
-        <v>24.079999923706001</v>
+        <v>30.099999904632998</v>
       </c>
     </row>
     <row r="630" spans="1:15" x14ac:dyDescent="0.35">
@@ -24824,10 +24824,10 @@
         <v>11.5</v>
       </c>
       <c r="N630">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O630">
-        <v>126.5</v>
+        <v>138</v>
       </c>
     </row>
     <row r="631" spans="1:15" x14ac:dyDescent="0.35">
@@ -24861,45 +24861,45 @@
     </row>
     <row r="632" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A632" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="B632" t="s">
-        <v>515</v>
+        <v>1215</v>
       </c>
       <c r="D632" t="s">
-        <v>516</v>
+        <v>60</v>
       </c>
       <c r="E632" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K632" t="s">
         <v>20</v>
       </c>
       <c r="L632" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M632">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N632">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O632">
-        <v>40</v>
+        <v>11</v>
       </c>
     </row>
     <row r="633" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A633" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B633" t="s">
-        <v>1156</v>
+        <v>515</v>
       </c>
       <c r="D633" t="s">
-        <v>34</v>
+        <v>516</v>
       </c>
       <c r="E633" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K633" t="s">
         <v>20</v>
@@ -24908,56 +24908,56 @@
         <v>21</v>
       </c>
       <c r="M633">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="N633">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O633">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="634" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A634" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="B634" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
       <c r="D634" t="s">
-        <v>1159</v>
+        <v>34</v>
       </c>
       <c r="E634" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K634" t="s">
         <v>20</v>
       </c>
       <c r="L634" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M634">
-        <v>7.25</v>
+        <v>5.5</v>
       </c>
       <c r="N634">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="O634">
-        <v>65.25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="635" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A635" t="s">
-        <v>1160</v>
+        <v>1157</v>
       </c>
       <c r="B635" t="s">
-        <v>1161</v>
+        <v>1216</v>
       </c>
       <c r="D635" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="E635" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K635" t="s">
         <v>20</v>
@@ -24966,24 +24966,24 @@
         <v>21</v>
       </c>
       <c r="M635">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="N635">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O635">
-        <v>11</v>
+        <v>63</v>
       </c>
     </row>
     <row r="636" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A636" t="s">
-        <v>1162</v>
+        <v>1158</v>
       </c>
       <c r="B636" t="s">
-        <v>1163</v>
+        <v>1159</v>
       </c>
       <c r="D636" t="s">
-        <v>589</v>
+        <v>34</v>
       </c>
       <c r="E636" t="s">
         <v>187</v>
@@ -24995,24 +24995,24 @@
         <v>21</v>
       </c>
       <c r="M636">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N636">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O636">
-        <v>42</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="637" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A637" t="s">
-        <v>1164</v>
+        <v>1160</v>
       </c>
       <c r="B637" t="s">
-        <v>1165</v>
+        <v>1161</v>
       </c>
       <c r="D637" t="s">
-        <v>1166</v>
+        <v>589</v>
       </c>
       <c r="E637" t="s">
         <v>187</v>
@@ -25024,24 +25024,24 @@
         <v>21</v>
       </c>
       <c r="M637">
+        <v>7</v>
+      </c>
+      <c r="N637">
         <v>6</v>
       </c>
-      <c r="N637">
-        <v>5</v>
-      </c>
       <c r="O637">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="638" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A638" t="s">
-        <v>1167</v>
+        <v>1162</v>
       </c>
       <c r="B638" t="s">
-        <v>1168</v>
+        <v>1163</v>
       </c>
       <c r="D638" t="s">
-        <v>1169</v>
+        <v>1164</v>
       </c>
       <c r="E638" t="s">
         <v>187</v>
@@ -25050,27 +25050,27 @@
         <v>20</v>
       </c>
       <c r="L638" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M638">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N638">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O638">
-        <v>2</v>
+        <v>36</v>
       </c>
     </row>
     <row r="639" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A639" t="s">
-        <v>1170</v>
+        <v>1165</v>
       </c>
       <c r="B639" t="s">
-        <v>1171</v>
+        <v>1166</v>
       </c>
       <c r="D639" t="s">
-        <v>179</v>
+        <v>1167</v>
       </c>
       <c r="E639" t="s">
         <v>187</v>
@@ -25079,24 +25079,27 @@
         <v>20</v>
       </c>
       <c r="L639" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="M639">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N639">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O639">
+        <v>4</v>
       </c>
     </row>
     <row r="640" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A640" t="s">
-        <v>1172</v>
+        <v>1168</v>
       </c>
       <c r="B640" t="s">
-        <v>1173</v>
+        <v>1169</v>
       </c>
       <c r="D640" t="s">
-        <v>1174</v>
+        <v>179</v>
       </c>
       <c r="E640" t="s">
         <v>187</v>
@@ -25105,27 +25108,27 @@
         <v>20</v>
       </c>
       <c r="L640" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M640">
         <v>6</v>
       </c>
       <c r="N640">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O640">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="641" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A641" t="s">
-        <v>1175</v>
+        <v>1170</v>
       </c>
       <c r="B641" t="s">
-        <v>775</v>
+        <v>1171</v>
       </c>
       <c r="D641" t="s">
-        <v>1176</v>
+        <v>1172</v>
       </c>
       <c r="E641" t="s">
         <v>187</v>
@@ -25134,27 +25137,27 @@
         <v>20</v>
       </c>
       <c r="L641" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M641">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N641">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="O641">
-        <v>120</v>
+        <v>6</v>
       </c>
     </row>
     <row r="642" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A642" t="s">
-        <v>1177</v>
+        <v>1173</v>
       </c>
       <c r="B642" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D642" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="E642" t="s">
         <v>187</v>
@@ -25166,24 +25169,24 @@
         <v>50</v>
       </c>
       <c r="M642">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N642">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="O642">
-        <v>36</v>
+        <v>140</v>
       </c>
     </row>
     <row r="643" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A643" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="B643" t="s">
-        <v>643</v>
+        <v>777</v>
       </c>
       <c r="D643" t="s">
-        <v>1178</v>
+        <v>1174</v>
       </c>
       <c r="E643" t="s">
         <v>187</v>
@@ -25192,24 +25195,27 @@
         <v>20</v>
       </c>
       <c r="L643" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M643">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="N643">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="O643">
+        <v>63</v>
       </c>
     </row>
     <row r="644" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A644" t="s">
-        <v>1179</v>
+        <v>1175</v>
       </c>
       <c r="B644" t="s">
-        <v>546</v>
+        <v>643</v>
       </c>
       <c r="D644" t="s">
-        <v>34</v>
+        <v>1176</v>
       </c>
       <c r="E644" t="s">
         <v>187</v>
@@ -25218,10 +25224,10 @@
         <v>20</v>
       </c>
       <c r="L644" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M644">
-        <v>6</v>
+        <v>8.25</v>
       </c>
       <c r="N644">
         <v>0</v>
@@ -25229,13 +25235,13 @@
     </row>
     <row r="645" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
-        <v>1180</v>
+        <v>1177</v>
       </c>
       <c r="B645" t="s">
-        <v>1181</v>
+        <v>546</v>
       </c>
       <c r="D645" t="s">
-        <v>205</v>
+        <v>34</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25247,24 +25253,21 @@
         <v>21</v>
       </c>
       <c r="M645">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N645">
-        <v>4</v>
-      </c>
-      <c r="O645">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="646" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B646" t="s">
-        <v>1183</v>
+        <v>1179</v>
       </c>
       <c r="D646" t="s">
-        <v>34</v>
+        <v>205</v>
       </c>
       <c r="E646" t="s">
         <v>187</v>
@@ -25276,24 +25279,24 @@
         <v>21</v>
       </c>
       <c r="M646">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N646">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O646">
-        <v>12</v>
+        <v>28</v>
       </c>
     </row>
     <row r="647" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
-        <v>1184</v>
+        <v>1180</v>
       </c>
       <c r="B647" t="s">
-        <v>1185</v>
+        <v>1181</v>
       </c>
       <c r="D647" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E647" t="s">
         <v>187</v>
@@ -25305,21 +25308,24 @@
         <v>21</v>
       </c>
       <c r="M647">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N647">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O647">
+        <v>12</v>
       </c>
     </row>
     <row r="648" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A648" t="s">
-        <v>1186</v>
+        <v>1182</v>
       </c>
       <c r="B648" t="s">
-        <v>1187</v>
+        <v>1183</v>
       </c>
       <c r="D648" t="s">
-        <v>1188</v>
+        <v>18</v>
       </c>
       <c r="E648" t="s">
         <v>187</v>
@@ -25328,27 +25334,24 @@
         <v>20</v>
       </c>
       <c r="L648" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M648">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N648">
-        <v>4</v>
-      </c>
-      <c r="O648">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="649" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B649" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D649" t="s">
         <v>1186</v>
-      </c>
-      <c r="B649" t="s">
-        <v>1189</v>
-      </c>
-      <c r="D649" t="s">
-        <v>1188</v>
       </c>
       <c r="E649" t="s">
         <v>187</v>
@@ -25360,24 +25363,24 @@
         <v>50</v>
       </c>
       <c r="M649">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N649">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="O649">
-        <v>84</v>
+        <v>25</v>
       </c>
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1190</v>
+        <v>1184</v>
       </c>
       <c r="B650" t="s">
-        <v>1191</v>
+        <v>1187</v>
       </c>
       <c r="D650" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="E650" t="s">
         <v>187</v>
@@ -25389,24 +25392,24 @@
         <v>50</v>
       </c>
       <c r="M650">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N650">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="O650">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="B651" t="s">
-        <v>1192</v>
+        <v>1189</v>
       </c>
       <c r="D651" t="s">
-        <v>18</v>
+        <v>1186</v>
       </c>
       <c r="E651" t="s">
         <v>187</v>
@@ -25415,36 +25418,39 @@
         <v>20</v>
       </c>
       <c r="L651" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M651">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N651">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="O651">
+        <v>66</v>
       </c>
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
+        <v>1188</v>
+      </c>
+      <c r="B652" t="s">
         <v>1190</v>
       </c>
-      <c r="B652" t="s">
-        <v>1193</v>
-      </c>
       <c r="D652" t="s">
-        <v>1194</v>
+        <v>18</v>
       </c>
       <c r="E652" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K652" t="s">
         <v>20</v>
       </c>
       <c r="L652" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M652">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N652">
         <v>0</v>
@@ -25452,68 +25458,68 @@
     </row>
     <row r="653" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
-        <v>1195</v>
+        <v>1188</v>
       </c>
       <c r="B653" t="s">
-        <v>1196</v>
+        <v>1191</v>
       </c>
       <c r="D653" t="s">
-        <v>1188</v>
+        <v>1192</v>
       </c>
       <c r="E653" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K653" t="s">
         <v>20</v>
       </c>
       <c r="L653" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="M653">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N653">
-        <v>11</v>
-      </c>
-      <c r="O653">
-        <v>121</v>
+        <v>0</v>
       </c>
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="B654" t="s">
-        <v>1197</v>
+        <v>1194</v>
       </c>
       <c r="D654" t="s">
-        <v>1194</v>
+        <v>1186</v>
       </c>
       <c r="E654" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K654" t="s">
         <v>20</v>
       </c>
       <c r="L654" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M654">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N654">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="O654">
+        <v>132</v>
       </c>
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1198</v>
+        <v>1193</v>
       </c>
       <c r="B655" t="s">
-        <v>1199</v>
+        <v>1195</v>
       </c>
       <c r="D655" t="s">
-        <v>1200</v>
+        <v>1192</v>
       </c>
       <c r="E655" t="s">
         <v>19</v>
@@ -25525,7 +25531,7 @@
         <v>21</v>
       </c>
       <c r="M655">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N655">
         <v>0</v>
@@ -25533,13 +25539,13 @@
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1201</v>
+        <v>1196</v>
       </c>
       <c r="B656" t="s">
-        <v>1202</v>
+        <v>1197</v>
       </c>
       <c r="D656" t="s">
-        <v>1203</v>
+        <v>1198</v>
       </c>
       <c r="E656" t="s">
         <v>19</v>
@@ -25551,7 +25557,7 @@
         <v>21</v>
       </c>
       <c r="M656">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N656">
         <v>0</v>
@@ -25559,16 +25565,16 @@
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1204</v>
+        <v>1199</v>
       </c>
       <c r="B657" t="s">
-        <v>1205</v>
+        <v>1200</v>
       </c>
       <c r="D657" t="s">
-        <v>1206</v>
+        <v>1201</v>
       </c>
       <c r="E657" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K657" t="s">
         <v>20</v>
@@ -25577,27 +25583,24 @@
         <v>21</v>
       </c>
       <c r="M657">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="N657">
-        <v>8</v>
-      </c>
-      <c r="O657">
-        <v>72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B658" t="s">
+        <v>1203</v>
+      </c>
+      <c r="D658" t="s">
         <v>1204</v>
       </c>
-      <c r="B658" t="s">
-        <v>1207</v>
-      </c>
-      <c r="D658" t="s">
-        <v>228</v>
-      </c>
       <c r="E658" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K658" t="s">
         <v>20</v>
@@ -25606,21 +25609,24 @@
         <v>21</v>
       </c>
       <c r="M658">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="N658">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="O658">
+        <v>72</v>
       </c>
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1208</v>
+        <v>1202</v>
       </c>
       <c r="B659" t="s">
-        <v>1209</v>
+        <v>1205</v>
       </c>
       <c r="D659" t="s">
-        <v>1210</v>
+        <v>228</v>
       </c>
       <c r="E659" t="s">
         <v>19</v>
@@ -25632,7 +25638,7 @@
         <v>21</v>
       </c>
       <c r="M659">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N659">
         <v>0</v>
@@ -25640,13 +25646,13 @@
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B660" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D660" t="s">
         <v>1208</v>
-      </c>
-      <c r="B660" t="s">
-        <v>1209</v>
-      </c>
-      <c r="D660" t="s">
-        <v>1211</v>
       </c>
       <c r="E660" t="s">
         <v>19</v>
@@ -25666,14 +25672,14 @@
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="B661" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D661" t="s">
         <v>1209</v>
       </c>
-      <c r="D661" t="s">
-        <v>1212</v>
-      </c>
       <c r="E661" t="s">
         <v>19</v>
       </c>
@@ -25684,7 +25690,7 @@
         <v>21</v>
       </c>
       <c r="M661">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="N661">
         <v>0</v>
@@ -25692,13 +25698,13 @@
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="B662" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="D662" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="E662" t="s">
         <v>19</v>
@@ -25710,7 +25716,7 @@
         <v>21</v>
       </c>
       <c r="M662">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="N662">
         <v>0</v>
@@ -25718,30 +25724,56 @@
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B663" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D663" t="s">
+        <v>1211</v>
+      </c>
+      <c r="E663" t="s">
+        <v>19</v>
+      </c>
+      <c r="K663" t="s">
+        <v>20</v>
+      </c>
+      <c r="L663" t="s">
+        <v>21</v>
+      </c>
+      <c r="M663">
+        <v>4</v>
+      </c>
+      <c r="N663">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="664" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A664" t="s">
+        <v>1212</v>
+      </c>
+      <c r="B664" t="s">
+        <v>1213</v>
+      </c>
+      <c r="D664" t="s">
         <v>1214</v>
       </c>
-      <c r="B663" t="s">
-        <v>1215</v>
-      </c>
-      <c r="D663" t="s">
-        <v>1216</v>
-      </c>
-      <c r="E663" t="s">
+      <c r="E664" t="s">
         <v>187</v>
       </c>
-      <c r="K663" t="s">
-        <v>20</v>
-      </c>
-      <c r="L663" t="s">
+      <c r="K664" t="s">
+        <v>20</v>
+      </c>
+      <c r="L664" t="s">
         <v>75</v>
       </c>
-      <c r="M663">
+      <c r="M664">
         <v>120</v>
       </c>
-      <c r="N663">
+      <c r="N664">
         <v>4</v>
       </c>
-      <c r="O663">
+      <c r="O664">
         <v>480</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour DPS — 21/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B37DDB-D671-4327-A780-117EAAFE16E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D489D3F-C8B4-4719-A86D-9627FFFEDB4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3996" uniqueCount="1217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4002" uniqueCount="1218">
   <si>
     <t>Début</t>
   </si>
@@ -3469,12 +3469,6 @@
     <t>21-05-2026</t>
   </si>
   <si>
-    <t>Exercice SOGEPP TRAPIL/TOTAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gennevilliers </t>
-  </si>
-  <si>
     <t>Salon SantExpo</t>
   </si>
   <si>
@@ -3674,6 +3668,15 @@
   </si>
   <si>
     <t>Renfort DPS-GE  - Concert DAMSO (J1)</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Finales CDF Handball</t>
+  </si>
+  <si>
+    <t>Finale régionale coupe de Paris</t>
+  </si>
+  <si>
+    <t>Villeparisis</t>
   </si>
 </sst>
 </file>
@@ -4028,7 +4031,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P664"/>
+  <dimension ref="A1:P665"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -24670,7 +24673,7 @@
         <v>34</v>
       </c>
       <c r="E625" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K625" t="s">
         <v>20</v>
@@ -24679,13 +24682,13 @@
         <v>21</v>
       </c>
       <c r="M625">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="N625">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O625">
-        <v>24</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="626" spans="1:15" x14ac:dyDescent="0.35">
@@ -24701,6 +24704,21 @@
       <c r="E626" t="s">
         <v>19</v>
       </c>
+      <c r="F626">
+        <v>1</v>
+      </c>
+      <c r="G626">
+        <v>0</v>
+      </c>
+      <c r="H626">
+        <v>0</v>
+      </c>
+      <c r="I626">
+        <v>0</v>
+      </c>
+      <c r="J626">
+        <v>0</v>
+      </c>
       <c r="K626" t="s">
         <v>20</v>
       </c>
@@ -24708,7 +24726,7 @@
         <v>21</v>
       </c>
       <c r="M626">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="N626">
         <v>6</v>
@@ -24725,7 +24743,7 @@
         <v>1148</v>
       </c>
       <c r="D627" t="s">
-        <v>1149</v>
+        <v>610</v>
       </c>
       <c r="E627" t="s">
         <v>19</v>
@@ -24737,21 +24755,24 @@
         <v>21</v>
       </c>
       <c r="M627">
-        <v>4.5</v>
+        <v>10</v>
       </c>
       <c r="N627">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="O627">
+        <v>40</v>
       </c>
     </row>
     <row r="628" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A628" t="s">
-        <v>1147</v>
+        <v>1149</v>
       </c>
       <c r="B628" t="s">
-        <v>1150</v>
+        <v>421</v>
       </c>
       <c r="D628" t="s">
-        <v>610</v>
+        <v>18</v>
       </c>
       <c r="E628" t="s">
         <v>19</v>
@@ -24763,56 +24784,56 @@
         <v>21</v>
       </c>
       <c r="M628">
-        <v>10</v>
+        <v>6.02</v>
       </c>
       <c r="N628">
         <v>5</v>
       </c>
       <c r="O628">
-        <v>40</v>
+        <v>30.099999904632998</v>
       </c>
     </row>
     <row r="629" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A629" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="B629" t="s">
-        <v>421</v>
+        <v>1215</v>
       </c>
       <c r="D629" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E629" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K629" t="s">
         <v>20</v>
       </c>
       <c r="L629" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M629">
-        <v>6.02</v>
+        <v>12.5</v>
       </c>
       <c r="N629">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O629">
-        <v>30.099999904632998</v>
+        <v>8</v>
       </c>
     </row>
     <row r="630" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A630" t="s">
-        <v>1152</v>
+        <v>1149</v>
       </c>
       <c r="B630" t="s">
-        <v>1107</v>
+        <v>1216</v>
       </c>
       <c r="D630" t="s">
-        <v>539</v>
+        <v>1217</v>
       </c>
       <c r="E630" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K630" t="s">
         <v>20</v>
@@ -24821,24 +24842,24 @@
         <v>21</v>
       </c>
       <c r="M630">
-        <v>11.5</v>
+        <v>3</v>
       </c>
       <c r="N630">
+        <v>4</v>
+      </c>
+      <c r="O630">
         <v>12</v>
-      </c>
-      <c r="O630">
-        <v>138</v>
       </c>
     </row>
     <row r="631" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A631" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="B631" t="s">
-        <v>1153</v>
+        <v>1107</v>
       </c>
       <c r="D631" t="s">
-        <v>55</v>
+        <v>539</v>
       </c>
       <c r="E631" t="s">
         <v>19</v>
@@ -24850,24 +24871,24 @@
         <v>21</v>
       </c>
       <c r="M631">
-        <v>5</v>
+        <v>11.5</v>
       </c>
       <c r="N631">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="O631">
-        <v>15</v>
+        <v>138</v>
       </c>
     </row>
     <row r="632" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A632" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="B632" t="s">
-        <v>1215</v>
+        <v>1151</v>
       </c>
       <c r="D632" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E632" t="s">
         <v>19</v>
@@ -24876,56 +24897,56 @@
         <v>20</v>
       </c>
       <c r="L632" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M632">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N632">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O632">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="633" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A633" t="s">
-        <v>1154</v>
+        <v>1150</v>
       </c>
       <c r="B633" t="s">
-        <v>515</v>
+        <v>1213</v>
       </c>
       <c r="D633" t="s">
-        <v>516</v>
+        <v>60</v>
       </c>
       <c r="E633" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K633" t="s">
         <v>20</v>
       </c>
       <c r="L633" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M633">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N633">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O633">
-        <v>40</v>
+        <v>11</v>
       </c>
     </row>
     <row r="634" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A634" t="s">
-        <v>1155</v>
+        <v>1152</v>
       </c>
       <c r="B634" t="s">
-        <v>1156</v>
+        <v>515</v>
       </c>
       <c r="D634" t="s">
-        <v>34</v>
+        <v>516</v>
       </c>
       <c r="E634" t="s">
         <v>19</v>
@@ -24937,24 +24958,24 @@
         <v>21</v>
       </c>
       <c r="M634">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="N634">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O634">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="635" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A635" t="s">
-        <v>1157</v>
+        <v>1153</v>
       </c>
       <c r="B635" t="s">
-        <v>1216</v>
+        <v>1154</v>
       </c>
       <c r="D635" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="E635" t="s">
         <v>19</v>
@@ -24966,27 +24987,27 @@
         <v>21</v>
       </c>
       <c r="M635">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N635">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="O635">
-        <v>63</v>
+        <v>22</v>
       </c>
     </row>
     <row r="636" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A636" t="s">
-        <v>1158</v>
+        <v>1155</v>
       </c>
       <c r="B636" t="s">
-        <v>1159</v>
+        <v>1214</v>
       </c>
       <c r="D636" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="E636" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K636" t="s">
         <v>20</v>
@@ -24995,24 +25016,24 @@
         <v>21</v>
       </c>
       <c r="M636">
-        <v>5.5</v>
+        <v>7.25</v>
       </c>
       <c r="N636">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O636">
-        <v>16.5</v>
+        <v>65.25</v>
       </c>
     </row>
     <row r="637" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A637" t="s">
-        <v>1160</v>
+        <v>1156</v>
       </c>
       <c r="B637" t="s">
-        <v>1161</v>
+        <v>1157</v>
       </c>
       <c r="D637" t="s">
-        <v>589</v>
+        <v>34</v>
       </c>
       <c r="E637" t="s">
         <v>187</v>
@@ -25024,24 +25045,24 @@
         <v>21</v>
       </c>
       <c r="M637">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N637">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O637">
-        <v>42</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="638" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A638" t="s">
-        <v>1162</v>
+        <v>1158</v>
       </c>
       <c r="B638" t="s">
-        <v>1163</v>
+        <v>1159</v>
       </c>
       <c r="D638" t="s">
-        <v>1164</v>
+        <v>589</v>
       </c>
       <c r="E638" t="s">
         <v>187</v>
@@ -25053,24 +25074,24 @@
         <v>21</v>
       </c>
       <c r="M638">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N638">
         <v>6</v>
       </c>
       <c r="O638">
-        <v>36</v>
+        <v>42</v>
       </c>
     </row>
     <row r="639" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A639" t="s">
-        <v>1165</v>
+        <v>1160</v>
       </c>
       <c r="B639" t="s">
-        <v>1166</v>
+        <v>1161</v>
       </c>
       <c r="D639" t="s">
-        <v>1167</v>
+        <v>1162</v>
       </c>
       <c r="E639" t="s">
         <v>187</v>
@@ -25079,27 +25100,27 @@
         <v>20</v>
       </c>
       <c r="L639" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M639">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N639">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O639">
-        <v>4</v>
+        <v>36</v>
       </c>
     </row>
     <row r="640" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A640" t="s">
-        <v>1168</v>
+        <v>1163</v>
       </c>
       <c r="B640" t="s">
-        <v>1169</v>
+        <v>1164</v>
       </c>
       <c r="D640" t="s">
-        <v>179</v>
+        <v>1165</v>
       </c>
       <c r="E640" t="s">
         <v>187</v>
@@ -25108,27 +25129,27 @@
         <v>20</v>
       </c>
       <c r="L640" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="M640">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N640">
         <v>2</v>
       </c>
       <c r="O640">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="641" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A641" t="s">
-        <v>1170</v>
+        <v>1166</v>
       </c>
       <c r="B641" t="s">
-        <v>1171</v>
+        <v>1167</v>
       </c>
       <c r="D641" t="s">
-        <v>1172</v>
+        <v>179</v>
       </c>
       <c r="E641" t="s">
         <v>187</v>
@@ -25137,27 +25158,27 @@
         <v>20</v>
       </c>
       <c r="L641" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M641">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N641">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O641">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="642" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A642" t="s">
-        <v>1173</v>
+        <v>1168</v>
       </c>
       <c r="B642" t="s">
-        <v>775</v>
+        <v>1169</v>
       </c>
       <c r="D642" t="s">
-        <v>1174</v>
+        <v>1170</v>
       </c>
       <c r="E642" t="s">
         <v>187</v>
@@ -25166,27 +25187,27 @@
         <v>20</v>
       </c>
       <c r="L642" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M642">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N642">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="O642">
-        <v>140</v>
+        <v>6</v>
       </c>
     </row>
     <row r="643" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A643" t="s">
-        <v>1175</v>
+        <v>1171</v>
       </c>
       <c r="B643" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D643" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="E643" t="s">
         <v>187</v>
@@ -25198,24 +25219,24 @@
         <v>50</v>
       </c>
       <c r="M643">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N643">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="O643">
-        <v>63</v>
+        <v>140</v>
       </c>
     </row>
     <row r="644" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A644" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B644" t="s">
-        <v>643</v>
+        <v>777</v>
       </c>
       <c r="D644" t="s">
-        <v>1176</v>
+        <v>1172</v>
       </c>
       <c r="E644" t="s">
         <v>187</v>
@@ -25224,24 +25245,27 @@
         <v>20</v>
       </c>
       <c r="L644" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M644">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="N644">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="O644">
+        <v>63</v>
       </c>
     </row>
     <row r="645" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
-        <v>1177</v>
+        <v>1173</v>
       </c>
       <c r="B645" t="s">
-        <v>546</v>
+        <v>643</v>
       </c>
       <c r="D645" t="s">
-        <v>34</v>
+        <v>1174</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25250,10 +25274,10 @@
         <v>20</v>
       </c>
       <c r="L645" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M645">
-        <v>6</v>
+        <v>8.25</v>
       </c>
       <c r="N645">
         <v>0</v>
@@ -25261,13 +25285,13 @@
     </row>
     <row r="646" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
-        <v>1178</v>
+        <v>1175</v>
       </c>
       <c r="B646" t="s">
-        <v>1179</v>
+        <v>546</v>
       </c>
       <c r="D646" t="s">
-        <v>205</v>
+        <v>34</v>
       </c>
       <c r="E646" t="s">
         <v>187</v>
@@ -25279,24 +25303,21 @@
         <v>21</v>
       </c>
       <c r="M646">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N646">
-        <v>4</v>
-      </c>
-      <c r="O646">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="647" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
-        <v>1180</v>
+        <v>1176</v>
       </c>
       <c r="B647" t="s">
-        <v>1181</v>
+        <v>1177</v>
       </c>
       <c r="D647" t="s">
-        <v>34</v>
+        <v>205</v>
       </c>
       <c r="E647" t="s">
         <v>187</v>
@@ -25308,24 +25329,24 @@
         <v>21</v>
       </c>
       <c r="M647">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N647">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O647">
-        <v>12</v>
+        <v>28</v>
       </c>
     </row>
     <row r="648" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A648" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B648" t="s">
-        <v>1183</v>
+        <v>1179</v>
       </c>
       <c r="D648" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E648" t="s">
         <v>187</v>
@@ -25337,21 +25358,24 @@
         <v>21</v>
       </c>
       <c r="M648">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N648">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O648">
+        <v>12</v>
       </c>
     </row>
     <row r="649" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
-        <v>1184</v>
+        <v>1180</v>
       </c>
       <c r="B649" t="s">
-        <v>1185</v>
+        <v>1181</v>
       </c>
       <c r="D649" t="s">
-        <v>1186</v>
+        <v>18</v>
       </c>
       <c r="E649" t="s">
         <v>187</v>
@@ -25360,27 +25384,24 @@
         <v>20</v>
       </c>
       <c r="L649" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M649">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N649">
-        <v>5</v>
-      </c>
-      <c r="O649">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
+        <v>1182</v>
+      </c>
+      <c r="B650" t="s">
+        <v>1183</v>
+      </c>
+      <c r="D650" t="s">
         <v>1184</v>
-      </c>
-      <c r="B650" t="s">
-        <v>1187</v>
-      </c>
-      <c r="D650" t="s">
-        <v>1186</v>
       </c>
       <c r="E650" t="s">
         <v>187</v>
@@ -25392,24 +25413,24 @@
         <v>50</v>
       </c>
       <c r="M650">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N650">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="O650">
-        <v>84</v>
+        <v>25</v>
       </c>
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1188</v>
+        <v>1182</v>
       </c>
       <c r="B651" t="s">
-        <v>1189</v>
+        <v>1185</v>
       </c>
       <c r="D651" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="E651" t="s">
         <v>187</v>
@@ -25421,24 +25442,24 @@
         <v>50</v>
       </c>
       <c r="M651">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N651">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="O651">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="B652" t="s">
-        <v>1190</v>
+        <v>1187</v>
       </c>
       <c r="D652" t="s">
-        <v>18</v>
+        <v>1184</v>
       </c>
       <c r="E652" t="s">
         <v>187</v>
@@ -25447,36 +25468,39 @@
         <v>20</v>
       </c>
       <c r="L652" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M652">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N652">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="O652">
+        <v>66</v>
       </c>
     </row>
     <row r="653" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B653" t="s">
         <v>1188</v>
       </c>
-      <c r="B653" t="s">
-        <v>1191</v>
-      </c>
       <c r="D653" t="s">
-        <v>1192</v>
+        <v>18</v>
       </c>
       <c r="E653" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K653" t="s">
         <v>20</v>
       </c>
       <c r="L653" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M653">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N653">
         <v>0</v>
@@ -25484,68 +25508,68 @@
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1193</v>
+        <v>1186</v>
       </c>
       <c r="B654" t="s">
-        <v>1194</v>
+        <v>1189</v>
       </c>
       <c r="D654" t="s">
-        <v>1186</v>
+        <v>1190</v>
       </c>
       <c r="E654" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K654" t="s">
         <v>20</v>
       </c>
       <c r="L654" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="M654">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N654">
-        <v>12</v>
-      </c>
-      <c r="O654">
-        <v>132</v>
+        <v>0</v>
       </c>
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="B655" t="s">
-        <v>1195</v>
+        <v>1192</v>
       </c>
       <c r="D655" t="s">
-        <v>1192</v>
+        <v>1184</v>
       </c>
       <c r="E655" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K655" t="s">
         <v>20</v>
       </c>
       <c r="L655" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M655">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="N655">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="O655">
+        <v>132</v>
       </c>
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1196</v>
+        <v>1191</v>
       </c>
       <c r="B656" t="s">
-        <v>1197</v>
+        <v>1193</v>
       </c>
       <c r="D656" t="s">
-        <v>1198</v>
+        <v>1190</v>
       </c>
       <c r="E656" t="s">
         <v>19</v>
@@ -25557,7 +25581,7 @@
         <v>21</v>
       </c>
       <c r="M656">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N656">
         <v>0</v>
@@ -25565,13 +25589,13 @@
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1199</v>
+        <v>1194</v>
       </c>
       <c r="B657" t="s">
-        <v>1200</v>
+        <v>1195</v>
       </c>
       <c r="D657" t="s">
-        <v>1201</v>
+        <v>1196</v>
       </c>
       <c r="E657" t="s">
         <v>19</v>
@@ -25583,7 +25607,7 @@
         <v>21</v>
       </c>
       <c r="M657">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N657">
         <v>0</v>
@@ -25591,16 +25615,16 @@
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1202</v>
+        <v>1197</v>
       </c>
       <c r="B658" t="s">
-        <v>1203</v>
+        <v>1198</v>
       </c>
       <c r="D658" t="s">
-        <v>1204</v>
+        <v>1199</v>
       </c>
       <c r="E658" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K658" t="s">
         <v>20</v>
@@ -25609,27 +25633,24 @@
         <v>21</v>
       </c>
       <c r="M658">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="N658">
-        <v>8</v>
-      </c>
-      <c r="O658">
-        <v>72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B659" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D659" t="s">
         <v>1202</v>
       </c>
-      <c r="B659" t="s">
-        <v>1205</v>
-      </c>
-      <c r="D659" t="s">
-        <v>228</v>
-      </c>
       <c r="E659" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K659" t="s">
         <v>20</v>
@@ -25638,21 +25659,24 @@
         <v>21</v>
       </c>
       <c r="M659">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="N659">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="O659">
+        <v>72</v>
       </c>
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>1206</v>
+        <v>1200</v>
       </c>
       <c r="B660" t="s">
-        <v>1207</v>
+        <v>1203</v>
       </c>
       <c r="D660" t="s">
-        <v>1208</v>
+        <v>228</v>
       </c>
       <c r="E660" t="s">
         <v>19</v>
@@ -25664,7 +25688,7 @@
         <v>21</v>
       </c>
       <c r="M660">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N660">
         <v>0</v>
@@ -25672,13 +25696,13 @@
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B661" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D661" t="s">
         <v>1206</v>
-      </c>
-      <c r="B661" t="s">
-        <v>1207</v>
-      </c>
-      <c r="D661" t="s">
-        <v>1209</v>
       </c>
       <c r="E661" t="s">
         <v>19</v>
@@ -25698,14 +25722,14 @@
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="B662" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D662" t="s">
         <v>1207</v>
       </c>
-      <c r="D662" t="s">
-        <v>1210</v>
-      </c>
       <c r="E662" t="s">
         <v>19</v>
       </c>
@@ -25716,7 +25740,7 @@
         <v>21</v>
       </c>
       <c r="M662">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="N662">
         <v>0</v>
@@ -25724,13 +25748,13 @@
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="B663" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="D663" t="s">
-        <v>1211</v>
+        <v>1208</v>
       </c>
       <c r="E663" t="s">
         <v>19</v>
@@ -25742,7 +25766,7 @@
         <v>21</v>
       </c>
       <c r="M663">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="N663">
         <v>0</v>
@@ -25750,30 +25774,56 @@
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B664" t="s">
+        <v>1205</v>
+      </c>
+      <c r="D664" t="s">
+        <v>1209</v>
+      </c>
+      <c r="E664" t="s">
+        <v>19</v>
+      </c>
+      <c r="K664" t="s">
+        <v>20</v>
+      </c>
+      <c r="L664" t="s">
+        <v>21</v>
+      </c>
+      <c r="M664">
+        <v>4</v>
+      </c>
+      <c r="N664">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="665" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A665" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B665" t="s">
+        <v>1211</v>
+      </c>
+      <c r="D665" t="s">
         <v>1212</v>
       </c>
-      <c r="B664" t="s">
-        <v>1213</v>
-      </c>
-      <c r="D664" t="s">
-        <v>1214</v>
-      </c>
-      <c r="E664" t="s">
+      <c r="E665" t="s">
         <v>187</v>
       </c>
-      <c r="K664" t="s">
-        <v>20</v>
-      </c>
-      <c r="L664" t="s">
+      <c r="K665" t="s">
+        <v>20</v>
+      </c>
+      <c r="L665" t="s">
         <v>75</v>
       </c>
-      <c r="M664">
+      <c r="M665">
         <v>120</v>
       </c>
-      <c r="N664">
+      <c r="N665">
         <v>4</v>
       </c>
-      <c r="O664">
+      <c r="O665">
         <v>480</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour DPS — 26/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD33B06-CA6F-4EC5-B50F-B8C16C26AFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B421DD9-8CDC-4EDD-9FB8-0F57A01FF657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4014" uniqueCount="1223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4032" uniqueCount="1227">
   <si>
     <t>Début</t>
   </si>
@@ -3529,15 +3529,6 @@
     <t>On sla coule 12</t>
   </si>
   <si>
-    <t>07-06-2026</t>
-  </si>
-  <si>
-    <t>[Prov] La ruée des fadas</t>
-  </si>
-  <si>
-    <t>IdF</t>
-  </si>
-  <si>
     <t>13-06-2026</t>
   </si>
   <si>
@@ -3568,9 +3559,6 @@
     <t>21-06-2026</t>
   </si>
   <si>
-    <t>[PROV] Fête de la musique</t>
-  </si>
-  <si>
     <t>26-06-2026</t>
   </si>
   <si>
@@ -3692,6 +3680,30 @@
   </si>
   <si>
     <t>25-05-2026</t>
+  </si>
+  <si>
+    <t>Fête de la musique</t>
+  </si>
+  <si>
+    <t>Place de la bastille</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Retransmission Match foot + Concert Bouss</t>
+  </si>
+  <si>
+    <t>[PROV] Retransimission Longchamps</t>
+  </si>
+  <si>
+    <t>[PROV] Fête de la victoire PSG</t>
+  </si>
+  <si>
+    <t>PdP</t>
+  </si>
+  <si>
+    <t>09-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Concert Doja Cat</t>
   </si>
 </sst>
 </file>
@@ -4046,7 +4058,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P667"/>
+  <dimension ref="A1:P670"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -24661,6 +24673,21 @@
       <c r="E624" t="s">
         <v>19</v>
       </c>
+      <c r="F624">
+        <v>0</v>
+      </c>
+      <c r="G624">
+        <v>0</v>
+      </c>
+      <c r="H624">
+        <v>0</v>
+      </c>
+      <c r="I624">
+        <v>0</v>
+      </c>
+      <c r="J624">
+        <v>0</v>
+      </c>
       <c r="K624" t="s">
         <v>20</v>
       </c>
@@ -24763,6 +24790,21 @@
       <c r="E627" t="s">
         <v>19</v>
       </c>
+      <c r="F627">
+        <v>5</v>
+      </c>
+      <c r="G627">
+        <v>1</v>
+      </c>
+      <c r="H627">
+        <v>0</v>
+      </c>
+      <c r="I627">
+        <v>0</v>
+      </c>
+      <c r="J627">
+        <v>0</v>
+      </c>
       <c r="K627" t="s">
         <v>20</v>
       </c>
@@ -24813,13 +24855,13 @@
         <v>1149</v>
       </c>
       <c r="B629" t="s">
-        <v>1215</v>
+        <v>1211</v>
       </c>
       <c r="D629" t="s">
         <v>34</v>
       </c>
       <c r="E629" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K629" t="s">
         <v>20</v>
@@ -24842,13 +24884,28 @@
         <v>1149</v>
       </c>
       <c r="B630" t="s">
-        <v>1216</v>
+        <v>1212</v>
       </c>
       <c r="D630" t="s">
-        <v>1217</v>
+        <v>1213</v>
       </c>
       <c r="E630" t="s">
         <v>19</v>
+      </c>
+      <c r="F630">
+        <v>0</v>
+      </c>
+      <c r="G630">
+        <v>0</v>
+      </c>
+      <c r="H630">
+        <v>0</v>
+      </c>
+      <c r="I630">
+        <v>0</v>
+      </c>
+      <c r="J630">
+        <v>0</v>
       </c>
       <c r="K630" t="s">
         <v>20</v>
@@ -24879,6 +24936,21 @@
       <c r="E631" t="s">
         <v>19</v>
       </c>
+      <c r="F631">
+        <v>24</v>
+      </c>
+      <c r="G631">
+        <v>1</v>
+      </c>
+      <c r="H631">
+        <v>0</v>
+      </c>
+      <c r="I631">
+        <v>2</v>
+      </c>
+      <c r="J631">
+        <v>0</v>
+      </c>
       <c r="K631" t="s">
         <v>20</v>
       </c>
@@ -24886,13 +24958,13 @@
         <v>21</v>
       </c>
       <c r="M631">
-        <v>11.5</v>
+        <v>12.4</v>
       </c>
       <c r="N631">
         <v>12</v>
       </c>
       <c r="O631">
-        <v>138</v>
+        <v>148.79999542236001</v>
       </c>
     </row>
     <row r="632" spans="1:15" x14ac:dyDescent="0.35">
@@ -24929,7 +25001,7 @@
         <v>1150</v>
       </c>
       <c r="B633" t="s">
-        <v>1213</v>
+        <v>1209</v>
       </c>
       <c r="D633" t="s">
         <v>60</v>
@@ -24955,31 +25027,46 @@
     </row>
     <row r="634" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A634" t="s">
-        <v>1222</v>
+        <v>1218</v>
       </c>
       <c r="B634" t="s">
-        <v>1221</v>
+        <v>1217</v>
       </c>
       <c r="D634" t="s">
-        <v>1220</v>
+        <v>1216</v>
       </c>
       <c r="E634" t="s">
         <v>19</v>
       </c>
+      <c r="F634">
+        <v>4</v>
+      </c>
+      <c r="G634">
+        <v>0</v>
+      </c>
+      <c r="H634">
+        <v>0</v>
+      </c>
+      <c r="I634">
+        <v>0</v>
+      </c>
+      <c r="J634">
+        <v>0</v>
+      </c>
       <c r="K634" t="s">
         <v>20</v>
       </c>
       <c r="L634" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="M634">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N634">
         <v>3</v>
       </c>
       <c r="O634">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="635" spans="1:15" x14ac:dyDescent="0.35">
@@ -25031,13 +25118,13 @@
         <v>21</v>
       </c>
       <c r="M636">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="N636">
         <v>4</v>
       </c>
       <c r="O636">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="637" spans="1:15" x14ac:dyDescent="0.35">
@@ -25045,13 +25132,13 @@
         <v>1153</v>
       </c>
       <c r="B637" t="s">
-        <v>1219</v>
+        <v>1215</v>
       </c>
       <c r="D637" t="s">
-        <v>1218</v>
+        <v>1214</v>
       </c>
       <c r="E637" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K637" t="s">
         <v>20</v>
@@ -25063,10 +25150,10 @@
         <v>2</v>
       </c>
       <c r="N637">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O637">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="638" spans="1:15" x14ac:dyDescent="0.35">
@@ -25074,7 +25161,7 @@
         <v>1155</v>
       </c>
       <c r="B638" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="D638" t="s">
         <v>60</v>
@@ -25109,7 +25196,7 @@
         <v>34</v>
       </c>
       <c r="E639" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K639" t="s">
         <v>20</v>
@@ -25121,10 +25208,10 @@
         <v>6</v>
       </c>
       <c r="N639">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O639">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="640" spans="1:15" x14ac:dyDescent="0.35">
@@ -25150,21 +25237,21 @@
         <v>7</v>
       </c>
       <c r="N640">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O640">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="641" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A641" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="B641" t="s">
-        <v>1161</v>
+        <v>1221</v>
       </c>
       <c r="D641" t="s">
-        <v>1162</v>
+        <v>34</v>
       </c>
       <c r="E641" t="s">
         <v>187</v>
@@ -25173,27 +25260,27 @@
         <v>20</v>
       </c>
       <c r="L641" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M641">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N641">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O641">
-        <v>36</v>
+        <v>8</v>
       </c>
     </row>
     <row r="642" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A642" t="s">
-        <v>1163</v>
+        <v>1158</v>
       </c>
       <c r="B642" t="s">
-        <v>1164</v>
+        <v>1222</v>
       </c>
       <c r="D642" t="s">
-        <v>1165</v>
+        <v>18</v>
       </c>
       <c r="E642" t="s">
         <v>187</v>
@@ -25202,56 +25289,56 @@
         <v>20</v>
       </c>
       <c r="L642" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="M642">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N642">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="O642">
-        <v>4</v>
+        <v>49</v>
       </c>
     </row>
     <row r="643" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A643" t="s">
-        <v>1166</v>
+        <v>1160</v>
       </c>
       <c r="B643" t="s">
-        <v>1167</v>
+        <v>1161</v>
       </c>
       <c r="D643" t="s">
-        <v>179</v>
+        <v>1162</v>
       </c>
       <c r="E643" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K643" t="s">
         <v>20</v>
       </c>
       <c r="L643" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M643">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N643">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O643">
-        <v>14</v>
+        <v>54</v>
       </c>
     </row>
     <row r="644" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A644" t="s">
-        <v>1168</v>
+        <v>1160</v>
       </c>
       <c r="B644" t="s">
-        <v>1169</v>
+        <v>1223</v>
       </c>
       <c r="D644" t="s">
-        <v>1170</v>
+        <v>1224</v>
       </c>
       <c r="E644" t="s">
         <v>187</v>
@@ -25263,24 +25350,24 @@
         <v>21</v>
       </c>
       <c r="M644">
+        <v>4</v>
+      </c>
+      <c r="N644">
         <v>6</v>
       </c>
-      <c r="N644">
-        <v>1</v>
-      </c>
       <c r="O644">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="645" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
-        <v>1171</v>
+        <v>1163</v>
       </c>
       <c r="B645" t="s">
-        <v>775</v>
+        <v>1164</v>
       </c>
       <c r="D645" t="s">
-        <v>1172</v>
+        <v>1165</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25289,27 +25376,27 @@
         <v>20</v>
       </c>
       <c r="L645" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M645">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="N645">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="O645">
-        <v>130</v>
+        <v>4</v>
       </c>
     </row>
     <row r="646" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
-        <v>1173</v>
+        <v>1166</v>
       </c>
       <c r="B646" t="s">
-        <v>777</v>
+        <v>1167</v>
       </c>
       <c r="D646" t="s">
-        <v>1172</v>
+        <v>179</v>
       </c>
       <c r="E646" t="s">
         <v>187</v>
@@ -25318,53 +25405,56 @@
         <v>20</v>
       </c>
       <c r="L646" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M646">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N646">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O646">
-        <v>63</v>
+        <v>21</v>
       </c>
     </row>
     <row r="647" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
-        <v>1173</v>
+        <v>1225</v>
       </c>
       <c r="B647" t="s">
-        <v>643</v>
+        <v>1226</v>
       </c>
       <c r="D647" t="s">
-        <v>1174</v>
+        <v>34</v>
       </c>
       <c r="E647" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K647" t="s">
         <v>20</v>
       </c>
       <c r="L647" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M647">
-        <v>8.25</v>
+        <v>6</v>
       </c>
       <c r="N647">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="O647">
+        <v>18</v>
       </c>
     </row>
     <row r="648" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A648" t="s">
-        <v>1175</v>
+        <v>1168</v>
       </c>
       <c r="B648" t="s">
-        <v>546</v>
+        <v>775</v>
       </c>
       <c r="D648" t="s">
-        <v>34</v>
+        <v>1169</v>
       </c>
       <c r="E648" t="s">
         <v>187</v>
@@ -25373,24 +25463,27 @@
         <v>20</v>
       </c>
       <c r="L648" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M648">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="N648">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="O648">
+        <v>120</v>
       </c>
     </row>
     <row r="649" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
-        <v>1176</v>
+        <v>1170</v>
       </c>
       <c r="B649" t="s">
-        <v>1177</v>
+        <v>777</v>
       </c>
       <c r="D649" t="s">
-        <v>205</v>
+        <v>1169</v>
       </c>
       <c r="E649" t="s">
         <v>187</v>
@@ -25399,27 +25492,27 @@
         <v>20</v>
       </c>
       <c r="L649" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M649">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N649">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="O649">
-        <v>28</v>
+        <v>108</v>
       </c>
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1178</v>
+        <v>1170</v>
       </c>
       <c r="B650" t="s">
-        <v>1179</v>
+        <v>643</v>
       </c>
       <c r="D650" t="s">
-        <v>34</v>
+        <v>1171</v>
       </c>
       <c r="E650" t="s">
         <v>187</v>
@@ -25428,27 +25521,24 @@
         <v>20</v>
       </c>
       <c r="L650" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M650">
-        <v>6</v>
+        <v>8.25</v>
       </c>
       <c r="N650">
-        <v>2</v>
-      </c>
-      <c r="O650">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1180</v>
+        <v>1172</v>
       </c>
       <c r="B651" t="s">
-        <v>1181</v>
+        <v>546</v>
       </c>
       <c r="D651" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E651" t="s">
         <v>187</v>
@@ -25460,21 +25550,24 @@
         <v>21</v>
       </c>
       <c r="M651">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N651">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="O651">
+        <v>6</v>
       </c>
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1182</v>
+        <v>1173</v>
       </c>
       <c r="B652" t="s">
-        <v>1183</v>
+        <v>1174</v>
       </c>
       <c r="D652" t="s">
-        <v>1184</v>
+        <v>205</v>
       </c>
       <c r="E652" t="s">
         <v>187</v>
@@ -25483,27 +25576,27 @@
         <v>20</v>
       </c>
       <c r="L652" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M652">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N652">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O652">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="653" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
-        <v>1182</v>
+        <v>1175</v>
       </c>
       <c r="B653" t="s">
-        <v>1185</v>
+        <v>1176</v>
       </c>
       <c r="D653" t="s">
-        <v>1184</v>
+        <v>34</v>
       </c>
       <c r="E653" t="s">
         <v>187</v>
@@ -25512,27 +25605,27 @@
         <v>20</v>
       </c>
       <c r="L653" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M653">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N653">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="O653">
-        <v>84</v>
+        <v>18</v>
       </c>
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1186</v>
+        <v>1177</v>
       </c>
       <c r="B654" t="s">
-        <v>1187</v>
+        <v>1219</v>
       </c>
       <c r="D654" t="s">
-        <v>1184</v>
+        <v>1220</v>
       </c>
       <c r="E654" t="s">
         <v>187</v>
@@ -25541,27 +25634,27 @@
         <v>20</v>
       </c>
       <c r="L654" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M654">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N654">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O654">
-        <v>66</v>
+        <v>40</v>
       </c>
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1186</v>
+        <v>1178</v>
       </c>
       <c r="B655" t="s">
-        <v>1188</v>
+        <v>1179</v>
       </c>
       <c r="D655" t="s">
-        <v>18</v>
+        <v>1180</v>
       </c>
       <c r="E655" t="s">
         <v>187</v>
@@ -25570,50 +25663,56 @@
         <v>20</v>
       </c>
       <c r="L655" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M655">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N655">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="O655">
+        <v>25</v>
       </c>
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1186</v>
+        <v>1178</v>
       </c>
       <c r="B656" t="s">
-        <v>1189</v>
+        <v>1181</v>
       </c>
       <c r="D656" t="s">
-        <v>1190</v>
+        <v>1180</v>
       </c>
       <c r="E656" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K656" t="s">
         <v>20</v>
       </c>
       <c r="L656" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="M656">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N656">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="O656">
+        <v>91</v>
       </c>
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1191</v>
+        <v>1182</v>
       </c>
       <c r="B657" t="s">
-        <v>1192</v>
+        <v>1183</v>
       </c>
       <c r="D657" t="s">
-        <v>1184</v>
+        <v>1180</v>
       </c>
       <c r="E657" t="s">
         <v>187</v>
@@ -25628,24 +25727,24 @@
         <v>11</v>
       </c>
       <c r="N657">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="O657">
-        <v>132</v>
+        <v>77</v>
       </c>
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1191</v>
+        <v>1182</v>
       </c>
       <c r="B658" t="s">
-        <v>1193</v>
+        <v>1184</v>
       </c>
       <c r="D658" t="s">
-        <v>1190</v>
+        <v>18</v>
       </c>
       <c r="E658" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K658" t="s">
         <v>20</v>
@@ -25654,7 +25753,7 @@
         <v>21</v>
       </c>
       <c r="M658">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N658">
         <v>0</v>
@@ -25662,13 +25761,13 @@
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1194</v>
+        <v>1182</v>
       </c>
       <c r="B659" t="s">
-        <v>1195</v>
+        <v>1185</v>
       </c>
       <c r="D659" t="s">
-        <v>1196</v>
+        <v>1186</v>
       </c>
       <c r="E659" t="s">
         <v>19</v>
@@ -25677,10 +25776,10 @@
         <v>20</v>
       </c>
       <c r="L659" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M659">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N659">
         <v>0</v>
@@ -25688,42 +25787,45 @@
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>1197</v>
+        <v>1187</v>
       </c>
       <c r="B660" t="s">
-        <v>1198</v>
+        <v>1188</v>
       </c>
       <c r="D660" t="s">
-        <v>1199</v>
+        <v>1180</v>
       </c>
       <c r="E660" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K660" t="s">
         <v>20</v>
       </c>
       <c r="L660" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M660">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N660">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="O660">
+        <v>143</v>
       </c>
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
-        <v>1200</v>
+        <v>1187</v>
       </c>
       <c r="B661" t="s">
-        <v>1201</v>
+        <v>1189</v>
       </c>
       <c r="D661" t="s">
-        <v>1202</v>
+        <v>1186</v>
       </c>
       <c r="E661" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K661" t="s">
         <v>20</v>
@@ -25732,24 +25834,21 @@
         <v>21</v>
       </c>
       <c r="M661">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N661">
-        <v>8</v>
-      </c>
-      <c r="O661">
-        <v>72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1200</v>
+        <v>1190</v>
       </c>
       <c r="B662" t="s">
-        <v>1203</v>
+        <v>1191</v>
       </c>
       <c r="D662" t="s">
-        <v>228</v>
+        <v>1192</v>
       </c>
       <c r="E662" t="s">
         <v>19</v>
@@ -25761,7 +25860,7 @@
         <v>21</v>
       </c>
       <c r="M662">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="N662">
         <v>0</v>
@@ -25769,13 +25868,13 @@
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>1204</v>
+        <v>1193</v>
       </c>
       <c r="B663" t="s">
-        <v>1205</v>
+        <v>1194</v>
       </c>
       <c r="D663" t="s">
-        <v>1206</v>
+        <v>1195</v>
       </c>
       <c r="E663" t="s">
         <v>19</v>
@@ -25795,16 +25894,16 @@
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1204</v>
+        <v>1196</v>
       </c>
       <c r="B664" t="s">
-        <v>1205</v>
+        <v>1197</v>
       </c>
       <c r="D664" t="s">
-        <v>1207</v>
+        <v>1198</v>
       </c>
       <c r="E664" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K664" t="s">
         <v>20</v>
@@ -25813,21 +25912,24 @@
         <v>21</v>
       </c>
       <c r="M664">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N664">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="O664">
+        <v>72</v>
       </c>
     </row>
     <row r="665" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A665" t="s">
-        <v>1204</v>
+        <v>1196</v>
       </c>
       <c r="B665" t="s">
-        <v>1205</v>
+        <v>1199</v>
       </c>
       <c r="D665" t="s">
-        <v>1208</v>
+        <v>228</v>
       </c>
       <c r="E665" t="s">
         <v>19</v>
@@ -25839,7 +25941,7 @@
         <v>21</v>
       </c>
       <c r="M665">
-        <v>1.5</v>
+        <v>11</v>
       </c>
       <c r="N665">
         <v>0</v>
@@ -25847,13 +25949,13 @@
     </row>
     <row r="666" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A666" t="s">
-        <v>1204</v>
+        <v>1200</v>
       </c>
       <c r="B666" t="s">
-        <v>1205</v>
+        <v>1201</v>
       </c>
       <c r="D666" t="s">
-        <v>1209</v>
+        <v>1202</v>
       </c>
       <c r="E666" t="s">
         <v>19</v>
@@ -25865,7 +25967,7 @@
         <v>21</v>
       </c>
       <c r="M666">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N666">
         <v>0</v>
@@ -25873,30 +25975,108 @@
     </row>
     <row r="667" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>1210</v>
+        <v>1200</v>
       </c>
       <c r="B667" t="s">
-        <v>1211</v>
+        <v>1201</v>
       </c>
       <c r="D667" t="s">
-        <v>1212</v>
+        <v>1203</v>
       </c>
       <c r="E667" t="s">
+        <v>19</v>
+      </c>
+      <c r="K667" t="s">
+        <v>20</v>
+      </c>
+      <c r="L667" t="s">
+        <v>21</v>
+      </c>
+      <c r="M667">
+        <v>3</v>
+      </c>
+      <c r="N667">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="668" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A668" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B668" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D668" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E668" t="s">
+        <v>19</v>
+      </c>
+      <c r="K668" t="s">
+        <v>20</v>
+      </c>
+      <c r="L668" t="s">
+        <v>21</v>
+      </c>
+      <c r="M668">
+        <v>1.5</v>
+      </c>
+      <c r="N668">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="669" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A669" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B669" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D669" t="s">
+        <v>1205</v>
+      </c>
+      <c r="E669" t="s">
+        <v>19</v>
+      </c>
+      <c r="K669" t="s">
+        <v>20</v>
+      </c>
+      <c r="L669" t="s">
+        <v>21</v>
+      </c>
+      <c r="M669">
+        <v>4</v>
+      </c>
+      <c r="N669">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="670" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A670" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B670" t="s">
+        <v>1207</v>
+      </c>
+      <c r="D670" t="s">
+        <v>1208</v>
+      </c>
+      <c r="E670" t="s">
         <v>187</v>
       </c>
-      <c r="K667" t="s">
-        <v>20</v>
-      </c>
-      <c r="L667" t="s">
+      <c r="K670" t="s">
+        <v>20</v>
+      </c>
+      <c r="L670" t="s">
         <v>75</v>
       </c>
-      <c r="M667">
+      <c r="M670">
         <v>120</v>
       </c>
-      <c r="N667">
+      <c r="N670">
         <v>4</v>
       </c>
-      <c r="O667">
+      <c r="O670">
         <v>480</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour DPS — 28/05/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B421DD9-8CDC-4EDD-9FB8-0F57A01FF657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B3CAC8-E435-48E4-9F02-4257D8AF8BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4032" uniqueCount="1227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4062" uniqueCount="1230">
   <si>
     <t>Début</t>
   </si>
@@ -3694,16 +3694,25 @@
     <t>[PROV] Retransimission Longchamps</t>
   </si>
   <si>
-    <t>[PROV] Fête de la victoire PSG</t>
-  </si>
-  <si>
-    <t>PdP</t>
-  </si>
-  <si>
     <t>09-06-2026</t>
   </si>
   <si>
     <t>Renfort DPS-ME - Concert Doja Cat</t>
+  </si>
+  <si>
+    <t>Renfort Canicule  Tour Eiffel</t>
+  </si>
+  <si>
+    <t>Renfort Présentation Trophéé LDC</t>
+  </si>
+  <si>
+    <t>05-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort Banquet des vins de Loire</t>
+  </si>
+  <si>
+    <t>Fête de la Musique Spotify</t>
   </si>
 </sst>
 </file>
@@ -4058,7 +4067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P670"/>
+  <dimension ref="A1:P675"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -24834,6 +24843,21 @@
       <c r="E628" t="s">
         <v>19</v>
       </c>
+      <c r="F628">
+        <v>10</v>
+      </c>
+      <c r="G628">
+        <v>1</v>
+      </c>
+      <c r="H628">
+        <v>0</v>
+      </c>
+      <c r="I628">
+        <v>0</v>
+      </c>
+      <c r="J628">
+        <v>10</v>
+      </c>
       <c r="K628" t="s">
         <v>20</v>
       </c>
@@ -25082,6 +25106,21 @@
       <c r="E635" t="s">
         <v>19</v>
       </c>
+      <c r="F635">
+        <v>2</v>
+      </c>
+      <c r="G635">
+        <v>0</v>
+      </c>
+      <c r="H635">
+        <v>0</v>
+      </c>
+      <c r="I635">
+        <v>0</v>
+      </c>
+      <c r="J635">
+        <v>0</v>
+      </c>
       <c r="K635" t="s">
         <v>20</v>
       </c>
@@ -25140,6 +25179,21 @@
       <c r="E637" t="s">
         <v>19</v>
       </c>
+      <c r="F637">
+        <v>0</v>
+      </c>
+      <c r="G637">
+        <v>0</v>
+      </c>
+      <c r="H637">
+        <v>0</v>
+      </c>
+      <c r="I637">
+        <v>0</v>
+      </c>
+      <c r="J637">
+        <v>0</v>
+      </c>
       <c r="K637" t="s">
         <v>20</v>
       </c>
@@ -25158,13 +25212,13 @@
     </row>
     <row r="638" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A638" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="B638" t="s">
-        <v>1210</v>
+        <v>1225</v>
       </c>
       <c r="D638" t="s">
-        <v>60</v>
+        <v>1216</v>
       </c>
       <c r="E638" t="s">
         <v>19</v>
@@ -25173,27 +25227,27 @@
         <v>20</v>
       </c>
       <c r="L638" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M638">
-        <v>7.25</v>
+        <v>12.5</v>
       </c>
       <c r="N638">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O638">
-        <v>65.25</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="639" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A639" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B639" t="s">
-        <v>1157</v>
+        <v>1210</v>
       </c>
       <c r="D639" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="E639" t="s">
         <v>19</v>
@@ -25205,27 +25259,27 @@
         <v>21</v>
       </c>
       <c r="M639">
-        <v>6</v>
+        <v>7.25</v>
       </c>
       <c r="N639">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="O639">
-        <v>24</v>
+        <v>65.25</v>
       </c>
     </row>
     <row r="640" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A640" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
       <c r="B640" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="D640" t="s">
-        <v>589</v>
+        <v>34</v>
       </c>
       <c r="E640" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K640" t="s">
         <v>20</v>
@@ -25234,13 +25288,13 @@
         <v>21</v>
       </c>
       <c r="M640">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N640">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O640">
-        <v>49</v>
+        <v>22</v>
       </c>
     </row>
     <row r="641" spans="1:15" x14ac:dyDescent="0.35">
@@ -25248,28 +25302,28 @@
         <v>1158</v>
       </c>
       <c r="B641" t="s">
-        <v>1221</v>
+        <v>1159</v>
       </c>
       <c r="D641" t="s">
-        <v>34</v>
+        <v>589</v>
       </c>
       <c r="E641" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K641" t="s">
         <v>20</v>
       </c>
       <c r="L641" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M641">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N641">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="O641">
-        <v>8</v>
+        <v>42</v>
       </c>
     </row>
     <row r="642" spans="1:15" x14ac:dyDescent="0.35">
@@ -25277,10 +25331,10 @@
         <v>1158</v>
       </c>
       <c r="B642" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="D642" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E642" t="s">
         <v>187</v>
@@ -25289,45 +25343,45 @@
         <v>20</v>
       </c>
       <c r="L642" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="M642">
         <v>7</v>
       </c>
       <c r="N642">
+        <v>1</v>
+      </c>
+      <c r="O642">
         <v>7</v>
-      </c>
-      <c r="O642">
-        <v>49</v>
       </c>
     </row>
     <row r="643" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A643" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="B643" t="s">
-        <v>1161</v>
+        <v>1222</v>
       </c>
       <c r="D643" t="s">
-        <v>1162</v>
+        <v>18</v>
       </c>
       <c r="E643" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K643" t="s">
         <v>20</v>
       </c>
       <c r="L643" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M643">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N643">
         <v>9</v>
       </c>
       <c r="O643">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="644" spans="1:15" x14ac:dyDescent="0.35">
@@ -25335,13 +25389,13 @@
         <v>1160</v>
       </c>
       <c r="B644" t="s">
-        <v>1223</v>
+        <v>1161</v>
       </c>
       <c r="D644" t="s">
-        <v>1224</v>
+        <v>1162</v>
       </c>
       <c r="E644" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K644" t="s">
         <v>20</v>
@@ -25350,24 +25404,24 @@
         <v>21</v>
       </c>
       <c r="M644">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N644">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O644">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="645" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
-        <v>1163</v>
+        <v>1160</v>
       </c>
       <c r="B645" t="s">
-        <v>1164</v>
+        <v>1226</v>
       </c>
       <c r="D645" t="s">
-        <v>1165</v>
+        <v>55</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25376,27 +25430,27 @@
         <v>20</v>
       </c>
       <c r="L645" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M645">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="N645">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O645">
-        <v>4</v>
+        <v>27</v>
       </c>
     </row>
     <row r="646" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
-        <v>1166</v>
+        <v>1163</v>
       </c>
       <c r="B646" t="s">
-        <v>1167</v>
+        <v>1164</v>
       </c>
       <c r="D646" t="s">
-        <v>179</v>
+        <v>1165</v>
       </c>
       <c r="E646" t="s">
         <v>187</v>
@@ -25408,27 +25462,27 @@
         <v>25</v>
       </c>
       <c r="M646">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N646">
         <v>3</v>
       </c>
       <c r="O646">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="647" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
-        <v>1225</v>
+        <v>1227</v>
       </c>
       <c r="B647" t="s">
-        <v>1226</v>
+        <v>397</v>
       </c>
       <c r="D647" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="E647" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K647" t="s">
         <v>20</v>
@@ -25437,24 +25491,24 @@
         <v>21</v>
       </c>
       <c r="M647">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N647">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O647">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="648" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A648" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="B648" t="s">
-        <v>775</v>
+        <v>1167</v>
       </c>
       <c r="D648" t="s">
-        <v>1169</v>
+        <v>179</v>
       </c>
       <c r="E648" t="s">
         <v>187</v>
@@ -25463,56 +25517,56 @@
         <v>20</v>
       </c>
       <c r="L648" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M648">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N648">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="O648">
-        <v>120</v>
+        <v>21</v>
       </c>
     </row>
     <row r="649" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
-        <v>1170</v>
+        <v>1223</v>
       </c>
       <c r="B649" t="s">
-        <v>777</v>
+        <v>1224</v>
       </c>
       <c r="D649" t="s">
-        <v>1169</v>
+        <v>34</v>
       </c>
       <c r="E649" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K649" t="s">
         <v>20</v>
       </c>
       <c r="L649" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M649">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N649">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="O649">
-        <v>108</v>
+        <v>18</v>
       </c>
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="B650" t="s">
-        <v>643</v>
+        <v>775</v>
       </c>
       <c r="D650" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="E650" t="s">
         <v>187</v>
@@ -25521,53 +25575,53 @@
         <v>20</v>
       </c>
       <c r="L650" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M650">
-        <v>8.25</v>
+        <v>10</v>
       </c>
       <c r="N650">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="O650">
+        <v>130</v>
       </c>
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1172</v>
+        <v>1168</v>
       </c>
       <c r="B651" t="s">
-        <v>546</v>
+        <v>1228</v>
       </c>
       <c r="D651" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="E651" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K651" t="s">
         <v>20</v>
       </c>
       <c r="L651" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M651">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N651">
-        <v>1</v>
-      </c>
-      <c r="O651">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="B652" t="s">
-        <v>1174</v>
+        <v>777</v>
       </c>
       <c r="D652" t="s">
-        <v>205</v>
+        <v>1169</v>
       </c>
       <c r="E652" t="s">
         <v>187</v>
@@ -25576,27 +25630,27 @@
         <v>20</v>
       </c>
       <c r="L652" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M652">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N652">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="O652">
-        <v>28</v>
+        <v>108</v>
       </c>
     </row>
     <row r="653" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
-        <v>1175</v>
+        <v>1170</v>
       </c>
       <c r="B653" t="s">
-        <v>1176</v>
+        <v>643</v>
       </c>
       <c r="D653" t="s">
-        <v>34</v>
+        <v>1171</v>
       </c>
       <c r="E653" t="s">
         <v>187</v>
@@ -25605,56 +25659,50 @@
         <v>20</v>
       </c>
       <c r="L653" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M653">
-        <v>6</v>
+        <v>8.25</v>
       </c>
       <c r="N653">
-        <v>3</v>
-      </c>
-      <c r="O653">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1177</v>
+        <v>1170</v>
       </c>
       <c r="B654" t="s">
-        <v>1219</v>
+        <v>1228</v>
       </c>
       <c r="D654" t="s">
-        <v>1220</v>
+        <v>18</v>
       </c>
       <c r="E654" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K654" t="s">
         <v>20</v>
       </c>
       <c r="L654" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M654">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N654">
-        <v>5</v>
-      </c>
-      <c r="O654">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1178</v>
+        <v>1172</v>
       </c>
       <c r="B655" t="s">
-        <v>1179</v>
+        <v>546</v>
       </c>
       <c r="D655" t="s">
-        <v>1180</v>
+        <v>34</v>
       </c>
       <c r="E655" t="s">
         <v>187</v>
@@ -25663,27 +25711,27 @@
         <v>20</v>
       </c>
       <c r="L655" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M655">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N655">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O655">
-        <v>25</v>
+        <v>6</v>
       </c>
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1178</v>
+        <v>1173</v>
       </c>
       <c r="B656" t="s">
-        <v>1181</v>
+        <v>1174</v>
       </c>
       <c r="D656" t="s">
-        <v>1180</v>
+        <v>205</v>
       </c>
       <c r="E656" t="s">
         <v>187</v>
@@ -25692,27 +25740,27 @@
         <v>20</v>
       </c>
       <c r="L656" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M656">
         <v>7</v>
       </c>
       <c r="N656">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="O656">
-        <v>91</v>
+        <v>28</v>
       </c>
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1182</v>
+        <v>1175</v>
       </c>
       <c r="B657" t="s">
-        <v>1183</v>
+        <v>1176</v>
       </c>
       <c r="D657" t="s">
-        <v>1180</v>
+        <v>34</v>
       </c>
       <c r="E657" t="s">
         <v>187</v>
@@ -25721,27 +25769,27 @@
         <v>20</v>
       </c>
       <c r="L657" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M657">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="N657">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O657">
-        <v>77</v>
+        <v>18</v>
       </c>
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
       <c r="B658" t="s">
-        <v>1184</v>
+        <v>1219</v>
       </c>
       <c r="D658" t="s">
-        <v>18</v>
+        <v>1220</v>
       </c>
       <c r="E658" t="s">
         <v>187</v>
@@ -25756,30 +25804,33 @@
         <v>8</v>
       </c>
       <c r="N658">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="O658">
+        <v>48</v>
       </c>
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
       <c r="B659" t="s">
-        <v>1185</v>
+        <v>1229</v>
       </c>
       <c r="D659" t="s">
-        <v>1186</v>
+        <v>202</v>
       </c>
       <c r="E659" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K659" t="s">
         <v>20</v>
       </c>
       <c r="L659" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M659">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N659">
         <v>0</v>
@@ -25787,10 +25838,10 @@
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>1187</v>
+        <v>1178</v>
       </c>
       <c r="B660" t="s">
-        <v>1188</v>
+        <v>1179</v>
       </c>
       <c r="D660" t="s">
         <v>1180</v>
@@ -25805,79 +25856,85 @@
         <v>50</v>
       </c>
       <c r="M660">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="N660">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="O660">
-        <v>143</v>
+        <v>30</v>
       </c>
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
-        <v>1187</v>
+        <v>1178</v>
       </c>
       <c r="B661" t="s">
-        <v>1189</v>
+        <v>1181</v>
       </c>
       <c r="D661" t="s">
-        <v>1186</v>
+        <v>1180</v>
       </c>
       <c r="E661" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K661" t="s">
         <v>20</v>
       </c>
       <c r="L661" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M661">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N661">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="O661">
+        <v>98</v>
       </c>
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1190</v>
+        <v>1182</v>
       </c>
       <c r="B662" t="s">
-        <v>1191</v>
+        <v>1183</v>
       </c>
       <c r="D662" t="s">
-        <v>1192</v>
+        <v>1180</v>
       </c>
       <c r="E662" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K662" t="s">
         <v>20</v>
       </c>
       <c r="L662" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M662">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N662">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="O662">
+        <v>99</v>
       </c>
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>1193</v>
+        <v>1182</v>
       </c>
       <c r="B663" t="s">
-        <v>1194</v>
+        <v>1184</v>
       </c>
       <c r="D663" t="s">
-        <v>1195</v>
+        <v>18</v>
       </c>
       <c r="E663" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K663" t="s">
         <v>20</v>
@@ -25886,7 +25943,7 @@
         <v>21</v>
       </c>
       <c r="M663">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N663">
         <v>0</v>
@@ -25894,68 +25951,68 @@
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1196</v>
+        <v>1182</v>
       </c>
       <c r="B664" t="s">
-        <v>1197</v>
+        <v>1185</v>
       </c>
       <c r="D664" t="s">
-        <v>1198</v>
+        <v>1186</v>
       </c>
       <c r="E664" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K664" t="s">
         <v>20</v>
       </c>
       <c r="L664" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M664">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N664">
-        <v>8</v>
-      </c>
-      <c r="O664">
-        <v>72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="665" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A665" t="s">
-        <v>1196</v>
+        <v>1187</v>
       </c>
       <c r="B665" t="s">
-        <v>1199</v>
+        <v>1188</v>
       </c>
       <c r="D665" t="s">
-        <v>228</v>
+        <v>1180</v>
       </c>
       <c r="E665" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K665" t="s">
         <v>20</v>
       </c>
       <c r="L665" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M665">
         <v>11</v>
       </c>
       <c r="N665">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="O665">
+        <v>143</v>
       </c>
     </row>
     <row r="666" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A666" t="s">
-        <v>1200</v>
+        <v>1187</v>
       </c>
       <c r="B666" t="s">
-        <v>1201</v>
+        <v>1189</v>
       </c>
       <c r="D666" t="s">
-        <v>1202</v>
+        <v>1186</v>
       </c>
       <c r="E666" t="s">
         <v>19</v>
@@ -25967,7 +26024,7 @@
         <v>21</v>
       </c>
       <c r="M666">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N666">
         <v>0</v>
@@ -25975,13 +26032,13 @@
     </row>
     <row r="667" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>1200</v>
+        <v>1190</v>
       </c>
       <c r="B667" t="s">
-        <v>1201</v>
+        <v>1191</v>
       </c>
       <c r="D667" t="s">
-        <v>1203</v>
+        <v>1192</v>
       </c>
       <c r="E667" t="s">
         <v>19</v>
@@ -25993,7 +26050,7 @@
         <v>21</v>
       </c>
       <c r="M667">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N667">
         <v>0</v>
@@ -26001,13 +26058,13 @@
     </row>
     <row r="668" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A668" t="s">
-        <v>1200</v>
+        <v>1193</v>
       </c>
       <c r="B668" t="s">
-        <v>1201</v>
+        <v>1194</v>
       </c>
       <c r="D668" t="s">
-        <v>1204</v>
+        <v>1195</v>
       </c>
       <c r="E668" t="s">
         <v>19</v>
@@ -26019,7 +26076,7 @@
         <v>21</v>
       </c>
       <c r="M668">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="N668">
         <v>0</v>
@@ -26027,16 +26084,16 @@
     </row>
     <row r="669" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A669" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="B669" t="s">
-        <v>1201</v>
+        <v>1197</v>
       </c>
       <c r="D669" t="s">
-        <v>1205</v>
+        <v>1198</v>
       </c>
       <c r="E669" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K669" t="s">
         <v>20</v>
@@ -26045,39 +26102,172 @@
         <v>21</v>
       </c>
       <c r="M669">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="N669">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="O669">
+        <v>81</v>
       </c>
     </row>
     <row r="670" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A670" t="s">
+        <v>1196</v>
+      </c>
+      <c r="B670" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D670" t="s">
+        <v>228</v>
+      </c>
+      <c r="E670" t="s">
+        <v>19</v>
+      </c>
+      <c r="K670" t="s">
+        <v>20</v>
+      </c>
+      <c r="L670" t="s">
+        <v>21</v>
+      </c>
+      <c r="M670">
+        <v>11</v>
+      </c>
+      <c r="N670">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A671" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B671" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D671" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E671" t="s">
+        <v>19</v>
+      </c>
+      <c r="K671" t="s">
+        <v>20</v>
+      </c>
+      <c r="L671" t="s">
+        <v>21</v>
+      </c>
+      <c r="M671">
+        <v>3</v>
+      </c>
+      <c r="N671">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="672" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A672" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B672" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D672" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E672" t="s">
+        <v>19</v>
+      </c>
+      <c r="K672" t="s">
+        <v>20</v>
+      </c>
+      <c r="L672" t="s">
+        <v>21</v>
+      </c>
+      <c r="M672">
+        <v>3</v>
+      </c>
+      <c r="N672">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A673" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B673" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D673" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E673" t="s">
+        <v>19</v>
+      </c>
+      <c r="K673" t="s">
+        <v>20</v>
+      </c>
+      <c r="L673" t="s">
+        <v>21</v>
+      </c>
+      <c r="M673">
+        <v>1.5</v>
+      </c>
+      <c r="N673">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A674" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B674" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D674" t="s">
+        <v>1205</v>
+      </c>
+      <c r="E674" t="s">
+        <v>19</v>
+      </c>
+      <c r="K674" t="s">
+        <v>20</v>
+      </c>
+      <c r="L674" t="s">
+        <v>21</v>
+      </c>
+      <c r="M674">
+        <v>4</v>
+      </c>
+      <c r="N674">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="675" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A675" t="s">
         <v>1206</v>
       </c>
-      <c r="B670" t="s">
+      <c r="B675" t="s">
         <v>1207</v>
       </c>
-      <c r="D670" t="s">
+      <c r="D675" t="s">
         <v>1208</v>
       </c>
-      <c r="E670" t="s">
+      <c r="E675" t="s">
         <v>187</v>
       </c>
-      <c r="K670" t="s">
-        <v>20</v>
-      </c>
-      <c r="L670" t="s">
+      <c r="K675" t="s">
+        <v>20</v>
+      </c>
+      <c r="L675" t="s">
         <v>75</v>
       </c>
-      <c r="M670">
+      <c r="M675">
         <v>120</v>
       </c>
-      <c r="N670">
-        <v>4</v>
-      </c>
-      <c r="O670">
-        <v>480</v>
+      <c r="N675">
+        <v>6</v>
+      </c>
+      <c r="O675">
+        <v>720</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mise à jour DPS — 01/06/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B3CAC8-E435-48E4-9F02-4257D8AF8BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC90CB3-78E6-40B4-88BF-94EFD391CAAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4062" uniqueCount="1230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4080" uniqueCount="1237">
   <si>
     <t>Début</t>
   </si>
@@ -3691,9 +3691,6 @@
     <t>Renfort DPS-ME - Retransmission Match foot + Concert Bouss</t>
   </si>
   <si>
-    <t>[PROV] Retransimission Longchamps</t>
-  </si>
-  <si>
     <t>09-06-2026</t>
   </si>
   <si>
@@ -3713,6 +3710,30 @@
   </si>
   <si>
     <t>Fête de la Musique Spotify</t>
+  </si>
+  <si>
+    <t>Renfort Fan Zone Finale Ligue des Champions</t>
+  </si>
+  <si>
+    <t>Hippodrome de Longchamps</t>
+  </si>
+  <si>
+    <t>Renfort Recensement VPS Finale LDC</t>
+  </si>
+  <si>
+    <t>Renfort DPS Champs-Elysées Finale LDC</t>
+  </si>
+  <si>
+    <t>Champs - Elysées</t>
+  </si>
+  <si>
+    <t>Renfort PlayOff - Demi Finale - Match 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fête la musique Playground </t>
+  </si>
+  <si>
+    <t>Rue du Général Renault (P</t>
   </si>
 </sst>
 </file>
@@ -4067,7 +4088,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P675"/>
+  <dimension ref="A1:P678"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -25215,7 +25236,7 @@
         <v>1153</v>
       </c>
       <c r="B638" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="D638" t="s">
         <v>1216</v>
@@ -25259,13 +25280,13 @@
         <v>21</v>
       </c>
       <c r="M639">
-        <v>7.25</v>
+        <v>7</v>
       </c>
       <c r="N639">
         <v>9</v>
       </c>
       <c r="O639">
-        <v>65.25</v>
+        <v>61</v>
       </c>
     </row>
     <row r="640" spans="1:15" x14ac:dyDescent="0.35">
@@ -25310,6 +25331,21 @@
       <c r="E641" t="s">
         <v>19</v>
       </c>
+      <c r="F641">
+        <v>1</v>
+      </c>
+      <c r="G641">
+        <v>0</v>
+      </c>
+      <c r="H641">
+        <v>0</v>
+      </c>
+      <c r="I641">
+        <v>0</v>
+      </c>
+      <c r="J641">
+        <v>0</v>
+      </c>
       <c r="K641" t="s">
         <v>20</v>
       </c>
@@ -25337,7 +25373,7 @@
         <v>34</v>
       </c>
       <c r="E642" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K642" t="s">
         <v>20</v>
@@ -25346,13 +25382,13 @@
         <v>25</v>
       </c>
       <c r="M642">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N642">
         <v>1</v>
       </c>
       <c r="O642">
-        <v>7</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="643" spans="1:15" x14ac:dyDescent="0.35">
@@ -25360,39 +25396,39 @@
         <v>1158</v>
       </c>
       <c r="B643" t="s">
-        <v>1222</v>
+        <v>1229</v>
       </c>
       <c r="D643" t="s">
-        <v>18</v>
+        <v>1230</v>
       </c>
       <c r="E643" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K643" t="s">
         <v>20</v>
       </c>
       <c r="L643" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M643">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N643">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O643">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="644" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A644" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="B644" t="s">
-        <v>1161</v>
+        <v>1231</v>
       </c>
       <c r="D644" t="s">
-        <v>1162</v>
+        <v>18</v>
       </c>
       <c r="E644" t="s">
         <v>19</v>
@@ -25404,24 +25440,24 @@
         <v>21</v>
       </c>
       <c r="M644">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="N644">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="O644">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="645" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="B645" t="s">
-        <v>1226</v>
+        <v>1232</v>
       </c>
       <c r="D645" t="s">
-        <v>55</v>
+        <v>1233</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25433,56 +25469,71 @@
         <v>21</v>
       </c>
       <c r="M645">
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="N645">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O645">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="646" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
-        <v>1163</v>
+        <v>1160</v>
       </c>
       <c r="B646" t="s">
-        <v>1164</v>
+        <v>1161</v>
       </c>
       <c r="D646" t="s">
-        <v>1165</v>
+        <v>1162</v>
       </c>
       <c r="E646" t="s">
-        <v>187</v>
+        <v>19</v>
+      </c>
+      <c r="F646">
+        <v>7</v>
+      </c>
+      <c r="G646">
+        <v>0</v>
+      </c>
+      <c r="H646">
+        <v>0</v>
+      </c>
+      <c r="I646">
+        <v>0</v>
+      </c>
+      <c r="J646">
+        <v>0</v>
       </c>
       <c r="K646" t="s">
         <v>20</v>
       </c>
       <c r="L646" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M646">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N646">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O646">
-        <v>6</v>
+        <v>54</v>
       </c>
     </row>
     <row r="647" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
-        <v>1227</v>
+        <v>1160</v>
       </c>
       <c r="B647" t="s">
-        <v>397</v>
+        <v>1225</v>
       </c>
       <c r="D647" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="E647" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K647" t="s">
         <v>20</v>
@@ -25491,27 +25542,27 @@
         <v>21</v>
       </c>
       <c r="M647">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="N647">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O647">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="648" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A648" t="s">
-        <v>1166</v>
+        <v>1163</v>
       </c>
       <c r="B648" t="s">
-        <v>1167</v>
+        <v>1164</v>
       </c>
       <c r="D648" t="s">
-        <v>179</v>
+        <v>1165</v>
       </c>
       <c r="E648" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K648" t="s">
         <v>20</v>
@@ -25520,53 +25571,50 @@
         <v>25</v>
       </c>
       <c r="M648">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N648">
         <v>3</v>
       </c>
       <c r="O648">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="649" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
-        <v>1223</v>
+        <v>1163</v>
       </c>
       <c r="B649" t="s">
-        <v>1224</v>
+        <v>1234</v>
       </c>
       <c r="D649" t="s">
-        <v>34</v>
+        <v>362</v>
       </c>
       <c r="E649" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K649" t="s">
         <v>20</v>
       </c>
       <c r="L649" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M649">
-        <v>6</v>
+        <v>4.75</v>
       </c>
       <c r="N649">
-        <v>3</v>
-      </c>
-      <c r="O649">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1168</v>
+        <v>1226</v>
       </c>
       <c r="B650" t="s">
-        <v>775</v>
+        <v>397</v>
       </c>
       <c r="D650" t="s">
-        <v>1169</v>
+        <v>18</v>
       </c>
       <c r="E650" t="s">
         <v>187</v>
@@ -25575,82 +25623,85 @@
         <v>20</v>
       </c>
       <c r="L650" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M650">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N650">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="O650">
-        <v>130</v>
+        <v>28</v>
       </c>
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="B651" t="s">
-        <v>1228</v>
+        <v>1167</v>
       </c>
       <c r="D651" t="s">
-        <v>18</v>
+        <v>179</v>
       </c>
       <c r="E651" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K651" t="s">
         <v>20</v>
       </c>
       <c r="L651" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="M651">
+        <v>7</v>
+      </c>
+      <c r="N651">
         <v>5</v>
       </c>
-      <c r="N651">
-        <v>0</v>
+      <c r="O651">
+        <v>35</v>
       </c>
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1170</v>
+        <v>1222</v>
       </c>
       <c r="B652" t="s">
-        <v>777</v>
+        <v>1223</v>
       </c>
       <c r="D652" t="s">
-        <v>1169</v>
+        <v>34</v>
       </c>
       <c r="E652" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K652" t="s">
         <v>20</v>
       </c>
       <c r="L652" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M652">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N652">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="O652">
-        <v>108</v>
+        <v>18</v>
       </c>
     </row>
     <row r="653" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="B653" t="s">
-        <v>643</v>
+        <v>775</v>
       </c>
       <c r="D653" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="E653" t="s">
         <v>187</v>
@@ -25659,13 +25710,16 @@
         <v>20</v>
       </c>
       <c r="L653" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M653">
-        <v>8.25</v>
+        <v>10</v>
       </c>
       <c r="N653">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="O653">
+        <v>140</v>
       </c>
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
@@ -25673,36 +25727,39 @@
         <v>1170</v>
       </c>
       <c r="B654" t="s">
-        <v>1228</v>
+        <v>777</v>
       </c>
       <c r="D654" t="s">
-        <v>18</v>
+        <v>1169</v>
       </c>
       <c r="E654" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K654" t="s">
         <v>20</v>
       </c>
       <c r="L654" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="M654">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N654">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="O654">
+        <v>117</v>
       </c>
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="B655" t="s">
-        <v>546</v>
+        <v>643</v>
       </c>
       <c r="D655" t="s">
-        <v>34</v>
+        <v>1171</v>
       </c>
       <c r="E655" t="s">
         <v>187</v>
@@ -25711,53 +25768,47 @@
         <v>20</v>
       </c>
       <c r="L655" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M655">
-        <v>6</v>
+        <v>8.25</v>
       </c>
       <c r="N655">
-        <v>1</v>
-      </c>
-      <c r="O655">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="B656" t="s">
-        <v>1174</v>
+        <v>1227</v>
       </c>
       <c r="D656" t="s">
-        <v>205</v>
+        <v>18</v>
       </c>
       <c r="E656" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K656" t="s">
         <v>20</v>
       </c>
       <c r="L656" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M656">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N656">
-        <v>4</v>
-      </c>
-      <c r="O656">
-        <v>28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1175</v>
+        <v>1172</v>
       </c>
       <c r="B657" t="s">
-        <v>1176</v>
+        <v>546</v>
       </c>
       <c r="D657" t="s">
         <v>34</v>
@@ -25775,21 +25826,21 @@
         <v>6</v>
       </c>
       <c r="N657">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O657">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1177</v>
+        <v>1173</v>
       </c>
       <c r="B658" t="s">
-        <v>1219</v>
+        <v>1174</v>
       </c>
       <c r="D658" t="s">
-        <v>1220</v>
+        <v>205</v>
       </c>
       <c r="E658" t="s">
         <v>187</v>
@@ -25801,24 +25852,24 @@
         <v>21</v>
       </c>
       <c r="M658">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N658">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O658">
-        <v>48</v>
+        <v>28</v>
       </c>
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="B659" t="s">
-        <v>1229</v>
+        <v>1176</v>
       </c>
       <c r="D659" t="s">
-        <v>202</v>
+        <v>34</v>
       </c>
       <c r="E659" t="s">
         <v>187</v>
@@ -25830,21 +25881,24 @@
         <v>21</v>
       </c>
       <c r="M659">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N659">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="O659">
+        <v>18</v>
       </c>
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B660" t="s">
-        <v>1179</v>
+        <v>1219</v>
       </c>
       <c r="D660" t="s">
-        <v>1180</v>
+        <v>1220</v>
       </c>
       <c r="E660" t="s">
         <v>187</v>
@@ -25853,27 +25907,27 @@
         <v>20</v>
       </c>
       <c r="L660" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M660">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N660">
         <v>6</v>
       </c>
       <c r="O660">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B661" t="s">
-        <v>1181</v>
+        <v>1228</v>
       </c>
       <c r="D661" t="s">
-        <v>1180</v>
+        <v>202</v>
       </c>
       <c r="E661" t="s">
         <v>187</v>
@@ -25882,27 +25936,27 @@
         <v>20</v>
       </c>
       <c r="L661" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M661">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N661">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="O661">
-        <v>98</v>
+        <v>8</v>
       </c>
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
       <c r="B662" t="s">
-        <v>1183</v>
+        <v>1235</v>
       </c>
       <c r="D662" t="s">
-        <v>1180</v>
+        <v>1236</v>
       </c>
       <c r="E662" t="s">
         <v>187</v>
@@ -25911,27 +25965,24 @@
         <v>20</v>
       </c>
       <c r="L662" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M662">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="N662">
-        <v>9</v>
-      </c>
-      <c r="O662">
-        <v>99</v>
+        <v>0</v>
       </c>
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B663" t="s">
-        <v>1184</v>
+        <v>1179</v>
       </c>
       <c r="D663" t="s">
-        <v>18</v>
+        <v>1180</v>
       </c>
       <c r="E663" t="s">
         <v>187</v>
@@ -25940,47 +25991,53 @@
         <v>20</v>
       </c>
       <c r="L663" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M663">
+        <v>5</v>
+      </c>
+      <c r="N663">
         <v>8</v>
       </c>
-      <c r="N663">
-        <v>0</v>
+      <c r="O663">
+        <v>40</v>
       </c>
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B664" t="s">
-        <v>1185</v>
+        <v>1181</v>
       </c>
       <c r="D664" t="s">
-        <v>1186</v>
+        <v>1180</v>
       </c>
       <c r="E664" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K664" t="s">
         <v>20</v>
       </c>
       <c r="L664" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="M664">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N664">
-        <v>0</v>
+        <v>17</v>
+      </c>
+      <c r="O664">
+        <v>119</v>
       </c>
     </row>
     <row r="665" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A665" t="s">
-        <v>1187</v>
+        <v>1182</v>
       </c>
       <c r="B665" t="s">
-        <v>1188</v>
+        <v>1183</v>
       </c>
       <c r="D665" t="s">
         <v>1180</v>
@@ -25998,24 +26055,24 @@
         <v>11</v>
       </c>
       <c r="N665">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="O665">
-        <v>143</v>
+        <v>121</v>
       </c>
     </row>
     <row r="666" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A666" t="s">
-        <v>1187</v>
+        <v>1182</v>
       </c>
       <c r="B666" t="s">
-        <v>1189</v>
+        <v>1184</v>
       </c>
       <c r="D666" t="s">
-        <v>1186</v>
+        <v>18</v>
       </c>
       <c r="E666" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K666" t="s">
         <v>20</v>
@@ -26024,7 +26081,7 @@
         <v>21</v>
       </c>
       <c r="M666">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N666">
         <v>0</v>
@@ -26032,13 +26089,13 @@
     </row>
     <row r="667" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>1190</v>
+        <v>1182</v>
       </c>
       <c r="B667" t="s">
-        <v>1191</v>
+        <v>1185</v>
       </c>
       <c r="D667" t="s">
-        <v>1192</v>
+        <v>1186</v>
       </c>
       <c r="E667" t="s">
         <v>19</v>
@@ -26047,10 +26104,10 @@
         <v>20</v>
       </c>
       <c r="L667" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M667">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N667">
         <v>0</v>
@@ -26058,42 +26115,45 @@
     </row>
     <row r="668" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A668" t="s">
-        <v>1193</v>
+        <v>1187</v>
       </c>
       <c r="B668" t="s">
-        <v>1194</v>
+        <v>1188</v>
       </c>
       <c r="D668" t="s">
-        <v>1195</v>
+        <v>1180</v>
       </c>
       <c r="E668" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K668" t="s">
         <v>20</v>
       </c>
       <c r="L668" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M668">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N668">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="O668">
+        <v>154</v>
       </c>
     </row>
     <row r="669" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A669" t="s">
-        <v>1196</v>
+        <v>1187</v>
       </c>
       <c r="B669" t="s">
-        <v>1197</v>
+        <v>1189</v>
       </c>
       <c r="D669" t="s">
-        <v>1198</v>
+        <v>1186</v>
       </c>
       <c r="E669" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K669" t="s">
         <v>20</v>
@@ -26102,24 +26162,21 @@
         <v>21</v>
       </c>
       <c r="M669">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N669">
-        <v>9</v>
-      </c>
-      <c r="O669">
-        <v>81</v>
+        <v>0</v>
       </c>
     </row>
     <row r="670" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A670" t="s">
-        <v>1196</v>
+        <v>1190</v>
       </c>
       <c r="B670" t="s">
-        <v>1199</v>
+        <v>1191</v>
       </c>
       <c r="D670" t="s">
-        <v>228</v>
+        <v>1192</v>
       </c>
       <c r="E670" t="s">
         <v>19</v>
@@ -26131,7 +26188,7 @@
         <v>21</v>
       </c>
       <c r="M670">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="N670">
         <v>0</v>
@@ -26139,13 +26196,13 @@
     </row>
     <row r="671" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A671" t="s">
-        <v>1200</v>
+        <v>1193</v>
       </c>
       <c r="B671" t="s">
-        <v>1201</v>
+        <v>1194</v>
       </c>
       <c r="D671" t="s">
-        <v>1202</v>
+        <v>1195</v>
       </c>
       <c r="E671" t="s">
         <v>19</v>
@@ -26165,16 +26222,16 @@
     </row>
     <row r="672" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A672" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="B672" t="s">
-        <v>1201</v>
+        <v>1197</v>
       </c>
       <c r="D672" t="s">
-        <v>1203</v>
+        <v>1198</v>
       </c>
       <c r="E672" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K672" t="s">
         <v>20</v>
@@ -26183,21 +26240,24 @@
         <v>21</v>
       </c>
       <c r="M672">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="N672">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="O672">
+        <v>363</v>
       </c>
     </row>
     <row r="673" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A673" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="B673" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="D673" t="s">
-        <v>1204</v>
+        <v>228</v>
       </c>
       <c r="E673" t="s">
         <v>19</v>
@@ -26209,7 +26269,7 @@
         <v>21</v>
       </c>
       <c r="M673">
-        <v>1.5</v>
+        <v>11</v>
       </c>
       <c r="N673">
         <v>0</v>
@@ -26223,7 +26283,7 @@
         <v>1201</v>
       </c>
       <c r="D674" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="E674" t="s">
         <v>19</v>
@@ -26235,7 +26295,7 @@
         <v>21</v>
       </c>
       <c r="M674">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N674">
         <v>0</v>
@@ -26243,31 +26303,109 @@
     </row>
     <row r="675" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A675" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B675" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D675" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E675" t="s">
+        <v>19</v>
+      </c>
+      <c r="K675" t="s">
+        <v>20</v>
+      </c>
+      <c r="L675" t="s">
+        <v>21</v>
+      </c>
+      <c r="M675">
+        <v>3</v>
+      </c>
+      <c r="N675">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="676" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A676" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B676" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D676" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E676" t="s">
+        <v>19</v>
+      </c>
+      <c r="K676" t="s">
+        <v>20</v>
+      </c>
+      <c r="L676" t="s">
+        <v>21</v>
+      </c>
+      <c r="M676">
+        <v>1.5</v>
+      </c>
+      <c r="N676">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="677" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A677" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B677" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D677" t="s">
+        <v>1205</v>
+      </c>
+      <c r="E677" t="s">
+        <v>19</v>
+      </c>
+      <c r="K677" t="s">
+        <v>20</v>
+      </c>
+      <c r="L677" t="s">
+        <v>21</v>
+      </c>
+      <c r="M677">
+        <v>4</v>
+      </c>
+      <c r="N677">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="678" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A678" t="s">
         <v>1206</v>
       </c>
-      <c r="B675" t="s">
+      <c r="B678" t="s">
         <v>1207</v>
       </c>
-      <c r="D675" t="s">
+      <c r="D678" t="s">
         <v>1208</v>
       </c>
-      <c r="E675" t="s">
+      <c r="E678" t="s">
         <v>187</v>
       </c>
-      <c r="K675" t="s">
-        <v>20</v>
-      </c>
-      <c r="L675" t="s">
+      <c r="K678" t="s">
+        <v>20</v>
+      </c>
+      <c r="L678" t="s">
         <v>75</v>
       </c>
-      <c r="M675">
+      <c r="M678">
         <v>120</v>
       </c>
-      <c r="N675">
-        <v>6</v>
-      </c>
-      <c r="O675">
-        <v>720</v>
+      <c r="N678">
+        <v>5</v>
+      </c>
+      <c r="O678">
+        <v>600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mise à jour DPS — 04/06/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC90CB3-78E6-40B4-88BF-94EFD391CAAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77938DA-98A7-41DF-9361-5F9AE8CFA636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4080" uniqueCount="1237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4110" uniqueCount="1248">
   <si>
     <t>Début</t>
   </si>
@@ -3706,9 +3706,6 @@
     <t>05-06-2026</t>
   </si>
   <si>
-    <t>Renfort Banquet des vins de Loire</t>
-  </si>
-  <si>
     <t>Fête de la Musique Spotify</t>
   </si>
   <si>
@@ -3734,6 +3731,42 @@
   </si>
   <si>
     <t>Rue du Général Renault (P</t>
+  </si>
+  <si>
+    <t>04-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort Cross de Bercy 2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-PE - Evènement d'entreprise Google</t>
+  </si>
+  <si>
+    <t>08-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort Concert  FKA TWIGS - BODY HIGH TOUR</t>
+  </si>
+  <si>
+    <t>11-06-2026</t>
+  </si>
+  <si>
+    <t>Tournage SAUT DANS LA SEINE</t>
+  </si>
+  <si>
+    <t>Pont Marie</t>
+  </si>
+  <si>
+    <t>15-06-2026</t>
+  </si>
+  <si>
+    <t>Soirée d'entreprise METRO</t>
+  </si>
+  <si>
+    <t>Paris - Musée des Arts Fo</t>
+  </si>
+  <si>
+    <t>Summer Party Google</t>
   </si>
 </sst>
 </file>
@@ -4088,7 +4121,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P678"/>
+  <dimension ref="A1:P683"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -25396,10 +25429,10 @@
         <v>1158</v>
       </c>
       <c r="B643" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D643" t="s">
         <v>1229</v>
-      </c>
-      <c r="D643" t="s">
-        <v>1230</v>
       </c>
       <c r="E643" t="s">
         <v>19</v>
@@ -25425,7 +25458,7 @@
         <v>1158</v>
       </c>
       <c r="B644" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="D644" t="s">
         <v>18</v>
@@ -25454,10 +25487,10 @@
         <v>1158</v>
       </c>
       <c r="B645" t="s">
+        <v>1231</v>
+      </c>
+      <c r="D645" t="s">
         <v>1232</v>
-      </c>
-      <c r="D645" t="s">
-        <v>1233</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25564,6 +25597,21 @@
       <c r="E648" t="s">
         <v>19</v>
       </c>
+      <c r="F648">
+        <v>1</v>
+      </c>
+      <c r="G648">
+        <v>0</v>
+      </c>
+      <c r="H648">
+        <v>0</v>
+      </c>
+      <c r="I648">
+        <v>0</v>
+      </c>
+      <c r="J648">
+        <v>0</v>
+      </c>
       <c r="K648" t="s">
         <v>20</v>
       </c>
@@ -25585,13 +25633,13 @@
         <v>1163</v>
       </c>
       <c r="B649" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
       <c r="D649" t="s">
         <v>362</v>
       </c>
       <c r="E649" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K649" t="s">
         <v>20</v>
@@ -25603,21 +25651,24 @@
         <v>4.75</v>
       </c>
       <c r="N649">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O649">
+        <v>9.5</v>
       </c>
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1226</v>
+        <v>1236</v>
       </c>
       <c r="B650" t="s">
-        <v>397</v>
+        <v>1237</v>
       </c>
       <c r="D650" t="s">
-        <v>18</v>
+        <v>190</v>
       </c>
       <c r="E650" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K650" t="s">
         <v>20</v>
@@ -25626,27 +25677,27 @@
         <v>21</v>
       </c>
       <c r="M650">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N650">
         <v>4</v>
       </c>
       <c r="O650">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1166</v>
+        <v>1236</v>
       </c>
       <c r="B651" t="s">
-        <v>1167</v>
+        <v>1238</v>
       </c>
       <c r="D651" t="s">
-        <v>179</v>
+        <v>34</v>
       </c>
       <c r="E651" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K651" t="s">
         <v>20</v>
@@ -25655,24 +25706,24 @@
         <v>25</v>
       </c>
       <c r="M651">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N651">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O651">
-        <v>35</v>
+        <v>12</v>
       </c>
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1222</v>
+        <v>1226</v>
       </c>
       <c r="B652" t="s">
-        <v>1223</v>
+        <v>397</v>
       </c>
       <c r="D652" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="E652" t="s">
         <v>19</v>
@@ -25684,53 +25735,53 @@
         <v>21</v>
       </c>
       <c r="M652">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N652">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O652">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="653" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="B653" t="s">
-        <v>775</v>
+        <v>1167</v>
       </c>
       <c r="D653" t="s">
-        <v>1169</v>
+        <v>179</v>
       </c>
       <c r="E653" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K653" t="s">
         <v>20</v>
       </c>
       <c r="L653" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M653">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N653">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="O653">
-        <v>140</v>
+        <v>21</v>
       </c>
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1170</v>
+        <v>1239</v>
       </c>
       <c r="B654" t="s">
-        <v>777</v>
+        <v>1240</v>
       </c>
       <c r="D654" t="s">
-        <v>1169</v>
+        <v>362</v>
       </c>
       <c r="E654" t="s">
         <v>187</v>
@@ -25739,53 +25790,56 @@
         <v>20</v>
       </c>
       <c r="L654" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M654">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N654">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="O654">
-        <v>117</v>
+        <v>10</v>
       </c>
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1170</v>
+        <v>1222</v>
       </c>
       <c r="B655" t="s">
-        <v>643</v>
+        <v>1223</v>
       </c>
       <c r="D655" t="s">
-        <v>1171</v>
+        <v>34</v>
       </c>
       <c r="E655" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K655" t="s">
         <v>20</v>
       </c>
       <c r="L655" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M655">
-        <v>8.25</v>
+        <v>6</v>
       </c>
       <c r="N655">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="O655">
+        <v>18</v>
       </c>
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1170</v>
+        <v>1241</v>
       </c>
       <c r="B656" t="s">
-        <v>1227</v>
+        <v>1242</v>
       </c>
       <c r="D656" t="s">
-        <v>18</v>
+        <v>1243</v>
       </c>
       <c r="E656" t="s">
         <v>19</v>
@@ -25794,10 +25848,10 @@
         <v>20</v>
       </c>
       <c r="L656" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="M656">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N656">
         <v>0</v>
@@ -25805,100 +25859,100 @@
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1172</v>
+        <v>1168</v>
       </c>
       <c r="B657" t="s">
-        <v>546</v>
+        <v>775</v>
       </c>
       <c r="D657" t="s">
-        <v>34</v>
+        <v>1169</v>
       </c>
       <c r="E657" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K657" t="s">
         <v>20</v>
       </c>
       <c r="L657" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M657">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="N657">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="O657">
-        <v>6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1173</v>
+        <v>1170</v>
       </c>
       <c r="B658" t="s">
-        <v>1174</v>
+        <v>777</v>
       </c>
       <c r="D658" t="s">
-        <v>205</v>
+        <v>1169</v>
       </c>
       <c r="E658" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K658" t="s">
         <v>20</v>
       </c>
       <c r="L658" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M658">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N658">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="O658">
-        <v>28</v>
+        <v>108</v>
       </c>
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1175</v>
+        <v>1170</v>
       </c>
       <c r="B659" t="s">
-        <v>1176</v>
+        <v>643</v>
       </c>
       <c r="D659" t="s">
-        <v>34</v>
+        <v>1171</v>
       </c>
       <c r="E659" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K659" t="s">
         <v>20</v>
       </c>
       <c r="L659" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M659">
-        <v>6</v>
+        <v>8.25</v>
       </c>
       <c r="N659">
         <v>3</v>
       </c>
       <c r="O659">
-        <v>18</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>1177</v>
+        <v>1244</v>
       </c>
       <c r="B660" t="s">
-        <v>1219</v>
+        <v>1245</v>
       </c>
       <c r="D660" t="s">
-        <v>1220</v>
+        <v>1246</v>
       </c>
       <c r="E660" t="s">
         <v>187</v>
@@ -25910,24 +25964,24 @@
         <v>21</v>
       </c>
       <c r="M660">
-        <v>8</v>
+        <v>5.5</v>
       </c>
       <c r="N660">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O660">
-        <v>48</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
-        <v>1177</v>
+        <v>1172</v>
       </c>
       <c r="B661" t="s">
-        <v>1228</v>
+        <v>546</v>
       </c>
       <c r="D661" t="s">
-        <v>202</v>
+        <v>34</v>
       </c>
       <c r="E661" t="s">
         <v>187</v>
@@ -25939,24 +25993,24 @@
         <v>21</v>
       </c>
       <c r="M661">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N661">
         <v>1</v>
       </c>
       <c r="O661">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1177</v>
+        <v>1173</v>
       </c>
       <c r="B662" t="s">
-        <v>1235</v>
+        <v>1174</v>
       </c>
       <c r="D662" t="s">
-        <v>1236</v>
+        <v>205</v>
       </c>
       <c r="E662" t="s">
         <v>187</v>
@@ -25965,24 +26019,27 @@
         <v>20</v>
       </c>
       <c r="L662" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M662">
-        <v>10.5</v>
+        <v>7</v>
       </c>
       <c r="N662">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="O662">
+        <v>28</v>
       </c>
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>1178</v>
+        <v>1175</v>
       </c>
       <c r="B663" t="s">
-        <v>1179</v>
+        <v>1176</v>
       </c>
       <c r="D663" t="s">
-        <v>1180</v>
+        <v>34</v>
       </c>
       <c r="E663" t="s">
         <v>187</v>
@@ -25991,27 +26048,27 @@
         <v>20</v>
       </c>
       <c r="L663" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M663">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N663">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="O663">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1178</v>
+        <v>1175</v>
       </c>
       <c r="B664" t="s">
-        <v>1181</v>
+        <v>1247</v>
       </c>
       <c r="D664" t="s">
-        <v>1180</v>
+        <v>583</v>
       </c>
       <c r="E664" t="s">
         <v>187</v>
@@ -26020,27 +26077,24 @@
         <v>20</v>
       </c>
       <c r="L664" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M664">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N664">
-        <v>17</v>
-      </c>
-      <c r="O664">
-        <v>119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="665" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A665" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
       <c r="B665" t="s">
-        <v>1183</v>
+        <v>1219</v>
       </c>
       <c r="D665" t="s">
-        <v>1180</v>
+        <v>1220</v>
       </c>
       <c r="E665" t="s">
         <v>187</v>
@@ -26049,27 +26103,27 @@
         <v>20</v>
       </c>
       <c r="L665" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M665">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N665">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="O665">
-        <v>121</v>
+        <v>48</v>
       </c>
     </row>
     <row r="666" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A666" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
       <c r="B666" t="s">
-        <v>1184</v>
+        <v>1227</v>
       </c>
       <c r="D666" t="s">
-        <v>18</v>
+        <v>202</v>
       </c>
       <c r="E666" t="s">
         <v>187</v>
@@ -26084,30 +26138,33 @@
         <v>8</v>
       </c>
       <c r="N666">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="O666">
+        <v>24</v>
       </c>
     </row>
     <row r="667" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
       <c r="B667" t="s">
-        <v>1185</v>
+        <v>1234</v>
       </c>
       <c r="D667" t="s">
-        <v>1186</v>
+        <v>1235</v>
       </c>
       <c r="E667" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K667" t="s">
         <v>20</v>
       </c>
       <c r="L667" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="M667">
-        <v>5</v>
+        <v>10.5</v>
       </c>
       <c r="N667">
         <v>0</v>
@@ -26115,10 +26172,10 @@
     </row>
     <row r="668" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A668" t="s">
-        <v>1187</v>
+        <v>1178</v>
       </c>
       <c r="B668" t="s">
-        <v>1188</v>
+        <v>1179</v>
       </c>
       <c r="D668" t="s">
         <v>1180</v>
@@ -26133,79 +26190,85 @@
         <v>50</v>
       </c>
       <c r="M668">
+        <v>5</v>
+      </c>
+      <c r="N668">
         <v>11</v>
       </c>
-      <c r="N668">
-        <v>14</v>
-      </c>
       <c r="O668">
-        <v>154</v>
+        <v>55</v>
       </c>
     </row>
     <row r="669" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A669" t="s">
-        <v>1187</v>
+        <v>1178</v>
       </c>
       <c r="B669" t="s">
-        <v>1189</v>
+        <v>1181</v>
       </c>
       <c r="D669" t="s">
-        <v>1186</v>
+        <v>1180</v>
       </c>
       <c r="E669" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K669" t="s">
         <v>20</v>
       </c>
       <c r="L669" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M669">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N669">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="O669">
+        <v>133</v>
       </c>
     </row>
     <row r="670" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A670" t="s">
-        <v>1190</v>
+        <v>1182</v>
       </c>
       <c r="B670" t="s">
-        <v>1191</v>
+        <v>1183</v>
       </c>
       <c r="D670" t="s">
-        <v>1192</v>
+        <v>1180</v>
       </c>
       <c r="E670" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K670" t="s">
         <v>20</v>
       </c>
       <c r="L670" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M670">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N670">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="O670">
+        <v>165</v>
       </c>
     </row>
     <row r="671" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A671" t="s">
-        <v>1193</v>
+        <v>1182</v>
       </c>
       <c r="B671" t="s">
-        <v>1194</v>
+        <v>1184</v>
       </c>
       <c r="D671" t="s">
-        <v>1195</v>
+        <v>18</v>
       </c>
       <c r="E671" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K671" t="s">
         <v>20</v>
@@ -26214,76 +26277,79 @@
         <v>21</v>
       </c>
       <c r="M671">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N671">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="O671">
+        <v>32</v>
       </c>
     </row>
     <row r="672" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A672" t="s">
-        <v>1196</v>
+        <v>1182</v>
       </c>
       <c r="B672" t="s">
-        <v>1197</v>
+        <v>1185</v>
       </c>
       <c r="D672" t="s">
-        <v>1198</v>
+        <v>1186</v>
       </c>
       <c r="E672" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K672" t="s">
         <v>20</v>
       </c>
       <c r="L672" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M672">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="N672">
-        <v>11</v>
-      </c>
-      <c r="O672">
-        <v>363</v>
+        <v>0</v>
       </c>
     </row>
     <row r="673" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A673" t="s">
-        <v>1196</v>
+        <v>1187</v>
       </c>
       <c r="B673" t="s">
-        <v>1199</v>
+        <v>1188</v>
       </c>
       <c r="D673" t="s">
-        <v>228</v>
+        <v>1180</v>
       </c>
       <c r="E673" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K673" t="s">
         <v>20</v>
       </c>
       <c r="L673" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M673">
         <v>11</v>
       </c>
       <c r="N673">
-        <v>0</v>
+        <v>16</v>
+      </c>
+      <c r="O673">
+        <v>176</v>
       </c>
     </row>
     <row r="674" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A674" t="s">
-        <v>1200</v>
+        <v>1187</v>
       </c>
       <c r="B674" t="s">
-        <v>1201</v>
+        <v>1189</v>
       </c>
       <c r="D674" t="s">
-        <v>1202</v>
+        <v>1186</v>
       </c>
       <c r="E674" t="s">
         <v>19</v>
@@ -26295,7 +26361,7 @@
         <v>21</v>
       </c>
       <c r="M674">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N674">
         <v>0</v>
@@ -26303,13 +26369,13 @@
     </row>
     <row r="675" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A675" t="s">
-        <v>1200</v>
+        <v>1190</v>
       </c>
       <c r="B675" t="s">
-        <v>1201</v>
+        <v>1191</v>
       </c>
       <c r="D675" t="s">
-        <v>1203</v>
+        <v>1192</v>
       </c>
       <c r="E675" t="s">
         <v>19</v>
@@ -26321,7 +26387,7 @@
         <v>21</v>
       </c>
       <c r="M675">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N675">
         <v>0</v>
@@ -26329,13 +26395,13 @@
     </row>
     <row r="676" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A676" t="s">
-        <v>1200</v>
+        <v>1193</v>
       </c>
       <c r="B676" t="s">
-        <v>1201</v>
+        <v>1194</v>
       </c>
       <c r="D676" t="s">
-        <v>1204</v>
+        <v>1195</v>
       </c>
       <c r="E676" t="s">
         <v>19</v>
@@ -26347,7 +26413,7 @@
         <v>21</v>
       </c>
       <c r="M676">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="N676">
         <v>0</v>
@@ -26355,16 +26421,16 @@
     </row>
     <row r="677" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A677" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="B677" t="s">
-        <v>1201</v>
+        <v>1197</v>
       </c>
       <c r="D677" t="s">
-        <v>1205</v>
+        <v>1198</v>
       </c>
       <c r="E677" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K677" t="s">
         <v>20</v>
@@ -26373,38 +26439,171 @@
         <v>21</v>
       </c>
       <c r="M677">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="N677">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="O677">
+        <v>363</v>
       </c>
     </row>
     <row r="678" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A678" t="s">
+        <v>1196</v>
+      </c>
+      <c r="B678" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D678" t="s">
+        <v>228</v>
+      </c>
+      <c r="E678" t="s">
+        <v>19</v>
+      </c>
+      <c r="K678" t="s">
+        <v>20</v>
+      </c>
+      <c r="L678" t="s">
+        <v>21</v>
+      </c>
+      <c r="M678">
+        <v>11</v>
+      </c>
+      <c r="N678">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="679" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A679" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B679" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D679" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E679" t="s">
+        <v>19</v>
+      </c>
+      <c r="K679" t="s">
+        <v>20</v>
+      </c>
+      <c r="L679" t="s">
+        <v>21</v>
+      </c>
+      <c r="M679">
+        <v>3</v>
+      </c>
+      <c r="N679">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="680" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A680" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B680" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D680" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E680" t="s">
+        <v>19</v>
+      </c>
+      <c r="K680" t="s">
+        <v>20</v>
+      </c>
+      <c r="L680" t="s">
+        <v>21</v>
+      </c>
+      <c r="M680">
+        <v>3</v>
+      </c>
+      <c r="N680">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A681" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B681" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D681" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E681" t="s">
+        <v>19</v>
+      </c>
+      <c r="K681" t="s">
+        <v>20</v>
+      </c>
+      <c r="L681" t="s">
+        <v>21</v>
+      </c>
+      <c r="M681">
+        <v>1.5</v>
+      </c>
+      <c r="N681">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="682" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A682" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B682" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D682" t="s">
+        <v>1205</v>
+      </c>
+      <c r="E682" t="s">
+        <v>19</v>
+      </c>
+      <c r="K682" t="s">
+        <v>20</v>
+      </c>
+      <c r="L682" t="s">
+        <v>21</v>
+      </c>
+      <c r="M682">
+        <v>4</v>
+      </c>
+      <c r="N682">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="683" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A683" t="s">
         <v>1206</v>
       </c>
-      <c r="B678" t="s">
+      <c r="B683" t="s">
         <v>1207</v>
       </c>
-      <c r="D678" t="s">
+      <c r="D683" t="s">
         <v>1208</v>
       </c>
-      <c r="E678" t="s">
+      <c r="E683" t="s">
         <v>187</v>
       </c>
-      <c r="K678" t="s">
-        <v>20</v>
-      </c>
-      <c r="L678" t="s">
+      <c r="K683" t="s">
+        <v>20</v>
+      </c>
+      <c r="L683" t="s">
         <v>75</v>
       </c>
-      <c r="M678">
+      <c r="M683">
         <v>120</v>
       </c>
-      <c r="N678">
+      <c r="N683">
         <v>5</v>
       </c>
-      <c r="O678">
+      <c r="O683">
         <v>600</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour DPS — 09/06/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E77938DA-98A7-41DF-9361-5F9AE8CFA636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{160CE6AD-2818-4AA0-9CA6-CD92F0108F51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4110" uniqueCount="1248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4140" uniqueCount="1257">
   <si>
     <t>Début</t>
   </si>
@@ -3767,6 +3767,33 @@
   </si>
   <si>
     <t>Summer Party Google</t>
+  </si>
+  <si>
+    <t>Forum emploi</t>
+  </si>
+  <si>
+    <t>Vitry-sur-Seine</t>
+  </si>
+  <si>
+    <t>12-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME  - Concert KALASH</t>
+  </si>
+  <si>
+    <t>25-06-2026</t>
+  </si>
+  <si>
+    <t>02-07-2026</t>
+  </si>
+  <si>
+    <t>Olympiades du groupe AFD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feu dartifice </t>
+  </si>
+  <si>
+    <t>Alfortville</t>
   </si>
 </sst>
 </file>
@@ -4121,7 +4148,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P683"/>
+  <dimension ref="A1:P688"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -25728,6 +25755,21 @@
       <c r="E652" t="s">
         <v>19</v>
       </c>
+      <c r="F652">
+        <v>5</v>
+      </c>
+      <c r="G652">
+        <v>0</v>
+      </c>
+      <c r="H652">
+        <v>0</v>
+      </c>
+      <c r="I652">
+        <v>0</v>
+      </c>
+      <c r="J652">
+        <v>0</v>
+      </c>
       <c r="K652" t="s">
         <v>20</v>
       </c>
@@ -25757,6 +25799,21 @@
       <c r="E653" t="s">
         <v>19</v>
       </c>
+      <c r="F653">
+        <v>0</v>
+      </c>
+      <c r="G653">
+        <v>0</v>
+      </c>
+      <c r="H653">
+        <v>0</v>
+      </c>
+      <c r="I653">
+        <v>0</v>
+      </c>
+      <c r="J653">
+        <v>0</v>
+      </c>
       <c r="K653" t="s">
         <v>20</v>
       </c>
@@ -25784,7 +25841,7 @@
         <v>362</v>
       </c>
       <c r="E654" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K654" t="s">
         <v>20</v>
@@ -25796,10 +25853,10 @@
         <v>5</v>
       </c>
       <c r="N654">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O654">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
@@ -25833,13 +25890,13 @@
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1241</v>
+        <v>1222</v>
       </c>
       <c r="B656" t="s">
-        <v>1242</v>
+        <v>1248</v>
       </c>
       <c r="D656" t="s">
-        <v>1243</v>
+        <v>1249</v>
       </c>
       <c r="E656" t="s">
         <v>19</v>
@@ -25848,24 +25905,27 @@
         <v>20</v>
       </c>
       <c r="L656" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M656">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N656">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O656">
+        <v>14</v>
       </c>
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1168</v>
+        <v>1241</v>
       </c>
       <c r="B657" t="s">
-        <v>775</v>
+        <v>1242</v>
       </c>
       <c r="D657" t="s">
-        <v>1169</v>
+        <v>1243</v>
       </c>
       <c r="E657" t="s">
         <v>19</v>
@@ -25874,27 +25934,24 @@
         <v>20</v>
       </c>
       <c r="L657" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M657">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="N657">
-        <v>13</v>
-      </c>
-      <c r="O657">
-        <v>130</v>
+        <v>0</v>
       </c>
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1170</v>
+        <v>1250</v>
       </c>
       <c r="B658" t="s">
-        <v>777</v>
+        <v>1251</v>
       </c>
       <c r="D658" t="s">
-        <v>1169</v>
+        <v>60</v>
       </c>
       <c r="E658" t="s">
         <v>19</v>
@@ -25903,27 +25960,27 @@
         <v>20</v>
       </c>
       <c r="L658" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M658">
-        <v>9</v>
+        <v>6.25</v>
       </c>
       <c r="N658">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="O658">
-        <v>108</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="B659" t="s">
-        <v>643</v>
+        <v>775</v>
       </c>
       <c r="D659" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="E659" t="s">
         <v>19</v>
@@ -25932,27 +25989,27 @@
         <v>20</v>
       </c>
       <c r="L659" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M659">
-        <v>8.25</v>
+        <v>10</v>
       </c>
       <c r="N659">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="O659">
-        <v>16.5</v>
+        <v>130</v>
       </c>
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>1244</v>
+        <v>1170</v>
       </c>
       <c r="B660" t="s">
-        <v>1245</v>
+        <v>777</v>
       </c>
       <c r="D660" t="s">
-        <v>1246</v>
+        <v>1169</v>
       </c>
       <c r="E660" t="s">
         <v>187</v>
@@ -25961,59 +26018,59 @@
         <v>20</v>
       </c>
       <c r="L660" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M660">
-        <v>5.5</v>
+        <v>9</v>
       </c>
       <c r="N660">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="O660">
-        <v>5.5</v>
+        <v>102</v>
       </c>
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A661" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="B661" t="s">
-        <v>546</v>
+        <v>643</v>
       </c>
       <c r="D661" t="s">
-        <v>34</v>
+        <v>1171</v>
       </c>
       <c r="E661" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K661" t="s">
         <v>20</v>
       </c>
       <c r="L661" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M661">
-        <v>6</v>
+        <v>8.25</v>
       </c>
       <c r="N661">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O661">
-        <v>6</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1173</v>
+        <v>1244</v>
       </c>
       <c r="B662" t="s">
-        <v>1174</v>
+        <v>1245</v>
       </c>
       <c r="D662" t="s">
-        <v>205</v>
+        <v>1246</v>
       </c>
       <c r="E662" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K662" t="s">
         <v>20</v>
@@ -26022,21 +26079,21 @@
         <v>21</v>
       </c>
       <c r="M662">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N662">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O662">
-        <v>28</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>1175</v>
+        <v>1172</v>
       </c>
       <c r="B663" t="s">
-        <v>1176</v>
+        <v>546</v>
       </c>
       <c r="D663" t="s">
         <v>34</v>
@@ -26054,21 +26111,21 @@
         <v>6</v>
       </c>
       <c r="N663">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O663">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B664" t="s">
-        <v>1247</v>
+        <v>1174</v>
       </c>
       <c r="D664" t="s">
-        <v>583</v>
+        <v>205</v>
       </c>
       <c r="E664" t="s">
         <v>187</v>
@@ -26080,21 +26137,24 @@
         <v>21</v>
       </c>
       <c r="M664">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N664">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="O664">
+        <v>28</v>
       </c>
     </row>
     <row r="665" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A665" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="B665" t="s">
-        <v>1219</v>
+        <v>1176</v>
       </c>
       <c r="D665" t="s">
-        <v>1220</v>
+        <v>34</v>
       </c>
       <c r="E665" t="s">
         <v>187</v>
@@ -26106,24 +26166,24 @@
         <v>21</v>
       </c>
       <c r="M665">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N665">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O665">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="666" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A666" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="B666" t="s">
-        <v>1227</v>
+        <v>1247</v>
       </c>
       <c r="D666" t="s">
-        <v>202</v>
+        <v>583</v>
       </c>
       <c r="E666" t="s">
         <v>187</v>
@@ -26135,13 +26195,10 @@
         <v>21</v>
       </c>
       <c r="M666">
-        <v>8</v>
+        <v>9.5</v>
       </c>
       <c r="N666">
-        <v>3</v>
-      </c>
-      <c r="O666">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="667" spans="1:15" x14ac:dyDescent="0.35">
@@ -26149,10 +26206,10 @@
         <v>1177</v>
       </c>
       <c r="B667" t="s">
-        <v>1234</v>
+        <v>1219</v>
       </c>
       <c r="D667" t="s">
-        <v>1235</v>
+        <v>1220</v>
       </c>
       <c r="E667" t="s">
         <v>187</v>
@@ -26161,24 +26218,27 @@
         <v>20</v>
       </c>
       <c r="L667" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M667">
-        <v>10.5</v>
+        <v>8</v>
       </c>
       <c r="N667">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="O667">
+        <v>48</v>
       </c>
     </row>
     <row r="668" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A668" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B668" t="s">
-        <v>1179</v>
+        <v>1227</v>
       </c>
       <c r="D668" t="s">
-        <v>1180</v>
+        <v>202</v>
       </c>
       <c r="E668" t="s">
         <v>187</v>
@@ -26187,27 +26247,27 @@
         <v>20</v>
       </c>
       <c r="L668" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M668">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N668">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="O668">
-        <v>55</v>
+        <v>24</v>
       </c>
     </row>
     <row r="669" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A669" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B669" t="s">
-        <v>1181</v>
+        <v>1234</v>
       </c>
       <c r="D669" t="s">
-        <v>1180</v>
+        <v>1235</v>
       </c>
       <c r="E669" t="s">
         <v>187</v>
@@ -26216,27 +26276,24 @@
         <v>20</v>
       </c>
       <c r="L669" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M669">
-        <v>7</v>
+        <v>10.5</v>
       </c>
       <c r="N669">
-        <v>19</v>
-      </c>
-      <c r="O669">
-        <v>133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="670" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A670" t="s">
-        <v>1182</v>
+        <v>1252</v>
       </c>
       <c r="B670" t="s">
-        <v>1183</v>
+        <v>770</v>
       </c>
       <c r="D670" t="s">
-        <v>1180</v>
+        <v>771</v>
       </c>
       <c r="E670" t="s">
         <v>187</v>
@@ -26245,27 +26302,27 @@
         <v>20</v>
       </c>
       <c r="L670" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M670">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="N670">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="O670">
-        <v>165</v>
+        <v>6</v>
       </c>
     </row>
     <row r="671" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A671" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B671" t="s">
-        <v>1184</v>
+        <v>1179</v>
       </c>
       <c r="D671" t="s">
-        <v>18</v>
+        <v>1180</v>
       </c>
       <c r="E671" t="s">
         <v>187</v>
@@ -26274,50 +26331,53 @@
         <v>20</v>
       </c>
       <c r="L671" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M671">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N671">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="O671">
-        <v>32</v>
+        <v>60</v>
       </c>
     </row>
     <row r="672" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A672" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B672" t="s">
-        <v>1185</v>
+        <v>1181</v>
       </c>
       <c r="D672" t="s">
-        <v>1186</v>
+        <v>1180</v>
       </c>
       <c r="E672" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K672" t="s">
         <v>20</v>
       </c>
       <c r="L672" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="M672">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N672">
-        <v>0</v>
+        <v>19</v>
+      </c>
+      <c r="O672">
+        <v>133</v>
       </c>
     </row>
     <row r="673" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A673" t="s">
-        <v>1187</v>
+        <v>1182</v>
       </c>
       <c r="B673" t="s">
-        <v>1188</v>
+        <v>1183</v>
       </c>
       <c r="D673" t="s">
         <v>1180</v>
@@ -26343,16 +26403,16 @@
     </row>
     <row r="674" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A674" t="s">
-        <v>1187</v>
+        <v>1182</v>
       </c>
       <c r="B674" t="s">
-        <v>1189</v>
+        <v>1184</v>
       </c>
       <c r="D674" t="s">
-        <v>1186</v>
+        <v>18</v>
       </c>
       <c r="E674" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K674" t="s">
         <v>20</v>
@@ -26361,21 +26421,24 @@
         <v>21</v>
       </c>
       <c r="M674">
+        <v>8</v>
+      </c>
+      <c r="N674">
         <v>5</v>
       </c>
-      <c r="N674">
-        <v>0</v>
+      <c r="O674">
+        <v>40</v>
       </c>
     </row>
     <row r="675" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A675" t="s">
-        <v>1190</v>
+        <v>1182</v>
       </c>
       <c r="B675" t="s">
-        <v>1191</v>
+        <v>1185</v>
       </c>
       <c r="D675" t="s">
-        <v>1192</v>
+        <v>1186</v>
       </c>
       <c r="E675" t="s">
         <v>19</v>
@@ -26384,10 +26447,10 @@
         <v>20</v>
       </c>
       <c r="L675" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="M675">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N675">
         <v>0</v>
@@ -26395,42 +26458,45 @@
     </row>
     <row r="676" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A676" t="s">
-        <v>1193</v>
+        <v>1187</v>
       </c>
       <c r="B676" t="s">
-        <v>1194</v>
+        <v>1188</v>
       </c>
       <c r="D676" t="s">
-        <v>1195</v>
+        <v>1180</v>
       </c>
       <c r="E676" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K676" t="s">
         <v>20</v>
       </c>
       <c r="L676" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="M676">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N676">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="O676">
+        <v>165</v>
       </c>
     </row>
     <row r="677" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A677" t="s">
-        <v>1196</v>
+        <v>1187</v>
       </c>
       <c r="B677" t="s">
-        <v>1197</v>
+        <v>1189</v>
       </c>
       <c r="D677" t="s">
-        <v>1198</v>
+        <v>1186</v>
       </c>
       <c r="E677" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K677" t="s">
         <v>20</v>
@@ -26439,24 +26505,21 @@
         <v>21</v>
       </c>
       <c r="M677">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="N677">
-        <v>11</v>
-      </c>
-      <c r="O677">
-        <v>363</v>
+        <v>0</v>
       </c>
     </row>
     <row r="678" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A678" t="s">
-        <v>1196</v>
+        <v>1190</v>
       </c>
       <c r="B678" t="s">
-        <v>1199</v>
+        <v>1191</v>
       </c>
       <c r="D678" t="s">
-        <v>228</v>
+        <v>1192</v>
       </c>
       <c r="E678" t="s">
         <v>19</v>
@@ -26468,7 +26531,7 @@
         <v>21</v>
       </c>
       <c r="M678">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="N678">
         <v>0</v>
@@ -26476,13 +26539,13 @@
     </row>
     <row r="679" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A679" t="s">
-        <v>1200</v>
+        <v>1193</v>
       </c>
       <c r="B679" t="s">
-        <v>1201</v>
+        <v>1194</v>
       </c>
       <c r="D679" t="s">
-        <v>1202</v>
+        <v>1195</v>
       </c>
       <c r="E679" t="s">
         <v>19</v>
@@ -26502,42 +26565,45 @@
     </row>
     <row r="680" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A680" t="s">
-        <v>1200</v>
+        <v>1253</v>
       </c>
       <c r="B680" t="s">
-        <v>1201</v>
+        <v>1254</v>
       </c>
       <c r="D680" t="s">
-        <v>1203</v>
+        <v>345</v>
       </c>
       <c r="E680" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K680" t="s">
         <v>20</v>
       </c>
       <c r="L680" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M680">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="N680">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="O680">
+        <v>2.75</v>
       </c>
     </row>
     <row r="681" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A681" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="B681" t="s">
-        <v>1201</v>
+        <v>1197</v>
       </c>
       <c r="D681" t="s">
-        <v>1204</v>
+        <v>1198</v>
       </c>
       <c r="E681" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K681" t="s">
         <v>20</v>
@@ -26546,21 +26612,24 @@
         <v>21</v>
       </c>
       <c r="M681">
-        <v>1.5</v>
+        <v>33</v>
       </c>
       <c r="N681">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="O681">
+        <v>363</v>
       </c>
     </row>
     <row r="682" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A682" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="B682" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="D682" t="s">
-        <v>1205</v>
+        <v>228</v>
       </c>
       <c r="E682" t="s">
         <v>19</v>
@@ -26572,7 +26641,7 @@
         <v>21</v>
       </c>
       <c r="M682">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N682">
         <v>0</v>
@@ -26580,30 +26649,160 @@
     </row>
     <row r="683" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A683" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B683" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D683" t="s">
+        <v>1202</v>
+      </c>
+      <c r="E683" t="s">
+        <v>19</v>
+      </c>
+      <c r="K683" t="s">
+        <v>20</v>
+      </c>
+      <c r="L683" t="s">
+        <v>21</v>
+      </c>
+      <c r="M683">
+        <v>3</v>
+      </c>
+      <c r="N683">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="684" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A684" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B684" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D684" t="s">
+        <v>1203</v>
+      </c>
+      <c r="E684" t="s">
+        <v>19</v>
+      </c>
+      <c r="K684" t="s">
+        <v>20</v>
+      </c>
+      <c r="L684" t="s">
+        <v>21</v>
+      </c>
+      <c r="M684">
+        <v>3</v>
+      </c>
+      <c r="N684">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="685" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A685" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B685" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D685" t="s">
+        <v>1204</v>
+      </c>
+      <c r="E685" t="s">
+        <v>19</v>
+      </c>
+      <c r="K685" t="s">
+        <v>20</v>
+      </c>
+      <c r="L685" t="s">
+        <v>21</v>
+      </c>
+      <c r="M685">
+        <v>1.5</v>
+      </c>
+      <c r="N685">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="686" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A686" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B686" t="s">
+        <v>1201</v>
+      </c>
+      <c r="D686" t="s">
+        <v>1205</v>
+      </c>
+      <c r="E686" t="s">
+        <v>19</v>
+      </c>
+      <c r="K686" t="s">
+        <v>20</v>
+      </c>
+      <c r="L686" t="s">
+        <v>21</v>
+      </c>
+      <c r="M686">
+        <v>4</v>
+      </c>
+      <c r="N686">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="687" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A687" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B687" t="s">
+        <v>1255</v>
+      </c>
+      <c r="D687" t="s">
+        <v>1256</v>
+      </c>
+      <c r="E687" t="s">
+        <v>187</v>
+      </c>
+      <c r="K687" t="s">
+        <v>20</v>
+      </c>
+      <c r="L687" t="s">
+        <v>25</v>
+      </c>
+      <c r="M687">
+        <v>4</v>
+      </c>
+      <c r="N687">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="688" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A688" t="s">
         <v>1206</v>
       </c>
-      <c r="B683" t="s">
+      <c r="B688" t="s">
         <v>1207</v>
       </c>
-      <c r="D683" t="s">
+      <c r="D688" t="s">
         <v>1208</v>
       </c>
-      <c r="E683" t="s">
+      <c r="E688" t="s">
         <v>187</v>
       </c>
-      <c r="K683" t="s">
-        <v>20</v>
-      </c>
-      <c r="L683" t="s">
+      <c r="K688" t="s">
+        <v>20</v>
+      </c>
+      <c r="L688" t="s">
         <v>75</v>
       </c>
-      <c r="M683">
+      <c r="M688">
         <v>120</v>
       </c>
-      <c r="N683">
+      <c r="N688">
         <v>5</v>
       </c>
-      <c r="O683">
+      <c r="O688">
         <v>600</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour DPS — 23/06/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{160CE6AD-2818-4AA0-9CA6-CD92F0108F51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D422330-40F1-4862-B67A-03482AF5134F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4140" uniqueCount="1257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4194" uniqueCount="1271">
   <si>
     <t>Début</t>
   </si>
@@ -3562,24 +3562,9 @@
     <t>26-06-2026</t>
   </si>
   <si>
-    <t>[PROV] Solidays J1 - 1/2</t>
-  </si>
-  <si>
-    <t>Hippodrome de Longchamp</t>
-  </si>
-  <si>
-    <t>[PROV] Solidays J1 - 2/2</t>
-  </si>
-  <si>
     <t>27-06-2026</t>
   </si>
   <si>
-    <t>[PROV] Solidays J2</t>
-  </si>
-  <si>
-    <t>[PROV] La marche des fiertés</t>
-  </si>
-  <si>
     <t>FestiMarne 2026 - J1</t>
   </si>
   <si>
@@ -3589,9 +3574,6 @@
     <t>28-06-2026</t>
   </si>
   <si>
-    <t>[PROV] Solidays J3</t>
-  </si>
-  <si>
     <t>FestiMarne 2026 - J2</t>
   </si>
   <si>
@@ -3646,9 +3628,6 @@
     <t>15-07-2026</t>
   </si>
   <si>
-    <t>[PROV] Vieilles Charrues 2026</t>
-  </si>
-  <si>
     <t>Carhaix (29)</t>
   </si>
   <si>
@@ -3682,12 +3661,6 @@
     <t>25-05-2026</t>
   </si>
   <si>
-    <t>Fête de la musique</t>
-  </si>
-  <si>
-    <t>Place de la bastille</t>
-  </si>
-  <si>
     <t>Renfort DPS-ME - Retransmission Match foot + Concert Bouss</t>
   </si>
   <si>
@@ -3727,9 +3700,6 @@
     <t>Renfort PlayOff - Demi Finale - Match 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Fête la musique Playground </t>
-  </si>
-  <si>
     <t>Rue du Général Renault (P</t>
   </si>
   <si>
@@ -3794,6 +3764,78 @@
   </si>
   <si>
     <t>Alfortville</t>
+  </si>
+  <si>
+    <t>19-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME  - Concert Foo Fighters</t>
+  </si>
+  <si>
+    <t>Fête la musique Playground</t>
+  </si>
+  <si>
+    <t>22-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME  - Concert  Iron Maiden</t>
+  </si>
+  <si>
+    <t>23-06-2026</t>
+  </si>
+  <si>
+    <t>Renfort PlayOff - Final J5</t>
+  </si>
+  <si>
+    <t>Renfort Solidays J1 - PSA Paris 2</t>
+  </si>
+  <si>
+    <t>Renfort Solidays J1 - VPS</t>
+  </si>
+  <si>
+    <t>Renfort Solidays J2 - PSA Cesar Circus</t>
+  </si>
+  <si>
+    <t>Renfort Solidays J2 - VPS</t>
+  </si>
+  <si>
+    <t>Renfort Solidays J3 - PSA Paris 1</t>
+  </si>
+  <si>
+    <t>Renfort Solidays J3 - VPS A</t>
+  </si>
+  <si>
+    <t>Renfort Solidays J3 - VPS B</t>
+  </si>
+  <si>
+    <t>30-06-2026</t>
+  </si>
+  <si>
+    <t>Du Stade vers l'emploi - LIFA</t>
+  </si>
+  <si>
+    <t>Évry-Courcouronnes</t>
+  </si>
+  <si>
+    <t>03-07-2026</t>
+  </si>
+  <si>
+    <t>Guinguette d'été</t>
+  </si>
+  <si>
+    <t>Paris - Place Raoul-Dautr</t>
+  </si>
+  <si>
+    <t>10-07-2026</t>
+  </si>
+  <si>
+    <t>11-07-2026</t>
+  </si>
+  <si>
+    <t>Course Copenhague-Paris 2026</t>
+  </si>
+  <si>
+    <t>Vieilles Charrues 2026</t>
   </si>
 </sst>
 </file>
@@ -4148,7 +4190,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P688"/>
+  <dimension ref="A1:P697"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -24960,7 +25002,7 @@
         <v>1149</v>
       </c>
       <c r="B629" t="s">
-        <v>1211</v>
+        <v>1204</v>
       </c>
       <c r="D629" t="s">
         <v>34</v>
@@ -24989,10 +25031,10 @@
         <v>1149</v>
       </c>
       <c r="B630" t="s">
-        <v>1212</v>
+        <v>1205</v>
       </c>
       <c r="D630" t="s">
-        <v>1213</v>
+        <v>1206</v>
       </c>
       <c r="E630" t="s">
         <v>19</v>
@@ -25106,7 +25148,7 @@
         <v>1150</v>
       </c>
       <c r="B633" t="s">
-        <v>1209</v>
+        <v>1202</v>
       </c>
       <c r="D633" t="s">
         <v>60</v>
@@ -25132,13 +25174,13 @@
     </row>
     <row r="634" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A634" t="s">
-        <v>1218</v>
+        <v>1211</v>
       </c>
       <c r="B634" t="s">
-        <v>1217</v>
+        <v>1210</v>
       </c>
       <c r="D634" t="s">
-        <v>1216</v>
+        <v>1209</v>
       </c>
       <c r="E634" t="s">
         <v>19</v>
@@ -25252,10 +25294,10 @@
         <v>1153</v>
       </c>
       <c r="B637" t="s">
-        <v>1215</v>
+        <v>1208</v>
       </c>
       <c r="D637" t="s">
-        <v>1214</v>
+        <v>1207</v>
       </c>
       <c r="E637" t="s">
         <v>19</v>
@@ -25296,10 +25338,10 @@
         <v>1153</v>
       </c>
       <c r="B638" t="s">
-        <v>1224</v>
+        <v>1215</v>
       </c>
       <c r="D638" t="s">
-        <v>1216</v>
+        <v>1209</v>
       </c>
       <c r="E638" t="s">
         <v>19</v>
@@ -25325,7 +25367,7 @@
         <v>1155</v>
       </c>
       <c r="B639" t="s">
-        <v>1210</v>
+        <v>1203</v>
       </c>
       <c r="D639" t="s">
         <v>60</v>
@@ -25427,7 +25469,7 @@
         <v>1158</v>
       </c>
       <c r="B642" t="s">
-        <v>1221</v>
+        <v>1212</v>
       </c>
       <c r="D642" t="s">
         <v>34</v>
@@ -25456,10 +25498,10 @@
         <v>1158</v>
       </c>
       <c r="B643" t="s">
-        <v>1228</v>
+        <v>1219</v>
       </c>
       <c r="D643" t="s">
-        <v>1229</v>
+        <v>1220</v>
       </c>
       <c r="E643" t="s">
         <v>19</v>
@@ -25485,7 +25527,7 @@
         <v>1158</v>
       </c>
       <c r="B644" t="s">
-        <v>1230</v>
+        <v>1221</v>
       </c>
       <c r="D644" t="s">
         <v>18</v>
@@ -25514,10 +25556,10 @@
         <v>1158</v>
       </c>
       <c r="B645" t="s">
-        <v>1231</v>
+        <v>1222</v>
       </c>
       <c r="D645" t="s">
-        <v>1232</v>
+        <v>1223</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25587,7 +25629,7 @@
         <v>1160</v>
       </c>
       <c r="B647" t="s">
-        <v>1225</v>
+        <v>1216</v>
       </c>
       <c r="D647" t="s">
         <v>55</v>
@@ -25660,7 +25702,7 @@
         <v>1163</v>
       </c>
       <c r="B649" t="s">
-        <v>1233</v>
+        <v>1224</v>
       </c>
       <c r="D649" t="s">
         <v>362</v>
@@ -25686,10 +25728,10 @@
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1236</v>
+        <v>1226</v>
       </c>
       <c r="B650" t="s">
-        <v>1237</v>
+        <v>1227</v>
       </c>
       <c r="D650" t="s">
         <v>190</v>
@@ -25715,10 +25757,10 @@
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1236</v>
+        <v>1226</v>
       </c>
       <c r="B651" t="s">
-        <v>1238</v>
+        <v>1228</v>
       </c>
       <c r="D651" t="s">
         <v>34</v>
@@ -25744,7 +25786,7 @@
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1226</v>
+        <v>1217</v>
       </c>
       <c r="B652" t="s">
         <v>397</v>
@@ -25832,10 +25874,10 @@
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1239</v>
+        <v>1229</v>
       </c>
       <c r="B654" t="s">
-        <v>1240</v>
+        <v>1230</v>
       </c>
       <c r="D654" t="s">
         <v>362</v>
@@ -25861,10 +25903,10 @@
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1222</v>
+        <v>1213</v>
       </c>
       <c r="B655" t="s">
-        <v>1223</v>
+        <v>1214</v>
       </c>
       <c r="D655" t="s">
         <v>34</v>
@@ -25890,16 +25932,31 @@
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1222</v>
+        <v>1213</v>
       </c>
       <c r="B656" t="s">
-        <v>1248</v>
+        <v>1238</v>
       </c>
       <c r="D656" t="s">
-        <v>1249</v>
+        <v>1239</v>
       </c>
       <c r="E656" t="s">
         <v>19</v>
+      </c>
+      <c r="F656">
+        <v>0</v>
+      </c>
+      <c r="G656">
+        <v>0</v>
+      </c>
+      <c r="H656">
+        <v>0</v>
+      </c>
+      <c r="I656">
+        <v>0</v>
+      </c>
+      <c r="J656">
+        <v>0</v>
       </c>
       <c r="K656" t="s">
         <v>20</v>
@@ -25919,16 +25976,31 @@
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1241</v>
+        <v>1231</v>
       </c>
       <c r="B657" t="s">
-        <v>1242</v>
+        <v>1232</v>
       </c>
       <c r="D657" t="s">
-        <v>1243</v>
+        <v>1233</v>
       </c>
       <c r="E657" t="s">
         <v>19</v>
+      </c>
+      <c r="F657">
+        <v>0</v>
+      </c>
+      <c r="G657">
+        <v>0</v>
+      </c>
+      <c r="H657">
+        <v>0</v>
+      </c>
+      <c r="I657">
+        <v>0</v>
+      </c>
+      <c r="J657">
+        <v>0</v>
       </c>
       <c r="K657" t="s">
         <v>20</v>
@@ -25945,10 +26017,10 @@
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1250</v>
+        <v>1240</v>
       </c>
       <c r="B658" t="s">
-        <v>1251</v>
+        <v>1241</v>
       </c>
       <c r="D658" t="s">
         <v>60</v>
@@ -25985,6 +26057,21 @@
       <c r="E659" t="s">
         <v>19</v>
       </c>
+      <c r="F659">
+        <v>37</v>
+      </c>
+      <c r="G659">
+        <v>0</v>
+      </c>
+      <c r="H659">
+        <v>0</v>
+      </c>
+      <c r="I659">
+        <v>0</v>
+      </c>
+      <c r="J659">
+        <v>0</v>
+      </c>
       <c r="K659" t="s">
         <v>20</v>
       </c>
@@ -25995,10 +26082,10 @@
         <v>10</v>
       </c>
       <c r="N659">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O659">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
@@ -26012,7 +26099,22 @@
         <v>1169</v>
       </c>
       <c r="E660" t="s">
-        <v>187</v>
+        <v>19</v>
+      </c>
+      <c r="F660">
+        <v>14</v>
+      </c>
+      <c r="G660">
+        <v>0</v>
+      </c>
+      <c r="H660">
+        <v>0</v>
+      </c>
+      <c r="I660">
+        <v>0</v>
+      </c>
+      <c r="J660">
+        <v>0</v>
       </c>
       <c r="K660" t="s">
         <v>20</v>
@@ -26024,10 +26126,10 @@
         <v>9</v>
       </c>
       <c r="N660">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O660">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
@@ -26043,6 +26145,21 @@
       <c r="E661" t="s">
         <v>19</v>
       </c>
+      <c r="F661">
+        <v>0</v>
+      </c>
+      <c r="G661">
+        <v>0</v>
+      </c>
+      <c r="H661">
+        <v>0</v>
+      </c>
+      <c r="I661">
+        <v>0</v>
+      </c>
+      <c r="J661">
+        <v>0</v>
+      </c>
       <c r="K661" t="s">
         <v>20</v>
       </c>
@@ -26061,16 +26178,31 @@
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1244</v>
+        <v>1234</v>
       </c>
       <c r="B662" t="s">
-        <v>1245</v>
+        <v>1235</v>
       </c>
       <c r="D662" t="s">
-        <v>1246</v>
+        <v>1236</v>
       </c>
       <c r="E662" t="s">
         <v>19</v>
+      </c>
+      <c r="F662">
+        <v>1</v>
+      </c>
+      <c r="G662">
+        <v>0</v>
+      </c>
+      <c r="H662">
+        <v>0</v>
+      </c>
+      <c r="I662">
+        <v>0</v>
+      </c>
+      <c r="J662">
+        <v>0</v>
       </c>
       <c r="K662" t="s">
         <v>20</v>
@@ -26099,7 +26231,7 @@
         <v>34</v>
       </c>
       <c r="E663" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K663" t="s">
         <v>20</v>
@@ -26108,13 +26240,13 @@
         <v>21</v>
       </c>
       <c r="M663">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="N663">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O663">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
@@ -26128,7 +26260,22 @@
         <v>205</v>
       </c>
       <c r="E664" t="s">
-        <v>187</v>
+        <v>19</v>
+      </c>
+      <c r="F664">
+        <v>10</v>
+      </c>
+      <c r="G664">
+        <v>0</v>
+      </c>
+      <c r="H664">
+        <v>0</v>
+      </c>
+      <c r="I664">
+        <v>0</v>
+      </c>
+      <c r="J664">
+        <v>0</v>
       </c>
       <c r="K664" t="s">
         <v>20</v>
@@ -26157,7 +26304,7 @@
         <v>34</v>
       </c>
       <c r="E665" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K665" t="s">
         <v>20</v>
@@ -26169,10 +26316,10 @@
         <v>6</v>
       </c>
       <c r="N665">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O665">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="666" spans="1:15" x14ac:dyDescent="0.35">
@@ -26180,13 +26327,28 @@
         <v>1175</v>
       </c>
       <c r="B666" t="s">
-        <v>1247</v>
+        <v>1237</v>
       </c>
       <c r="D666" t="s">
         <v>583</v>
       </c>
       <c r="E666" t="s">
-        <v>187</v>
+        <v>19</v>
+      </c>
+      <c r="F666">
+        <v>0</v>
+      </c>
+      <c r="G666">
+        <v>0</v>
+      </c>
+      <c r="H666">
+        <v>0</v>
+      </c>
+      <c r="I666">
+        <v>0</v>
+      </c>
+      <c r="J666">
+        <v>0</v>
       </c>
       <c r="K666" t="s">
         <v>20</v>
@@ -26195,39 +26357,42 @@
         <v>21</v>
       </c>
       <c r="M666">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="N666">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="O666">
+        <v>47.5</v>
       </c>
     </row>
     <row r="667" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>1177</v>
+        <v>1247</v>
       </c>
       <c r="B667" t="s">
-        <v>1219</v>
+        <v>1248</v>
       </c>
       <c r="D667" t="s">
-        <v>1220</v>
+        <v>60</v>
       </c>
       <c r="E667" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K667" t="s">
         <v>20</v>
       </c>
       <c r="L667" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M667">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="N667">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="O667">
-        <v>48</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="668" spans="1:15" x14ac:dyDescent="0.35">
@@ -26235,13 +26400,28 @@
         <v>1177</v>
       </c>
       <c r="B668" t="s">
-        <v>1227</v>
+        <v>1218</v>
       </c>
       <c r="D668" t="s">
         <v>202</v>
       </c>
       <c r="E668" t="s">
-        <v>187</v>
+        <v>19</v>
+      </c>
+      <c r="F668">
+        <v>19</v>
+      </c>
+      <c r="G668">
+        <v>0</v>
+      </c>
+      <c r="H668">
+        <v>0</v>
+      </c>
+      <c r="I668">
+        <v>1</v>
+      </c>
+      <c r="J668">
+        <v>0</v>
       </c>
       <c r="K668" t="s">
         <v>20</v>
@@ -26253,10 +26433,10 @@
         <v>8</v>
       </c>
       <c r="N668">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O668">
-        <v>24</v>
+        <v>72</v>
       </c>
     </row>
     <row r="669" spans="1:15" x14ac:dyDescent="0.35">
@@ -26264,13 +26444,28 @@
         <v>1177</v>
       </c>
       <c r="B669" t="s">
-        <v>1234</v>
+        <v>1249</v>
       </c>
       <c r="D669" t="s">
-        <v>1235</v>
+        <v>1225</v>
       </c>
       <c r="E669" t="s">
-        <v>187</v>
+        <v>19</v>
+      </c>
+      <c r="F669">
+        <v>0</v>
+      </c>
+      <c r="G669">
+        <v>0</v>
+      </c>
+      <c r="H669">
+        <v>0</v>
+      </c>
+      <c r="I669">
+        <v>0</v>
+      </c>
+      <c r="J669">
+        <v>0</v>
       </c>
       <c r="K669" t="s">
         <v>20</v>
@@ -26279,140 +26474,143 @@
         <v>25</v>
       </c>
       <c r="M669">
-        <v>10.5</v>
+        <v>13</v>
       </c>
       <c r="N669">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O669">
+        <v>21</v>
       </c>
     </row>
     <row r="670" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A670" t="s">
-        <v>1252</v>
+        <v>1250</v>
       </c>
       <c r="B670" t="s">
-        <v>770</v>
+        <v>1251</v>
       </c>
       <c r="D670" t="s">
-        <v>771</v>
+        <v>60</v>
       </c>
       <c r="E670" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K670" t="s">
         <v>20</v>
       </c>
       <c r="L670" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M670">
-        <v>3</v>
+        <v>6.75</v>
       </c>
       <c r="N670">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O670">
-        <v>6</v>
+        <v>27</v>
       </c>
     </row>
     <row r="671" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A671" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="B671" t="s">
-        <v>1179</v>
+        <v>1253</v>
       </c>
       <c r="D671" t="s">
-        <v>1180</v>
+        <v>362</v>
       </c>
       <c r="E671" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K671" t="s">
         <v>20</v>
       </c>
       <c r="L671" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M671">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="N671">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="O671">
-        <v>60</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="672" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A672" t="s">
-        <v>1178</v>
+        <v>1242</v>
       </c>
       <c r="B672" t="s">
-        <v>1181</v>
+        <v>770</v>
       </c>
       <c r="D672" t="s">
-        <v>1180</v>
+        <v>771</v>
       </c>
       <c r="E672" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K672" t="s">
         <v>20</v>
       </c>
       <c r="L672" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M672">
+        <v>3.5</v>
+      </c>
+      <c r="N672">
+        <v>2</v>
+      </c>
+      <c r="O672">
         <v>7</v>
-      </c>
-      <c r="N672">
-        <v>19</v>
-      </c>
-      <c r="O672">
-        <v>133</v>
       </c>
     </row>
     <row r="673" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A673" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B673" t="s">
-        <v>1183</v>
+        <v>1254</v>
       </c>
       <c r="D673" t="s">
-        <v>1180</v>
+        <v>663</v>
       </c>
       <c r="E673" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K673" t="s">
         <v>20</v>
       </c>
       <c r="L673" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M673">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="N673">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="O673">
-        <v>176</v>
+        <v>96</v>
       </c>
     </row>
     <row r="674" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A674" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B674" t="s">
-        <v>1184</v>
+        <v>1255</v>
       </c>
       <c r="D674" t="s">
-        <v>18</v>
+        <v>663</v>
       </c>
       <c r="E674" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K674" t="s">
         <v>20</v>
@@ -26421,24 +26619,24 @@
         <v>21</v>
       </c>
       <c r="M674">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="N674">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O674">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="675" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A675" t="s">
-        <v>1182</v>
+        <v>1179</v>
       </c>
       <c r="B675" t="s">
-        <v>1185</v>
+        <v>1180</v>
       </c>
       <c r="D675" t="s">
-        <v>1186</v>
+        <v>1181</v>
       </c>
       <c r="E675" t="s">
         <v>19</v>
@@ -26458,42 +26656,42 @@
     </row>
     <row r="676" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A676" t="s">
-        <v>1187</v>
+        <v>1179</v>
       </c>
       <c r="B676" t="s">
-        <v>1188</v>
+        <v>1256</v>
       </c>
       <c r="D676" t="s">
-        <v>1180</v>
+        <v>663</v>
       </c>
       <c r="E676" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K676" t="s">
         <v>20</v>
       </c>
       <c r="L676" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M676">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="N676">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="O676">
-        <v>165</v>
+        <v>64</v>
       </c>
     </row>
     <row r="677" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A677" t="s">
-        <v>1187</v>
+        <v>1179</v>
       </c>
       <c r="B677" t="s">
-        <v>1189</v>
+        <v>1257</v>
       </c>
       <c r="D677" t="s">
-        <v>1186</v>
+        <v>663</v>
       </c>
       <c r="E677" t="s">
         <v>19</v>
@@ -26505,21 +26703,24 @@
         <v>21</v>
       </c>
       <c r="M677">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="N677">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="O677">
+        <v>64</v>
       </c>
     </row>
     <row r="678" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A678" t="s">
-        <v>1190</v>
+        <v>1182</v>
       </c>
       <c r="B678" t="s">
-        <v>1191</v>
+        <v>1183</v>
       </c>
       <c r="D678" t="s">
-        <v>1192</v>
+        <v>1181</v>
       </c>
       <c r="E678" t="s">
         <v>19</v>
@@ -26531,7 +26732,7 @@
         <v>21</v>
       </c>
       <c r="M678">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N678">
         <v>0</v>
@@ -26539,13 +26740,13 @@
     </row>
     <row r="679" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A679" t="s">
-        <v>1193</v>
+        <v>1182</v>
       </c>
       <c r="B679" t="s">
-        <v>1194</v>
+        <v>1258</v>
       </c>
       <c r="D679" t="s">
-        <v>1195</v>
+        <v>663</v>
       </c>
       <c r="E679" t="s">
         <v>19</v>
@@ -26557,53 +26758,56 @@
         <v>21</v>
       </c>
       <c r="M679">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="N679">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="O679">
+        <v>44</v>
       </c>
     </row>
     <row r="680" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A680" t="s">
-        <v>1253</v>
+        <v>1182</v>
       </c>
       <c r="B680" t="s">
-        <v>1254</v>
+        <v>1259</v>
       </c>
       <c r="D680" t="s">
-        <v>345</v>
+        <v>663</v>
       </c>
       <c r="E680" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K680" t="s">
         <v>20</v>
       </c>
       <c r="L680" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M680">
-        <v>2.75</v>
+        <v>11</v>
       </c>
       <c r="N680">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O680">
-        <v>2.75</v>
+        <v>44</v>
       </c>
     </row>
     <row r="681" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A681" t="s">
-        <v>1196</v>
+        <v>1182</v>
       </c>
       <c r="B681" t="s">
-        <v>1197</v>
+        <v>1260</v>
       </c>
       <c r="D681" t="s">
-        <v>1198</v>
+        <v>663</v>
       </c>
       <c r="E681" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K681" t="s">
         <v>20</v>
@@ -26612,24 +26816,24 @@
         <v>21</v>
       </c>
       <c r="M681">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="N681">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="O681">
-        <v>363</v>
+        <v>44</v>
       </c>
     </row>
     <row r="682" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A682" t="s">
-        <v>1196</v>
+        <v>1184</v>
       </c>
       <c r="B682" t="s">
-        <v>1199</v>
+        <v>1185</v>
       </c>
       <c r="D682" t="s">
-        <v>228</v>
+        <v>1186</v>
       </c>
       <c r="E682" t="s">
         <v>19</v>
@@ -26641,7 +26845,7 @@
         <v>21</v>
       </c>
       <c r="M682">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="N682">
         <v>0</v>
@@ -26649,39 +26853,42 @@
     </row>
     <row r="683" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A683" t="s">
-        <v>1200</v>
+        <v>1261</v>
       </c>
       <c r="B683" t="s">
-        <v>1201</v>
+        <v>1262</v>
       </c>
       <c r="D683" t="s">
-        <v>1202</v>
+        <v>1263</v>
       </c>
       <c r="E683" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K683" t="s">
         <v>20</v>
       </c>
       <c r="L683" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M683">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="N683">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="O683">
+        <v>2.5</v>
       </c>
     </row>
     <row r="684" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A684" t="s">
-        <v>1200</v>
+        <v>1187</v>
       </c>
       <c r="B684" t="s">
-        <v>1201</v>
+        <v>1188</v>
       </c>
       <c r="D684" t="s">
-        <v>1203</v>
+        <v>1189</v>
       </c>
       <c r="E684" t="s">
         <v>19</v>
@@ -26701,65 +26908,71 @@
     </row>
     <row r="685" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A685" t="s">
-        <v>1200</v>
+        <v>1243</v>
       </c>
       <c r="B685" t="s">
-        <v>1201</v>
+        <v>1244</v>
       </c>
       <c r="D685" t="s">
-        <v>1204</v>
+        <v>345</v>
       </c>
       <c r="E685" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K685" t="s">
         <v>20</v>
       </c>
       <c r="L685" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M685">
-        <v>1.5</v>
+        <v>2.75</v>
       </c>
       <c r="N685">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O685">
+        <v>5.5</v>
       </c>
     </row>
     <row r="686" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A686" t="s">
-        <v>1200</v>
+        <v>1264</v>
       </c>
       <c r="B686" t="s">
-        <v>1201</v>
+        <v>1265</v>
       </c>
       <c r="D686" t="s">
-        <v>1205</v>
+        <v>1266</v>
       </c>
       <c r="E686" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K686" t="s">
         <v>20</v>
       </c>
       <c r="L686" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M686">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N686">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="O686">
+        <v>6</v>
       </c>
     </row>
     <row r="687" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A687" t="s">
-        <v>1200</v>
+        <v>1264</v>
       </c>
       <c r="B687" t="s">
-        <v>1255</v>
+        <v>316</v>
       </c>
       <c r="D687" t="s">
-        <v>1256</v>
+        <v>18</v>
       </c>
       <c r="E687" t="s">
         <v>187</v>
@@ -26768,24 +26981,27 @@
         <v>20</v>
       </c>
       <c r="L687" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M687">
-        <v>4</v>
+        <v>3.25</v>
       </c>
       <c r="N687">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="O687">
+        <v>3.25</v>
       </c>
     </row>
     <row r="688" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A688" t="s">
-        <v>1206</v>
+        <v>1190</v>
       </c>
       <c r="B688" t="s">
-        <v>1207</v>
+        <v>1191</v>
       </c>
       <c r="D688" t="s">
-        <v>1208</v>
+        <v>1192</v>
       </c>
       <c r="E688" t="s">
         <v>187</v>
@@ -26794,16 +27010,259 @@
         <v>20</v>
       </c>
       <c r="L688" t="s">
+        <v>21</v>
+      </c>
+      <c r="M688">
+        <v>33</v>
+      </c>
+      <c r="N688">
+        <v>13</v>
+      </c>
+      <c r="O688">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="689" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A689" t="s">
+        <v>1190</v>
+      </c>
+      <c r="B689" t="s">
+        <v>1193</v>
+      </c>
+      <c r="D689" t="s">
+        <v>228</v>
+      </c>
+      <c r="E689" t="s">
+        <v>19</v>
+      </c>
+      <c r="K689" t="s">
+        <v>20</v>
+      </c>
+      <c r="L689" t="s">
+        <v>21</v>
+      </c>
+      <c r="M689">
+        <v>11</v>
+      </c>
+      <c r="N689">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="690" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A690" t="s">
+        <v>1267</v>
+      </c>
+      <c r="B690" t="s">
+        <v>421</v>
+      </c>
+      <c r="D690" t="s">
+        <v>18</v>
+      </c>
+      <c r="E690" t="s">
+        <v>187</v>
+      </c>
+      <c r="K690" t="s">
+        <v>20</v>
+      </c>
+      <c r="L690" t="s">
+        <v>21</v>
+      </c>
+      <c r="M690">
+        <v>6.02</v>
+      </c>
+      <c r="N690">
+        <v>1</v>
+      </c>
+      <c r="O690">
+        <v>6.0199999809265003</v>
+      </c>
+    </row>
+    <row r="691" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A691" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B691" t="s">
+        <v>1269</v>
+      </c>
+      <c r="D691" t="s">
+        <v>18</v>
+      </c>
+      <c r="E691" t="s">
+        <v>187</v>
+      </c>
+      <c r="K691" t="s">
+        <v>20</v>
+      </c>
+      <c r="L691" t="s">
+        <v>21</v>
+      </c>
+      <c r="M691">
+        <v>7</v>
+      </c>
+      <c r="N691">
+        <v>1</v>
+      </c>
+      <c r="O691">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="692" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A692" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B692" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D692" t="s">
+        <v>1196</v>
+      </c>
+      <c r="E692" t="s">
+        <v>19</v>
+      </c>
+      <c r="K692" t="s">
+        <v>20</v>
+      </c>
+      <c r="L692" t="s">
+        <v>21</v>
+      </c>
+      <c r="M692">
+        <v>3</v>
+      </c>
+      <c r="N692">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A693" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B693" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D693" t="s">
+        <v>1197</v>
+      </c>
+      <c r="E693" t="s">
+        <v>19</v>
+      </c>
+      <c r="K693" t="s">
+        <v>20</v>
+      </c>
+      <c r="L693" t="s">
+        <v>21</v>
+      </c>
+      <c r="M693">
+        <v>3</v>
+      </c>
+      <c r="N693">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="694" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A694" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B694" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D694" t="s">
+        <v>1198</v>
+      </c>
+      <c r="E694" t="s">
+        <v>19</v>
+      </c>
+      <c r="K694" t="s">
+        <v>20</v>
+      </c>
+      <c r="L694" t="s">
+        <v>21</v>
+      </c>
+      <c r="M694">
+        <v>1.5</v>
+      </c>
+      <c r="N694">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="695" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A695" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B695" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D695" t="s">
+        <v>1199</v>
+      </c>
+      <c r="E695" t="s">
+        <v>19</v>
+      </c>
+      <c r="K695" t="s">
+        <v>20</v>
+      </c>
+      <c r="L695" t="s">
+        <v>21</v>
+      </c>
+      <c r="M695">
+        <v>4</v>
+      </c>
+      <c r="N695">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="696" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A696" t="s">
+        <v>1194</v>
+      </c>
+      <c r="B696" t="s">
+        <v>1245</v>
+      </c>
+      <c r="D696" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E696" t="s">
+        <v>187</v>
+      </c>
+      <c r="K696" t="s">
+        <v>20</v>
+      </c>
+      <c r="L696" t="s">
+        <v>25</v>
+      </c>
+      <c r="M696">
+        <v>4</v>
+      </c>
+      <c r="N696">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="697" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A697" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B697" t="s">
+        <v>1270</v>
+      </c>
+      <c r="D697" t="s">
+        <v>1201</v>
+      </c>
+      <c r="E697" t="s">
+        <v>19</v>
+      </c>
+      <c r="K697" t="s">
+        <v>20</v>
+      </c>
+      <c r="L697" t="s">
         <v>75</v>
       </c>
-      <c r="M688">
+      <c r="M697">
         <v>120</v>
       </c>
-      <c r="N688">
-        <v>5</v>
-      </c>
-      <c r="O688">
-        <v>600</v>
+      <c r="N697">
+        <v>4</v>
+      </c>
+      <c r="O697">
+        <v>480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mise à jour DPS — 08/07/2026
</commit_message>
<xml_diff>
--- a/data/export_dps.xlsx
+++ b/data/export_dps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haithem.aloui\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D422330-40F1-4862-B67A-03482AF5134F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD86106-8C8E-4267-8602-255426BD8C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,11 +19,24 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Statistiques dactivites  Di'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4194" uniqueCount="1271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4200" uniqueCount="1274">
   <si>
     <t>Début</t>
   </si>
@@ -3559,24 +3572,6 @@
     <t>21-06-2026</t>
   </si>
   <si>
-    <t>26-06-2026</t>
-  </si>
-  <si>
-    <t>27-06-2026</t>
-  </si>
-  <si>
-    <t>FestiMarne 2026 - J1</t>
-  </si>
-  <si>
-    <t>Marne</t>
-  </si>
-  <si>
-    <t>28-06-2026</t>
-  </si>
-  <si>
-    <t>FestiMarne 2026 - J2</t>
-  </si>
-  <si>
     <t>29-06-2026</t>
   </si>
   <si>
@@ -3589,21 +3584,9 @@
     <t>01-07-2026</t>
   </si>
   <si>
-    <t>Spectacle sur l'eau</t>
-  </si>
-  <si>
-    <t>Canal de l'ourcq</t>
-  </si>
-  <si>
     <t>04-07-2026</t>
   </si>
   <si>
-    <t>Company Cup 2026</t>
-  </si>
-  <si>
-    <t>Annecy</t>
-  </si>
-  <si>
     <t xml:space="preserve">Renfort Compagny Cup </t>
   </si>
   <si>
@@ -3622,15 +3605,6 @@
     <t>Triel Sur Seine</t>
   </si>
   <si>
-    <t xml:space="preserve"> Bonneuil-sur-Marne</t>
-  </si>
-  <si>
-    <t>15-07-2026</t>
-  </si>
-  <si>
-    <t>Carhaix (29)</t>
-  </si>
-  <si>
     <t>Renfort DPS-ME - Rocket League Paris Major 2 (J3)</t>
   </si>
   <si>
@@ -3760,9 +3734,6 @@
     <t>Olympiades du groupe AFD</t>
   </si>
   <si>
-    <t xml:space="preserve">Feu dartifice </t>
-  </si>
-  <si>
     <t>Alfortville</t>
   </si>
   <si>
@@ -3787,27 +3758,6 @@
     <t>Renfort PlayOff - Final J5</t>
   </si>
   <si>
-    <t>Renfort Solidays J1 - PSA Paris 2</t>
-  </si>
-  <si>
-    <t>Renfort Solidays J1 - VPS</t>
-  </si>
-  <si>
-    <t>Renfort Solidays J2 - PSA Cesar Circus</t>
-  </si>
-  <si>
-    <t>Renfort Solidays J2 - VPS</t>
-  </si>
-  <si>
-    <t>Renfort Solidays J3 - PSA Paris 1</t>
-  </si>
-  <si>
-    <t>Renfort Solidays J3 - VPS A</t>
-  </si>
-  <si>
-    <t>Renfort Solidays J3 - VPS B</t>
-  </si>
-  <si>
     <t>30-06-2026</t>
   </si>
   <si>
@@ -3835,7 +3785,79 @@
     <t>Course Copenhague-Paris 2026</t>
   </si>
   <si>
-    <t>Vieilles Charrues 2026</t>
+    <t>Renfort Spectacle EDGAR-YVES JR - J1</t>
+  </si>
+  <si>
+    <t>Renfort Concert ROBYN</t>
+  </si>
+  <si>
+    <t>05-07-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME  - Concert  Bad Bunny</t>
+  </si>
+  <si>
+    <t>06-07-2026</t>
+  </si>
+  <si>
+    <t>Défilé DIOR Haute Couture - VPS EVAC</t>
+  </si>
+  <si>
+    <t>Renfort Défilé DIOR Haute Couture - PAPS</t>
+  </si>
+  <si>
+    <t>07-07-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Concert Luke Combs</t>
+  </si>
+  <si>
+    <t>08-07-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Concert Def Leppard</t>
+  </si>
+  <si>
+    <t>09-07-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Concert Vulpeck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feu dartifice alfortville  </t>
+  </si>
+  <si>
+    <t>14-07-2026</t>
+  </si>
+  <si>
+    <t>Renfort Revue militaire - 14 juillet</t>
+  </si>
+  <si>
+    <t>19-07-2026</t>
+  </si>
+  <si>
+    <t>Renfort DPS-ME - Concert Romeo Santos &amp; Prince Royce</t>
+  </si>
+  <si>
+    <t>26-07-2026</t>
+  </si>
+  <si>
+    <t>Bel été 2026</t>
+  </si>
+  <si>
+    <t>La Courneuve - Parc Georg</t>
+  </si>
+  <si>
+    <t>Fête foraine des Tuileries</t>
+  </si>
+  <si>
+    <t>14-10-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Course scolaire UNSS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forêt de Bondy </t>
   </si>
 </sst>
 </file>
@@ -4190,7 +4212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P697"/>
+  <dimension ref="A1:P698"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
@@ -25002,7 +25024,7 @@
         <v>1149</v>
       </c>
       <c r="B629" t="s">
-        <v>1204</v>
+        <v>1191</v>
       </c>
       <c r="D629" t="s">
         <v>34</v>
@@ -25031,10 +25053,10 @@
         <v>1149</v>
       </c>
       <c r="B630" t="s">
-        <v>1205</v>
+        <v>1192</v>
       </c>
       <c r="D630" t="s">
-        <v>1206</v>
+        <v>1193</v>
       </c>
       <c r="E630" t="s">
         <v>19</v>
@@ -25148,7 +25170,7 @@
         <v>1150</v>
       </c>
       <c r="B633" t="s">
-        <v>1202</v>
+        <v>1189</v>
       </c>
       <c r="D633" t="s">
         <v>60</v>
@@ -25174,13 +25196,13 @@
     </row>
     <row r="634" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A634" t="s">
-        <v>1211</v>
+        <v>1198</v>
       </c>
       <c r="B634" t="s">
-        <v>1210</v>
+        <v>1197</v>
       </c>
       <c r="D634" t="s">
-        <v>1209</v>
+        <v>1196</v>
       </c>
       <c r="E634" t="s">
         <v>19</v>
@@ -25294,10 +25316,10 @@
         <v>1153</v>
       </c>
       <c r="B637" t="s">
-        <v>1208</v>
+        <v>1195</v>
       </c>
       <c r="D637" t="s">
-        <v>1207</v>
+        <v>1194</v>
       </c>
       <c r="E637" t="s">
         <v>19</v>
@@ -25338,10 +25360,10 @@
         <v>1153</v>
       </c>
       <c r="B638" t="s">
-        <v>1215</v>
+        <v>1202</v>
       </c>
       <c r="D638" t="s">
-        <v>1209</v>
+        <v>1196</v>
       </c>
       <c r="E638" t="s">
         <v>19</v>
@@ -25367,7 +25389,7 @@
         <v>1155</v>
       </c>
       <c r="B639" t="s">
-        <v>1203</v>
+        <v>1190</v>
       </c>
       <c r="D639" t="s">
         <v>60</v>
@@ -25469,7 +25491,7 @@
         <v>1158</v>
       </c>
       <c r="B642" t="s">
-        <v>1212</v>
+        <v>1199</v>
       </c>
       <c r="D642" t="s">
         <v>34</v>
@@ -25498,10 +25520,10 @@
         <v>1158</v>
       </c>
       <c r="B643" t="s">
-        <v>1219</v>
+        <v>1206</v>
       </c>
       <c r="D643" t="s">
-        <v>1220</v>
+        <v>1207</v>
       </c>
       <c r="E643" t="s">
         <v>19</v>
@@ -25527,7 +25549,7 @@
         <v>1158</v>
       </c>
       <c r="B644" t="s">
-        <v>1221</v>
+        <v>1208</v>
       </c>
       <c r="D644" t="s">
         <v>18</v>
@@ -25556,10 +25578,10 @@
         <v>1158</v>
       </c>
       <c r="B645" t="s">
-        <v>1222</v>
+        <v>1209</v>
       </c>
       <c r="D645" t="s">
-        <v>1223</v>
+        <v>1210</v>
       </c>
       <c r="E645" t="s">
         <v>187</v>
@@ -25629,7 +25651,7 @@
         <v>1160</v>
       </c>
       <c r="B647" t="s">
-        <v>1216</v>
+        <v>1203</v>
       </c>
       <c r="D647" t="s">
         <v>55</v>
@@ -25702,7 +25724,7 @@
         <v>1163</v>
       </c>
       <c r="B649" t="s">
-        <v>1224</v>
+        <v>1211</v>
       </c>
       <c r="D649" t="s">
         <v>362</v>
@@ -25728,10 +25750,10 @@
     </row>
     <row r="650" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
-        <v>1226</v>
+        <v>1213</v>
       </c>
       <c r="B650" t="s">
-        <v>1227</v>
+        <v>1214</v>
       </c>
       <c r="D650" t="s">
         <v>190</v>
@@ -25757,10 +25779,10 @@
     </row>
     <row r="651" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
-        <v>1226</v>
+        <v>1213</v>
       </c>
       <c r="B651" t="s">
-        <v>1228</v>
+        <v>1215</v>
       </c>
       <c r="D651" t="s">
         <v>34</v>
@@ -25786,7 +25808,7 @@
     </row>
     <row r="652" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
-        <v>1217</v>
+        <v>1204</v>
       </c>
       <c r="B652" t="s">
         <v>397</v>
@@ -25874,10 +25896,10 @@
     </row>
     <row r="654" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
-        <v>1229</v>
+        <v>1216</v>
       </c>
       <c r="B654" t="s">
-        <v>1230</v>
+        <v>1217</v>
       </c>
       <c r="D654" t="s">
         <v>362</v>
@@ -25903,10 +25925,10 @@
     </row>
     <row r="655" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
-        <v>1213</v>
+        <v>1200</v>
       </c>
       <c r="B655" t="s">
-        <v>1214</v>
+        <v>1201</v>
       </c>
       <c r="D655" t="s">
         <v>34</v>
@@ -25932,13 +25954,13 @@
     </row>
     <row r="656" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
-        <v>1213</v>
+        <v>1200</v>
       </c>
       <c r="B656" t="s">
-        <v>1238</v>
+        <v>1225</v>
       </c>
       <c r="D656" t="s">
-        <v>1239</v>
+        <v>1226</v>
       </c>
       <c r="E656" t="s">
         <v>19</v>
@@ -25976,13 +25998,13 @@
     </row>
     <row r="657" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A657" t="s">
-        <v>1231</v>
+        <v>1218</v>
       </c>
       <c r="B657" t="s">
-        <v>1232</v>
+        <v>1219</v>
       </c>
       <c r="D657" t="s">
-        <v>1233</v>
+        <v>1220</v>
       </c>
       <c r="E657" t="s">
         <v>19</v>
@@ -26017,10 +26039,10 @@
     </row>
     <row r="658" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A658" t="s">
-        <v>1240</v>
+        <v>1227</v>
       </c>
       <c r="B658" t="s">
-        <v>1241</v>
+        <v>1228</v>
       </c>
       <c r="D658" t="s">
         <v>60</v>
@@ -26046,54 +26068,39 @@
     </row>
     <row r="659" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A659" t="s">
-        <v>1168</v>
+        <v>1227</v>
       </c>
       <c r="B659" t="s">
-        <v>775</v>
+        <v>1249</v>
       </c>
       <c r="D659" t="s">
-        <v>1169</v>
+        <v>362</v>
       </c>
       <c r="E659" t="s">
         <v>19</v>
       </c>
-      <c r="F659">
-        <v>37</v>
-      </c>
-      <c r="G659">
-        <v>0</v>
-      </c>
-      <c r="H659">
-        <v>0</v>
-      </c>
-      <c r="I659">
-        <v>0</v>
-      </c>
-      <c r="J659">
-        <v>0</v>
-      </c>
       <c r="K659" t="s">
         <v>20</v>
       </c>
       <c r="L659" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="M659">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N659">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="O659">
-        <v>136</v>
+        <v>5</v>
       </c>
     </row>
     <row r="660" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A660" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="B660" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D660" t="s">
         <v>1169</v>
@@ -26102,7 +26109,7 @@
         <v>19</v>
       </c>
       <c r="F660">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G660">
         <v>0</v>
@@ -26123,13 +26130,13 @@
         <v>50</v>
       </c>
       <c r="M660">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N660">
         <v>14</v>
       </c>
       <c r="O660">
-        <v>111</v>
+        <v>136</v>
       </c>
     </row>
     <row r="661" spans="1:15" x14ac:dyDescent="0.35">
@@ -26137,16 +26144,16 @@
         <v>1170</v>
       </c>
       <c r="B661" t="s">
-        <v>643</v>
+        <v>777</v>
       </c>
       <c r="D661" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="E661" t="s">
         <v>19</v>
       </c>
       <c r="F661">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G661">
         <v>0</v>
@@ -26164,33 +26171,33 @@
         <v>20</v>
       </c>
       <c r="L661" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="M661">
-        <v>8.25</v>
+        <v>9</v>
       </c>
       <c r="N661">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="O661">
-        <v>16.5</v>
+        <v>111</v>
       </c>
     </row>
     <row r="662" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A662" t="s">
-        <v>1234</v>
+        <v>1170</v>
       </c>
       <c r="B662" t="s">
-        <v>1235</v>
+        <v>643</v>
       </c>
       <c r="D662" t="s">
-        <v>1236</v>
+        <v>1171</v>
       </c>
       <c r="E662" t="s">
         <v>19</v>
       </c>
       <c r="F662">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G662">
         <v>0</v>
@@ -26208,30 +26215,45 @@
         <v>20</v>
       </c>
       <c r="L662" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M662">
-        <v>5.5</v>
+        <v>8.25</v>
       </c>
       <c r="N662">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O662">
-        <v>27.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="663" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A663" t="s">
-        <v>1172</v>
+        <v>1221</v>
       </c>
       <c r="B663" t="s">
-        <v>546</v>
+        <v>1222</v>
       </c>
       <c r="D663" t="s">
-        <v>34</v>
+        <v>1223</v>
       </c>
       <c r="E663" t="s">
         <v>19</v>
+      </c>
+      <c r="F663">
+        <v>1</v>
+      </c>
+      <c r="G663">
+        <v>0</v>
+      </c>
+      <c r="H663">
+        <v>0</v>
+      </c>
+      <c r="I663">
+        <v>0</v>
+      </c>
+      <c r="J663">
+        <v>0</v>
       </c>
       <c r="K663" t="s">
         <v>20</v>
@@ -26243,40 +26265,25 @@
         <v>5.5</v>
       </c>
       <c r="N663">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O663">
-        <v>22</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="664" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A664" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B664" t="s">
-        <v>1174</v>
+        <v>546</v>
       </c>
       <c r="D664" t="s">
-        <v>205</v>
+        <v>34</v>
       </c>
       <c r="E664" t="s">
         <v>19</v>
       </c>
-      <c r="F664">
-        <v>10</v>
-      </c>
-      <c r="G664">
-        <v>0</v>
-      </c>
-      <c r="H664">
-        <v>0</v>
-      </c>
-      <c r="I664">
-        <v>0</v>
-      </c>
-      <c r="J664">
-        <v>0</v>
-      </c>
       <c r="K664" t="s">
         <v>20</v>
       </c>
@@ -26284,28 +26291,43 @@
         <v>21</v>
       </c>
       <c r="M664">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="N664">
         <v>4</v>
       </c>
       <c r="O664">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
     <row r="665" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A665" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="B665" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="D665" t="s">
-        <v>34</v>
+        <v>205</v>
       </c>
       <c r="E665" t="s">
         <v>19</v>
       </c>
+      <c r="F665">
+        <v>10</v>
+      </c>
+      <c r="G665">
+        <v>0</v>
+      </c>
+      <c r="H665">
+        <v>0</v>
+      </c>
+      <c r="I665">
+        <v>0</v>
+      </c>
+      <c r="J665">
+        <v>0</v>
+      </c>
       <c r="K665" t="s">
         <v>20</v>
       </c>
@@ -26313,13 +26335,13 @@
         <v>21</v>
       </c>
       <c r="M665">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N665">
         <v>4</v>
       </c>
       <c r="O665">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="666" spans="1:15" x14ac:dyDescent="0.35">
@@ -26327,29 +26349,14 @@
         <v>1175</v>
       </c>
       <c r="B666" t="s">
-        <v>1237</v>
+        <v>1176</v>
       </c>
       <c r="D666" t="s">
-        <v>583</v>
+        <v>34</v>
       </c>
       <c r="E666" t="s">
         <v>19</v>
       </c>
-      <c r="F666">
-        <v>0</v>
-      </c>
-      <c r="G666">
-        <v>0</v>
-      </c>
-      <c r="H666">
-        <v>0</v>
-      </c>
-      <c r="I666">
-        <v>0</v>
-      </c>
-      <c r="J666">
-        <v>0</v>
-      </c>
       <c r="K666" t="s">
         <v>20</v>
       </c>
@@ -26357,86 +26364,86 @@
         <v>21</v>
       </c>
       <c r="M666">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N666">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O666">
-        <v>47.5</v>
+        <v>24</v>
       </c>
     </row>
     <row r="667" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A667" t="s">
-        <v>1247</v>
+        <v>1175</v>
       </c>
       <c r="B667" t="s">
-        <v>1248</v>
+        <v>1224</v>
       </c>
       <c r="D667" t="s">
-        <v>60</v>
+        <v>583</v>
       </c>
       <c r="E667" t="s">
         <v>19</v>
       </c>
+      <c r="F667">
+        <v>0</v>
+      </c>
+      <c r="G667">
+        <v>0</v>
+      </c>
+      <c r="H667">
+        <v>0</v>
+      </c>
+      <c r="I667">
+        <v>0</v>
+      </c>
+      <c r="J667">
+        <v>0</v>
+      </c>
       <c r="K667" t="s">
         <v>20</v>
       </c>
       <c r="L667" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M667">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="N667">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O667">
-        <v>7.5</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="668" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A668" t="s">
-        <v>1177</v>
+        <v>1233</v>
       </c>
       <c r="B668" t="s">
-        <v>1218</v>
+        <v>1234</v>
       </c>
       <c r="D668" t="s">
-        <v>202</v>
+        <v>60</v>
       </c>
       <c r="E668" t="s">
         <v>19</v>
       </c>
-      <c r="F668">
-        <v>19</v>
-      </c>
-      <c r="G668">
-        <v>0</v>
-      </c>
-      <c r="H668">
-        <v>0</v>
-      </c>
-      <c r="I668">
+      <c r="K668" t="s">
+        <v>20</v>
+      </c>
+      <c r="L668" t="s">
+        <v>25</v>
+      </c>
+      <c r="M668">
+        <v>7.5</v>
+      </c>
+      <c r="N668">
         <v>1</v>
       </c>
-      <c r="J668">
-        <v>0</v>
-      </c>
-      <c r="K668" t="s">
-        <v>20</v>
-      </c>
-      <c r="L668" t="s">
-        <v>21</v>
-      </c>
-      <c r="M668">
-        <v>8</v>
-      </c>
-      <c r="N668">
-        <v>9</v>
-      </c>
       <c r="O668">
-        <v>72</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="669" spans="1:15" x14ac:dyDescent="0.35">
@@ -26444,16 +26451,16 @@
         <v>1177</v>
       </c>
       <c r="B669" t="s">
-        <v>1249</v>
+        <v>1205</v>
       </c>
       <c r="D669" t="s">
-        <v>1225</v>
+        <v>202</v>
       </c>
       <c r="E669" t="s">
         <v>19</v>
       </c>
       <c r="F669">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G669">
         <v>0</v>
@@ -26462,7 +26469,7 @@
         <v>0</v>
       </c>
       <c r="I669">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J669">
         <v>0</v>
@@ -26471,56 +26478,71 @@
         <v>20</v>
       </c>
       <c r="L669" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M669">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N669">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="O669">
-        <v>21</v>
+        <v>72</v>
       </c>
     </row>
     <row r="670" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A670" t="s">
-        <v>1250</v>
+        <v>1177</v>
       </c>
       <c r="B670" t="s">
-        <v>1251</v>
+        <v>1235</v>
       </c>
       <c r="D670" t="s">
-        <v>60</v>
+        <v>1212</v>
       </c>
       <c r="E670" t="s">
         <v>19</v>
       </c>
+      <c r="F670">
+        <v>0</v>
+      </c>
+      <c r="G670">
+        <v>0</v>
+      </c>
+      <c r="H670">
+        <v>0</v>
+      </c>
+      <c r="I670">
+        <v>0</v>
+      </c>
+      <c r="J670">
+        <v>0</v>
+      </c>
       <c r="K670" t="s">
         <v>20</v>
       </c>
       <c r="L670" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M670">
-        <v>6.75</v>
+        <v>13</v>
       </c>
       <c r="N670">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O670">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="671" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A671" t="s">
-        <v>1252</v>
+        <v>1236</v>
       </c>
       <c r="B671" t="s">
-        <v>1253</v>
+        <v>1237</v>
       </c>
       <c r="D671" t="s">
-        <v>362</v>
+        <v>60</v>
       </c>
       <c r="E671" t="s">
         <v>19</v>
@@ -26529,27 +26551,27 @@
         <v>20</v>
       </c>
       <c r="L671" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M671">
-        <v>4.75</v>
+        <v>6.5</v>
       </c>
       <c r="N671">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O671">
-        <v>9.5</v>
+        <v>26</v>
       </c>
     </row>
     <row r="672" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A672" t="s">
-        <v>1242</v>
+        <v>1238</v>
       </c>
       <c r="B672" t="s">
-        <v>770</v>
+        <v>1239</v>
       </c>
       <c r="D672" t="s">
-        <v>771</v>
+        <v>362</v>
       </c>
       <c r="E672" t="s">
         <v>19</v>
@@ -26561,42 +26583,57 @@
         <v>25</v>
       </c>
       <c r="M672">
-        <v>3.5</v>
+        <v>4.75</v>
       </c>
       <c r="N672">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O672">
-        <v>7</v>
+        <v>14.25</v>
       </c>
     </row>
     <row r="673" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A673" t="s">
-        <v>1178</v>
+        <v>1229</v>
       </c>
       <c r="B673" t="s">
-        <v>1254</v>
+        <v>770</v>
       </c>
       <c r="D673" t="s">
-        <v>663</v>
+        <v>771</v>
       </c>
       <c r="E673" t="s">
         <v>19</v>
       </c>
+      <c r="F673">
+        <v>0</v>
+      </c>
+      <c r="G673">
+        <v>0</v>
+      </c>
+      <c r="H673">
+        <v>0</v>
+      </c>
+      <c r="I673">
+        <v>0</v>
+      </c>
+      <c r="J673">
+        <v>0</v>
+      </c>
       <c r="K673" t="s">
         <v>20</v>
       </c>
       <c r="L673" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M673">
-        <v>16</v>
+        <v>3.5</v>
       </c>
       <c r="N673">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O673">
-        <v>96</v>
+        <v>7</v>
       </c>
     </row>
     <row r="674" spans="1:15" x14ac:dyDescent="0.35">
@@ -26604,10 +26641,10 @@
         <v>1178</v>
       </c>
       <c r="B674" t="s">
-        <v>1255</v>
+        <v>1179</v>
       </c>
       <c r="D674" t="s">
-        <v>663</v>
+        <v>1180</v>
       </c>
       <c r="E674" t="s">
         <v>19</v>
@@ -26619,50 +26656,65 @@
         <v>21</v>
       </c>
       <c r="M674">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="N674">
-        <v>4</v>
-      </c>
-      <c r="O674">
-        <v>44</v>
+        <v>0</v>
       </c>
     </row>
     <row r="675" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A675" t="s">
-        <v>1179</v>
+        <v>1240</v>
       </c>
       <c r="B675" t="s">
-        <v>1180</v>
+        <v>1241</v>
       </c>
       <c r="D675" t="s">
-        <v>1181</v>
+        <v>1242</v>
       </c>
       <c r="E675" t="s">
         <v>19</v>
       </c>
+      <c r="F675">
+        <v>0</v>
+      </c>
+      <c r="G675">
+        <v>0</v>
+      </c>
+      <c r="H675">
+        <v>0</v>
+      </c>
+      <c r="I675">
+        <v>0</v>
+      </c>
+      <c r="J675">
+        <v>0</v>
+      </c>
       <c r="K675" t="s">
         <v>20</v>
       </c>
       <c r="L675" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="M675">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="N675">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="O675">
+        <v>7.5</v>
       </c>
     </row>
     <row r="676" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A676" t="s">
-        <v>1179</v>
+        <v>1181</v>
       </c>
       <c r="B676" t="s">
-        <v>1256</v>
+        <v>1250</v>
       </c>
       <c r="D676" t="s">
-        <v>663</v>
+        <v>362</v>
       </c>
       <c r="E676" t="s">
         <v>19</v>
@@ -26674,83 +26726,122 @@
         <v>21</v>
       </c>
       <c r="M676">
-        <v>17</v>
+        <v>5.5</v>
       </c>
       <c r="N676">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O676">
-        <v>64</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="677" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A677" t="s">
-        <v>1179</v>
+        <v>1230</v>
       </c>
       <c r="B677" t="s">
-        <v>1257</v>
+        <v>1231</v>
       </c>
       <c r="D677" t="s">
-        <v>663</v>
+        <v>345</v>
       </c>
       <c r="E677" t="s">
         <v>19</v>
       </c>
+      <c r="F677">
+        <v>2</v>
+      </c>
+      <c r="G677">
+        <v>0</v>
+      </c>
+      <c r="H677">
+        <v>0</v>
+      </c>
+      <c r="I677">
+        <v>0</v>
+      </c>
       <c r="K677" t="s">
         <v>20</v>
       </c>
       <c r="L677" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M677">
-        <v>17</v>
+        <v>2.75</v>
       </c>
       <c r="N677">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O677">
-        <v>64</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="678" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A678" t="s">
-        <v>1182</v>
+        <v>1243</v>
       </c>
       <c r="B678" t="s">
-        <v>1183</v>
+        <v>1244</v>
       </c>
       <c r="D678" t="s">
-        <v>1181</v>
+        <v>1245</v>
       </c>
       <c r="E678" t="s">
         <v>19</v>
       </c>
+      <c r="F678">
+        <v>0</v>
+      </c>
+      <c r="G678">
+        <v>0</v>
+      </c>
+      <c r="H678">
+        <v>0</v>
+      </c>
+      <c r="I678">
+        <v>0</v>
+      </c>
+      <c r="J678">
+        <v>0</v>
+      </c>
       <c r="K678" t="s">
         <v>20</v>
       </c>
       <c r="L678" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M678">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N678">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="O678">
+        <v>12</v>
       </c>
     </row>
     <row r="679" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A679" t="s">
-        <v>1182</v>
+        <v>1243</v>
       </c>
       <c r="B679" t="s">
-        <v>1258</v>
+        <v>316</v>
       </c>
       <c r="D679" t="s">
-        <v>663</v>
+        <v>18</v>
       </c>
       <c r="E679" t="s">
         <v>19</v>
       </c>
+      <c r="F679">
+        <v>0</v>
+      </c>
+      <c r="I679">
+        <v>0</v>
+      </c>
+      <c r="J679">
+        <v>0</v>
+      </c>
       <c r="K679" t="s">
         <v>20</v>
       </c>
@@ -26758,13 +26849,13 @@
         <v>21</v>
       </c>
       <c r="M679">
-        <v>11</v>
+        <v>3.25</v>
       </c>
       <c r="N679">
         <v>4</v>
       </c>
       <c r="O679">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="680" spans="1:15" x14ac:dyDescent="0.35">
@@ -26772,10 +26863,10 @@
         <v>1182</v>
       </c>
       <c r="B680" t="s">
-        <v>1259</v>
+        <v>1183</v>
       </c>
       <c r="D680" t="s">
-        <v>663</v>
+        <v>228</v>
       </c>
       <c r="E680" t="s">
         <v>19</v>
@@ -26790,21 +26881,21 @@
         <v>11</v>
       </c>
       <c r="N680">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="O680">
-        <v>44</v>
+        <v>132</v>
       </c>
     </row>
     <row r="681" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A681" t="s">
-        <v>1182</v>
+        <v>1251</v>
       </c>
       <c r="B681" t="s">
-        <v>1260</v>
+        <v>1252</v>
       </c>
       <c r="D681" t="s">
-        <v>663</v>
+        <v>60</v>
       </c>
       <c r="E681" t="s">
         <v>19</v>
@@ -26813,27 +26904,27 @@
         <v>20</v>
       </c>
       <c r="L681" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M681">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N681">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O681">
-        <v>44</v>
+        <v>14</v>
       </c>
     </row>
     <row r="682" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A682" t="s">
-        <v>1184</v>
+        <v>1251</v>
       </c>
       <c r="B682" t="s">
-        <v>1185</v>
+        <v>529</v>
       </c>
       <c r="D682" t="s">
-        <v>1186</v>
+        <v>362</v>
       </c>
       <c r="E682" t="s">
         <v>19</v>
@@ -26842,56 +26933,68 @@
         <v>20</v>
       </c>
       <c r="L682" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M682">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N682">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="O682">
+        <v>6</v>
       </c>
     </row>
     <row r="683" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A683" t="s">
-        <v>1261</v>
+        <v>1253</v>
       </c>
       <c r="B683" t="s">
-        <v>1262</v>
+        <v>1254</v>
       </c>
       <c r="D683" t="s">
-        <v>1263</v>
+        <v>462</v>
       </c>
       <c r="E683" t="s">
         <v>187</v>
       </c>
+      <c r="F683">
+        <v>0</v>
+      </c>
+      <c r="I683">
+        <v>0</v>
+      </c>
+      <c r="J683">
+        <v>0</v>
+      </c>
       <c r="K683" t="s">
         <v>20</v>
       </c>
       <c r="L683" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M683">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="N683">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O683">
-        <v>2.5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="684" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A684" t="s">
-        <v>1187</v>
+        <v>1253</v>
       </c>
       <c r="B684" t="s">
-        <v>1188</v>
+        <v>1255</v>
       </c>
       <c r="D684" t="s">
-        <v>1189</v>
+        <v>462</v>
       </c>
       <c r="E684" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K684" t="s">
         <v>20</v>
@@ -26900,79 +27003,82 @@
         <v>21</v>
       </c>
       <c r="M684">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N684">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="O684">
+        <v>16</v>
       </c>
     </row>
     <row r="685" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A685" t="s">
-        <v>1243</v>
+        <v>1256</v>
       </c>
       <c r="B685" t="s">
-        <v>1244</v>
+        <v>1257</v>
       </c>
       <c r="D685" t="s">
-        <v>345</v>
+        <v>34</v>
       </c>
       <c r="E685" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K685" t="s">
         <v>20</v>
       </c>
       <c r="L685" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M685">
-        <v>2.75</v>
+        <v>6</v>
       </c>
       <c r="N685">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O685">
-        <v>5.5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="686" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A686" t="s">
-        <v>1264</v>
+        <v>1258</v>
       </c>
       <c r="B686" t="s">
-        <v>1265</v>
+        <v>1259</v>
       </c>
       <c r="D686" t="s">
-        <v>1266</v>
+        <v>34</v>
       </c>
       <c r="E686" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K686" t="s">
         <v>20</v>
       </c>
       <c r="L686" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M686">
         <v>6</v>
       </c>
       <c r="N686">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O686">
-        <v>6</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="687" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A687" t="s">
-        <v>1264</v>
+        <v>1260</v>
       </c>
       <c r="B687" t="s">
-        <v>316</v>
+        <v>1261</v>
       </c>
       <c r="D687" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="E687" t="s">
         <v>187</v>
@@ -26984,27 +27090,27 @@
         <v>21</v>
       </c>
       <c r="M687">
-        <v>3.25</v>
+        <v>6</v>
       </c>
       <c r="N687">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O687">
-        <v>3.25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="688" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A688" t="s">
-        <v>1190</v>
+        <v>1246</v>
       </c>
       <c r="B688" t="s">
-        <v>1191</v>
+        <v>421</v>
       </c>
       <c r="D688" t="s">
-        <v>1192</v>
+        <v>18</v>
       </c>
       <c r="E688" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K688" t="s">
         <v>20</v>
@@ -27013,24 +27119,24 @@
         <v>21</v>
       </c>
       <c r="M688">
-        <v>33</v>
+        <v>6.02</v>
       </c>
       <c r="N688">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="O688">
-        <v>429</v>
+        <v>24.079999923706001</v>
       </c>
     </row>
     <row r="689" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A689" t="s">
-        <v>1190</v>
+        <v>1247</v>
       </c>
       <c r="B689" t="s">
-        <v>1193</v>
+        <v>1248</v>
       </c>
       <c r="D689" t="s">
-        <v>228</v>
+        <v>18</v>
       </c>
       <c r="E689" t="s">
         <v>19</v>
@@ -27042,24 +27148,27 @@
         <v>21</v>
       </c>
       <c r="M689">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N689">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="O689">
+        <v>49</v>
       </c>
     </row>
     <row r="690" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A690" t="s">
-        <v>1267</v>
+        <v>1184</v>
       </c>
       <c r="B690" t="s">
-        <v>421</v>
+        <v>1185</v>
       </c>
       <c r="D690" t="s">
-        <v>18</v>
+        <v>1186</v>
       </c>
       <c r="E690" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K690" t="s">
         <v>20</v>
@@ -27068,27 +27177,24 @@
         <v>21</v>
       </c>
       <c r="M690">
-        <v>6.02</v>
+        <v>3</v>
       </c>
       <c r="N690">
-        <v>1</v>
-      </c>
-      <c r="O690">
-        <v>6.0199999809265003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="691" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A691" t="s">
-        <v>1268</v>
+        <v>1184</v>
       </c>
       <c r="B691" t="s">
-        <v>1269</v>
+        <v>1185</v>
       </c>
       <c r="D691" t="s">
-        <v>18</v>
+        <v>1187</v>
       </c>
       <c r="E691" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="K691" t="s">
         <v>20</v>
@@ -27097,24 +27203,21 @@
         <v>21</v>
       </c>
       <c r="M691">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="N691">
-        <v>1</v>
-      </c>
-      <c r="O691">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="692" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A692" t="s">
-        <v>1194</v>
+        <v>1184</v>
       </c>
       <c r="B692" t="s">
-        <v>1195</v>
+        <v>1185</v>
       </c>
       <c r="D692" t="s">
-        <v>1196</v>
+        <v>1188</v>
       </c>
       <c r="E692" t="s">
         <v>19</v>
@@ -27126,7 +27229,7 @@
         <v>21</v>
       </c>
       <c r="M692">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="N692">
         <v>0</v>
@@ -27134,39 +27237,42 @@
     </row>
     <row r="693" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A693" t="s">
-        <v>1194</v>
+        <v>1184</v>
       </c>
       <c r="B693" t="s">
-        <v>1195</v>
+        <v>1262</v>
       </c>
       <c r="D693" t="s">
-        <v>1197</v>
+        <v>1232</v>
       </c>
       <c r="E693" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K693" t="s">
         <v>20</v>
       </c>
       <c r="L693" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="M693">
+        <v>4</v>
+      </c>
+      <c r="N693">
         <v>3</v>
       </c>
-      <c r="N693">
-        <v>0</v>
+      <c r="O693">
+        <v>12</v>
       </c>
     </row>
     <row r="694" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A694" t="s">
-        <v>1194</v>
+        <v>1263</v>
       </c>
       <c r="B694" t="s">
-        <v>1195</v>
+        <v>1264</v>
       </c>
       <c r="D694" t="s">
-        <v>1198</v>
+        <v>852</v>
       </c>
       <c r="E694" t="s">
         <v>19</v>
@@ -27178,24 +27284,27 @@
         <v>21</v>
       </c>
       <c r="M694">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="N694">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="O694">
+        <v>25</v>
       </c>
     </row>
     <row r="695" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A695" t="s">
-        <v>1194</v>
+        <v>1265</v>
       </c>
       <c r="B695" t="s">
-        <v>1195</v>
+        <v>1266</v>
       </c>
       <c r="D695" t="s">
-        <v>1199</v>
+        <v>34</v>
       </c>
       <c r="E695" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K695" t="s">
         <v>20</v>
@@ -27204,7 +27313,7 @@
         <v>21</v>
       </c>
       <c r="M695">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N695">
         <v>0</v>
@@ -27212,13 +27321,13 @@
     </row>
     <row r="696" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A696" t="s">
-        <v>1194</v>
+        <v>1267</v>
       </c>
       <c r="B696" t="s">
-        <v>1245</v>
+        <v>1268</v>
       </c>
       <c r="D696" t="s">
-        <v>1246</v>
+        <v>1269</v>
       </c>
       <c r="E696" t="s">
         <v>187</v>
@@ -27227,42 +27336,68 @@
         <v>20</v>
       </c>
       <c r="L696" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="M696">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N696">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="O696">
+        <v>30</v>
       </c>
     </row>
     <row r="697" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A697" t="s">
-        <v>1200</v>
+        <v>1267</v>
       </c>
       <c r="B697" t="s">
         <v>1270</v>
       </c>
       <c r="D697" t="s">
-        <v>1201</v>
+        <v>724</v>
       </c>
       <c r="E697" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="K697" t="s">
         <v>20</v>
       </c>
       <c r="L697" t="s">
+        <v>25</v>
+      </c>
+      <c r="M697">
+        <v>6</v>
+      </c>
+      <c r="N697">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A698" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B698" t="s">
+        <v>1272</v>
+      </c>
+      <c r="D698" t="s">
+        <v>1273</v>
+      </c>
+      <c r="E698" t="s">
+        <v>187</v>
+      </c>
+      <c r="K698" t="s">
+        <v>20</v>
+      </c>
+      <c r="L698" t="s">
         <v>75</v>
       </c>
-      <c r="M697">
-        <v>120</v>
-      </c>
-      <c r="N697">
-        <v>4</v>
-      </c>
-      <c r="O697">
-        <v>480</v>
+      <c r="M698">
+        <v>5</v>
+      </c>
+      <c r="N698">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>